<commit_message>
TS001 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
   <si>
     <t>TC ID</t>
   </si>
@@ -40,6 +40,113 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>TC001</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Verify login with valid username and password</t>
+  </si>
+  <si>
+    <t>1. Open OrangeHRM URL 
+2. Enter valid username 
+3. Enter valid password 
+4. Click Login</t>
+  </si>
+  <si>
+    <t>User should be redirected to Dashboard page</t>
+  </si>
+  <si>
+    <t>As per execution</t>
+  </si>
+  <si>
+    <t>Verify login with invalid username</t>
+  </si>
+  <si>
+    <t>1. Open Login page 
+2. Enter invalid username 
+3. Enter valid password 
+4. Click Login</t>
+  </si>
+  <si>
+    <t>Error message should be displayed</t>
+  </si>
+  <si>
+    <t>Verify login with invalid password</t>
+  </si>
+  <si>
+    <t>1. Open Login page 
+2. Enter valid username 
+3. Enter invalid password 
+4. Click Login</t>
+  </si>
+  <si>
+    <t>Verify login with invalid username and password</t>
+  </si>
+  <si>
+    <t>1. Enter invalid username and password 
+2. Click Login</t>
+  </si>
+  <si>
+    <t>Verify login with empty username</t>
+  </si>
+  <si>
+    <t>1. Leave username blank 
+2. Enter password 
+3. Click Login</t>
+  </si>
+  <si>
+    <t>Required validation message should be displayed</t>
+  </si>
+  <si>
+    <t>Verify login with empty password</t>
+  </si>
+  <si>
+    <t>1. Enter username 
+2. Leave password blank 
+3. Click Login</t>
+  </si>
+  <si>
+    <t>Verify login with both fields empty</t>
+  </si>
+  <si>
+    <t>1. Leave username and password blank 
+2. Click Login</t>
+  </si>
+  <si>
+    <t>Required validation messages should be displayed</t>
+  </si>
+  <si>
+    <t>Verify password masking functionality</t>
+  </si>
+  <si>
+    <t>1. Enter password in password field</t>
+  </si>
+  <si>
+    <t>Password should be masked</t>
+  </si>
+  <si>
+    <t>Verify Login button functionality</t>
+  </si>
+  <si>
+    <t>1. Enter valid credentials 
+2. Click Login button</t>
+  </si>
+  <si>
+    <t>Login should be successful</t>
+  </si>
+  <si>
+    <t>Verify login using Enter key</t>
+  </si>
+  <si>
+    <t>1. Enter valid credentials 
+2. Press Enter</t>
+  </si>
+  <si>
+    <t>Pass/Fail</t>
   </si>
 </sst>
 </file>
@@ -75,8 +182,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,30 +479,162 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.7265625" style="2"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="C9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TS002 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="65">
   <si>
     <t>TC ID</t>
   </si>
@@ -147,14 +147,112 @@
   </si>
   <si>
     <t>Pass/Fail</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>Verify Forgot Password link navigation</t>
+  </si>
+  <si>
+    <t>1. Open Login page 
+2. Click Forgot Password</t>
+  </si>
+  <si>
+    <t>Forgot Password page should open</t>
+  </si>
+  <si>
+    <t>Verify password reset with valid username</t>
+  </si>
+  <si>
+    <t>1. Open Forgot Password page 
+2. Enter valid username 
+3. Click Reset</t>
+  </si>
+  <si>
+    <t>Password reset message should be displayed</t>
+  </si>
+  <si>
+    <t>Verify password reset with invalid username</t>
+  </si>
+  <si>
+    <t>1. Enter invalid username 
+2. Click Reset</t>
+  </si>
+  <si>
+    <t>Appropriate message should be displayed</t>
+  </si>
+  <si>
+    <t>Verify username field validation in Forgot Password</t>
+  </si>
+  <si>
+    <t>1. Leave username blank 
+2. Click Reset</t>
+  </si>
+  <si>
+    <t>Verify Cancel button functionality</t>
+  </si>
+  <si>
+    <t>1. Open Forgot Password page 
+2. Click Cancel</t>
+  </si>
+  <si>
+    <t>User should be redirected to Login page</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>TC015</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -182,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -198,6 +296,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -479,12 +580,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.90625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.7265625" style="2" bestFit="1" customWidth="1"/>
@@ -493,25 +594,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -538,106 +639,330 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="C4" t="s">
+      <c r="F3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="F5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="C6" t="s">
+      <c r="A6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="F6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="C7" t="s">
+      <c r="A7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="F7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="C8" t="s">
+      <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="F8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="C9" t="s">
+      <c r="A9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="F9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="C10" t="s">
+      <c r="A10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="F10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="C11" t="s">
+      <c r="A11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>33</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TS003 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="84">
   <si>
     <t>TC ID</t>
   </si>
@@ -237,6 +237,70 @@
   </si>
   <si>
     <t>TC015</t>
+  </si>
+  <si>
+    <t>Verify logout from user profile menu</t>
+  </si>
+  <si>
+    <t>1. Login successfully 
+2. Click profile menu 
+3. Click Logout</t>
+  </si>
+  <si>
+    <t>Verify session termination after logout</t>
+  </si>
+  <si>
+    <t>1. Login 
+2. Logout 
+3. Try accessing protected URL</t>
+  </si>
+  <si>
+    <t>Access should be denied</t>
+  </si>
+  <si>
+    <t>Verify browser back button after logout</t>
+  </si>
+  <si>
+    <t>1. Login 
+2. Logout 
+3. Press browser Back button</t>
+  </si>
+  <si>
+    <t>Dashboard should not be accessible</t>
+  </si>
+  <si>
+    <t>Verify logout option visibility</t>
+  </si>
+  <si>
+    <t>1. Login 
+2. Open profile menu</t>
+  </si>
+  <si>
+    <t>Logout option should be visible</t>
+  </si>
+  <si>
+    <t>Verify redirection to login page after logout</t>
+  </si>
+  <si>
+    <t>1. Logout from application</t>
+  </si>
+  <si>
+    <t>Login page should be displayed</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>TC020</t>
   </si>
 </sst>
 </file>
@@ -580,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -961,6 +1025,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="17" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" t="s">
+        <v>78</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS004 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="124">
   <si>
     <t>TC ID</t>
   </si>
@@ -301,6 +301,146 @@
   </si>
   <si>
     <t>TC020</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Verify Dashboard page loads successfully</t>
+  </si>
+  <si>
+    <t>1. Open OrangeHRM URL. 
+2. Enter valid credentials. 
+3. Click Login.</t>
+  </si>
+  <si>
+    <t>Dashboard page should load successfully.</t>
+  </si>
+  <si>
+    <t>Verify Time at Work widget display</t>
+  </si>
+  <si>
+    <t>1. Login to OrangeHRM. 
+2. Navigate to Dashboard. 
+3. Locate "Time at Work" widget.</t>
+  </si>
+  <si>
+    <t>Time at Work widget should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify My Actions widget display</t>
+  </si>
+  <si>
+    <t>1. Login to application. 
+2. Open Dashboard page. 
+3. Locate "My Actions" section</t>
+  </si>
+  <si>
+    <t>My Actions widget should be visible.</t>
+  </si>
+  <si>
+    <t>Verify Quick Launch widget display</t>
+  </si>
+  <si>
+    <t>Quick Launch options should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Scroll to Quick Launch section.</t>
+  </si>
+  <si>
+    <t>Verify Buzz Latest Posts widget display</t>
+  </si>
+  <si>
+    <t>Buzz Latest Posts section should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login to application. 
+2. Open Dashboard. 
+3. Locate Buzz Latest Posts widget.</t>
+  </si>
+  <si>
+    <t>Verify Employees on Leave Today widget display</t>
+  </si>
+  <si>
+    <t>Widget should be visible with employee leave information.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Navigate to Dashboard. 
+3. Locate Employees on Leave Today widget.</t>
+  </si>
+  <si>
+    <t>Verify Employee Distribution by Sub Unit chart</t>
+  </si>
+  <si>
+    <t>Chart should be displayed properly.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Scroll to Employee Distribution by Sub Unit chart.</t>
+  </si>
+  <si>
+    <t>Verify Employee Distribution by Location chart</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Scroll to Employee Distribution by Location chart.</t>
+  </si>
+  <si>
+    <t>Verify dashboard widgets load data correctly</t>
+  </si>
+  <si>
+    <t>All widgets should display valid data without errors.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Check all widgets one by one.</t>
+  </si>
+  <si>
+    <t>Verify dashboard scrolling functionality</t>
+  </si>
+  <si>
+    <t>Dashboard should scroll smoothly and all widgets should be accessible.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Scroll from top to bottom.</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>TC028</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>TC030</t>
   </si>
 </sst>
 </file>
@@ -644,11 +784,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.90625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43.1796875" style="2" bestFit="1" customWidth="1"/>
@@ -1140,6 +1280,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="22" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" t="s">
+        <v>91</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B30" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS005 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="164">
   <si>
     <t>TC ID</t>
   </si>
@@ -441,6 +441,144 @@
   </si>
   <si>
     <t>TC030</t>
+  </si>
+  <si>
+    <t>Verify Assign Leave quick launch navigation</t>
+  </si>
+  <si>
+    <t>Assign Leave page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click Assign Leave icon in Quick Launch.</t>
+  </si>
+  <si>
+    <t>Verify Leave List quick launch navigation</t>
+  </si>
+  <si>
+    <t>Leave List page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click Leave List icon.</t>
+  </si>
+  <si>
+    <t>Verify Timesheets quick launch navigation</t>
+  </si>
+  <si>
+    <t>Timesheets page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click Timesheets icon.</t>
+  </si>
+  <si>
+    <t>Verify Apply Leave quick launch navigation</t>
+  </si>
+  <si>
+    <t>Apply Leave page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click Apply Leave icon.</t>
+  </si>
+  <si>
+    <t>Verify My Leave quick launch navigation</t>
+  </si>
+  <si>
+    <t>My Leave page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click My Leave icon.</t>
+  </si>
+  <si>
+    <t>Verify My Timesheet quick launch navigation</t>
+  </si>
+  <si>
+    <t>My Timesheet page should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click My Timesheet icon.</t>
+  </si>
+  <si>
+    <t>Verify profile menu navigation</t>
+  </si>
+  <si>
+    <t>Profile menu options should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Click profile icon in top-right corner.</t>
+  </si>
+  <si>
+    <t>Verify Help icon navigation</t>
+  </si>
+  <si>
+    <t>Help page or help information should open.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Click Help (?) icon.</t>
+  </si>
+  <si>
+    <t>Verify Buzz Latest Posts navigation</t>
+  </si>
+  <si>
+    <t>Relevant Buzz post details should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click any Buzz post.</t>
+  </si>
+  <si>
+    <t>Verify My Actions navigation</t>
+  </si>
+  <si>
+    <t>Relevant page should open successfully.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Open Dashboard. 
+3. Click any action available under My Actions.</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>TC034</t>
+  </si>
+  <si>
+    <t>TC035</t>
+  </si>
+  <si>
+    <t>TC036</t>
+  </si>
+  <si>
+    <t>TC037</t>
+  </si>
+  <si>
+    <t>TC038</t>
+  </si>
+  <si>
+    <t>TC039</t>
+  </si>
+  <si>
+    <t>TC040</t>
   </si>
 </sst>
 </file>
@@ -784,7 +922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1510,6 +1648,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B34" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B35" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B36" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B40" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B41" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS006 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="188">
   <si>
     <t>TC ID</t>
   </si>
@@ -579,6 +579,90 @@
   </si>
   <si>
     <t>TC040</t>
+  </si>
+  <si>
+    <t>PIM</t>
+  </si>
+  <si>
+    <t>Verify Add Employee page opens</t>
+  </si>
+  <si>
+    <t>Add Employee page should open successfully.</t>
+  </si>
+  <si>
+    <t>1. Login to OrangeHRM. 
+2. Navigate to PIM. 
+3. Click Add Employee tab.</t>
+  </si>
+  <si>
+    <t>Verify employee creation with valid data</t>
+  </si>
+  <si>
+    <t>Employee should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page. 
+2. Enter First Name. 
+3. Enter Last Name. 
+4. Click Save.</t>
+  </si>
+  <si>
+    <t>Verify mandatory field validation</t>
+  </si>
+  <si>
+    <t>Validation message should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page. 
+2. Leave required fields blank. 
+3. Click Save.</t>
+  </si>
+  <si>
+    <t>Verify employee photo upload</t>
+  </si>
+  <si>
+    <t>Image should be uploaded successfully.</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page. 
+2. Click profile image upload icon. 
+3. Select image.</t>
+  </si>
+  <si>
+    <t>Verify employee ID field display</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page.</t>
+  </si>
+  <si>
+    <t>Employee ID field should be visible.</t>
+  </si>
+  <si>
+    <t>Verify Create Login Details option</t>
+  </si>
+  <si>
+    <t>Login credential fields should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page. 
+2. Enable Create Login Details.</t>
+  </si>
+  <si>
+    <t>Verify Save button functionality</t>
+  </si>
+  <si>
+    <t>Employee details should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter employee details. 
+2. Click Save.</t>
+  </si>
+  <si>
+    <t>User should be redirected without saving data.</t>
+  </si>
+  <si>
+    <t>1. Open Add Employee page. 
+2. Click Cancel.</t>
   </si>
 </sst>
 </file>
@@ -922,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1878,6 +1962,106 @@
         <v>36</v>
       </c>
     </row>
+    <row r="42" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B42" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="C43" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C44" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C45" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="C46" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="C47" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="C48" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="49" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C49" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C52" s="3"/>
+    </row>
+    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C53" s="3"/>
+    </row>
+    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C54" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS007 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="229">
   <si>
     <t>TC ID</t>
   </si>
@@ -663,6 +663,137 @@
   <si>
     <t>1. Open Add Employee page. 
 2. Click Cancel.</t>
+  </si>
+  <si>
+    <t>TC041</t>
+  </si>
+  <si>
+    <t>TC042</t>
+  </si>
+  <si>
+    <t>TC043</t>
+  </si>
+  <si>
+    <t>TC044</t>
+  </si>
+  <si>
+    <t>TC045</t>
+  </si>
+  <si>
+    <t>TC046</t>
+  </si>
+  <si>
+    <t>TC047</t>
+  </si>
+  <si>
+    <t>TC048</t>
+  </si>
+  <si>
+    <t>Verify Employee List page display</t>
+  </si>
+  <si>
+    <t>Employee List page should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login. 
+2. Navigate to PIM → Employee List.</t>
+  </si>
+  <si>
+    <t>Verify search by Employee Name</t>
+  </si>
+  <si>
+    <t>Matching employee record should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify search by Employee ID</t>
+  </si>
+  <si>
+    <t>1. Enter Employee ID. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify search by Job Title</t>
+  </si>
+  <si>
+    <t>Matching records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Job Title. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify search by Employment Status</t>
+  </si>
+  <si>
+    <t>1. Select Employment Status. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify search by Supervisor Name</t>
+  </si>
+  <si>
+    <t>Matching employee records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Supervisor Name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify search by Sub Unit</t>
+  </si>
+  <si>
+    <t>1. Select Sub Unit. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Reset button functionality</t>
+  </si>
+  <si>
+    <t>All filters should be cleared.</t>
+  </si>
+  <si>
+    <t>1. Apply search filters. 
+2. Click Reset.</t>
+  </si>
+  <si>
+    <t>Verify employee records display</t>
+  </si>
+  <si>
+    <t>1. Open Employee List page.</t>
+  </si>
+  <si>
+    <t>Employee records table should be displayed.</t>
+  </si>
+  <si>
+    <t>TC049</t>
+  </si>
+  <si>
+    <t>TC050</t>
+  </si>
+  <si>
+    <t>TC051</t>
+  </si>
+  <si>
+    <t>TC052</t>
+  </si>
+  <si>
+    <t>TC053</t>
+  </si>
+  <si>
+    <t>TC054</t>
+  </si>
+  <si>
+    <t>TC055</t>
+  </si>
+  <si>
+    <t>TC056</t>
+  </si>
+  <si>
+    <t>TC057</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -1963,6 +2094,9 @@
       </c>
     </row>
     <row r="42" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>188</v>
+      </c>
       <c r="B42" s="2" t="s">
         <v>164</v>
       </c>
@@ -1975,8 +2109,20 @@
       <c r="E42" s="3" t="s">
         <v>166</v>
       </c>
+      <c r="F42" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="43" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C43" s="3" t="s">
         <v>168</v>
       </c>
@@ -1986,8 +2132,20 @@
       <c r="E43" s="3" t="s">
         <v>169</v>
       </c>
+      <c r="F43" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C44" s="3" t="s">
         <v>171</v>
       </c>
@@ -1997,8 +2155,20 @@
       <c r="E44" s="3" t="s">
         <v>172</v>
       </c>
+      <c r="F44" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="45" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C45" s="3" t="s">
         <v>174</v>
       </c>
@@ -2008,8 +2178,20 @@
       <c r="E45" s="3" t="s">
         <v>175</v>
       </c>
+      <c r="F45" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C46" s="3" t="s">
         <v>177</v>
       </c>
@@ -2019,8 +2201,20 @@
       <c r="E46" s="3" t="s">
         <v>179</v>
       </c>
+      <c r="F46" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C47" s="3" t="s">
         <v>180</v>
       </c>
@@ -2030,8 +2224,20 @@
       <c r="E47" s="3" t="s">
         <v>181</v>
       </c>
+      <c r="F47" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C48" s="3" t="s">
         <v>183</v>
       </c>
@@ -2041,8 +2247,20 @@
       <c r="E48" s="3" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="49" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="F48" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>164</v>
+      </c>
       <c r="C49" s="3" t="s">
         <v>57</v>
       </c>
@@ -2052,15 +2270,219 @@
       <c r="E49" s="3" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C52" s="3"/>
-    </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C53" s="3"/>
-    </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
-      <c r="C54" s="3"/>
+      <c r="F49" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A54" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A56" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
TS008 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="253">
   <si>
     <t>TC ID</t>
   </si>
@@ -794,6 +794,86 @@
   </si>
   <si>
     <t>TC057</t>
+  </si>
+  <si>
+    <t>Verify Edit employee option availability</t>
+  </si>
+  <si>
+    <t>1. Open Employee List.</t>
+  </si>
+  <si>
+    <t>Edit icon should be visible for employee records.</t>
+  </si>
+  <si>
+    <t>Verify edit employee details</t>
+  </si>
+  <si>
+    <t>Employee information should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Edit icon. 
+2. Modify employee details. 
+3. Save changes.</t>
+  </si>
+  <si>
+    <t>Verify update employee personal information</t>
+  </si>
+  <si>
+    <t>1. Edit employee profile. 
+2. Change details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Updated information should be saved.</t>
+  </si>
+  <si>
+    <t>Verify update employee contact information</t>
+  </si>
+  <si>
+    <t>Updated contact information should be saved.</t>
+  </si>
+  <si>
+    <t>1. Open employee profile. 
+2. Update contact information. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Save button while editing</t>
+  </si>
+  <si>
+    <t>Changes should be stored successfully.</t>
+  </si>
+  <si>
+    <t>1. Modify employee data. 
+2. Click Save.</t>
+  </si>
+  <si>
+    <t>Verify Cancel operation during edit</t>
+  </si>
+  <si>
+    <t>Changes should not be saved.</t>
+  </si>
+  <si>
+    <t>1. Edit employee details. 
+2. Click Cancel.</t>
+  </si>
+  <si>
+    <t>TC058</t>
+  </si>
+  <si>
+    <t>TC059</t>
+  </si>
+  <si>
+    <t>TC060</t>
+  </si>
+  <si>
+    <t>TC061</t>
+  </si>
+  <si>
+    <t>TC062</t>
+  </si>
+  <si>
+    <t>TC063</t>
   </si>
 </sst>
 </file>
@@ -1137,7 +1217,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -2484,6 +2564,144 @@
         <v>36</v>
       </c>
     </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS009 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="272">
   <si>
     <t>TC ID</t>
   </si>
@@ -874,6 +874,67 @@
   </si>
   <si>
     <t>TC063</t>
+  </si>
+  <si>
+    <t>Verify Delete employee option availability</t>
+  </si>
+  <si>
+    <t>Delete icon should be visible.</t>
+  </si>
+  <si>
+    <t>Verify employee deletion</t>
+  </si>
+  <si>
+    <t>Employee record should be removed successfully.</t>
+  </si>
+  <si>
+    <t>1. Select employee. 
+2. Click Delete icon. 
+3. Confirm deletion.</t>
+  </si>
+  <si>
+    <t>Verify delete confirmation popup</t>
+  </si>
+  <si>
+    <t>1. Click Delete icon.</t>
+  </si>
+  <si>
+    <t>Confirmation popup should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify cancel deletion operation</t>
+  </si>
+  <si>
+    <t>Employee record should not be deleted.</t>
+  </si>
+  <si>
+    <t>1. Click Delete icon. 
+2. Click Cancel.</t>
+  </si>
+  <si>
+    <t>Verify deleted employee record is removed from list</t>
+  </si>
+  <si>
+    <t>Employee record should not be found.</t>
+  </si>
+  <si>
+    <t>1. Delete employee. 
+2. Search for deleted employee.</t>
+  </si>
+  <si>
+    <t>TC064</t>
+  </si>
+  <si>
+    <t>TC065</t>
+  </si>
+  <si>
+    <t>TC066</t>
+  </si>
+  <si>
+    <t>TC067</t>
+  </si>
+  <si>
+    <t>TC068</t>
   </si>
 </sst>
 </file>
@@ -1217,7 +1278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
@@ -2702,6 +2763,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A66" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS011 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="311">
   <si>
     <t>TC ID</t>
   </si>
@@ -998,6 +998,72 @@
   </si>
   <si>
     <t>TC073</t>
+  </si>
+  <si>
+    <t>Verify pending leave requests in Leave List</t>
+  </si>
+  <si>
+    <t>Pending leave requests should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login as approver/admin. 
+2. Navigate to Leave → Leave List. 3. Search pending requests.</t>
+  </si>
+  <si>
+    <t>Verify leave approval functionality</t>
+  </si>
+  <si>
+    <t>Leave status should change to Approved.</t>
+  </si>
+  <si>
+    <t>1. Open pending leave request. 
+2. Select Approve option. 
+3. Confirm action.</t>
+  </si>
+  <si>
+    <t>Verify leave rejection functionality</t>
+  </si>
+  <si>
+    <t>Leave status should change to Rejected.</t>
+  </si>
+  <si>
+    <t>1. Open pending leave request. 
+2. Select Reject option. 
+3. Confirm action.</t>
+  </si>
+  <si>
+    <t>Verify leave balance update after approval</t>
+  </si>
+  <si>
+    <t>Leave balance should be reduced accordingly.</t>
+  </si>
+  <si>
+    <t>1. Approve leave request. 
+2. Check employee leave balance.</t>
+  </si>
+  <si>
+    <t>Verify approved/rejected status visibility</t>
+  </si>
+  <si>
+    <t>1. Open Leave List after approval/rejection.</t>
+  </si>
+  <si>
+    <t>Updated leave status should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>TC074</t>
+  </si>
+  <si>
+    <t>TC075</t>
+  </si>
+  <si>
+    <t>TC076</t>
+  </si>
+  <si>
+    <t>TC077</t>
+  </si>
+  <si>
+    <t>TC078</t>
   </si>
 </sst>
 </file>
@@ -1338,13 +1404,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3053,6 +3119,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="75" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS012 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="329">
   <si>
     <t>TC ID</t>
   </si>
@@ -1064,6 +1064,64 @@
   </si>
   <si>
     <t>TC078</t>
+  </si>
+  <si>
+    <t>Verify My Leave page displays leave records</t>
+  </si>
+  <si>
+    <t>Applied leave records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Leave → My Leave. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify leave search using filters</t>
+  </si>
+  <si>
+    <t>Matching leave records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Status, Date Range or Leave Type. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify leave status tracking</t>
+  </si>
+  <si>
+    <t>Current status (Pending, Approved, Rejected, Cancelled) should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Open My Leave page. 
+2. View leave records.</t>
+  </si>
+  <si>
+    <t>Verify leave cancellation functionality</t>
+  </si>
+  <si>
+    <t>Leave request should be cancelled successfully.</t>
+  </si>
+  <si>
+    <t>1. Open pending leave request. 
+2. Click Cancel.</t>
+  </si>
+  <si>
+    <t>All selected filters should be cleared.</t>
+  </si>
+  <si>
+    <t>TC079</t>
+  </si>
+  <si>
+    <t>TC080</t>
+  </si>
+  <si>
+    <t>TC081</t>
+  </si>
+  <si>
+    <t>TC082</t>
+  </si>
+  <si>
+    <t>TC083</t>
   </si>
 </sst>
 </file>
@@ -1404,7 +1462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3234,6 +3292,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="80" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="F80" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F82" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A83" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A84" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS013 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="350">
   <si>
     <t>TC ID</t>
   </si>
@@ -1122,6 +1122,73 @@
   </si>
   <si>
     <t>TC083</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Verify Timesheet page opens successfully</t>
+  </si>
+  <si>
+    <t>Timesheet page should open successfully.</t>
+  </si>
+  <si>
+    <t>1. Login to OrangeHRM. 
+2. Navigate to Time → Timesheets → My Timesheets.</t>
+  </si>
+  <si>
+    <t>Verify Edit Timesheet functionality</t>
+  </si>
+  <si>
+    <t>User should be able to edit timesheet details.</t>
+  </si>
+  <si>
+    <t>1. Open My Timesheet page. 
+2. Click Edit.</t>
+  </si>
+  <si>
+    <t>Verify creation of new timesheet entry</t>
+  </si>
+  <si>
+    <t>New timesheet entry should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Open timesheet. 
+2. Add project/activity hours. 
+3. Save changes.</t>
+  </si>
+  <si>
+    <t>Verify timesheet period navigation</t>
+  </si>
+  <si>
+    <t>1. Click Previous/Next period arrows.</t>
+  </si>
+  <si>
+    <t>Timesheet should display selected week period.</t>
+  </si>
+  <si>
+    <t>Verify empty timesheet display</t>
+  </si>
+  <si>
+    <t>1. Open a timesheet with no entries.</t>
+  </si>
+  <si>
+    <t>"No Records Found" message should be displayed.</t>
+  </si>
+  <si>
+    <t>TC084</t>
+  </si>
+  <si>
+    <t>TC085</t>
+  </si>
+  <si>
+    <t>TC086</t>
+  </si>
+  <si>
+    <t>TC087</t>
+  </si>
+  <si>
+    <t>TC088</t>
   </si>
 </sst>
 </file>
@@ -1462,7 +1529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3407,6 +3474,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="85" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G85" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A87" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A88" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A89" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS014 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="370">
   <si>
     <t>TC ID</t>
   </si>
@@ -1189,6 +1189,69 @@
   </si>
   <si>
     <t>TC088</t>
+  </si>
+  <si>
+    <t>Verify Submit button availability</t>
+  </si>
+  <si>
+    <t>1. Open completed timesheet.</t>
+  </si>
+  <si>
+    <t>Submit button should be enabled.</t>
+  </si>
+  <si>
+    <t>Verify successful timesheet submission</t>
+  </si>
+  <si>
+    <t>Timesheet should be submitted successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter timesheet data. 
+2. Click Submit.</t>
+  </si>
+  <si>
+    <t>Verify status change after submission</t>
+  </si>
+  <si>
+    <t>1. Submit timesheet.</t>
+  </si>
+  <si>
+    <t>Status should change from "Not Submitted" to "Submitted".</t>
+  </si>
+  <si>
+    <t>Verify submission without data</t>
+  </si>
+  <si>
+    <t>Appropriate validation/error message should appear.</t>
+  </si>
+  <si>
+    <t>1. Open blank timesheet. 
+2. Click Submit.</t>
+  </si>
+  <si>
+    <t>Verify submitted timesheet becomes read-only</t>
+  </si>
+  <si>
+    <t>User should not be able to modify submitted timesheet directly.</t>
+  </si>
+  <si>
+    <t>1. Submit timesheet. 
+2. Reopen timesheet.</t>
+  </si>
+  <si>
+    <t>TC089</t>
+  </si>
+  <si>
+    <t>TC090</t>
+  </si>
+  <si>
+    <t>TC091</t>
+  </si>
+  <si>
+    <t>TC092</t>
+  </si>
+  <si>
+    <t>TC093</t>
   </si>
 </sst>
 </file>
@@ -1529,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3589,6 +3652,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A91" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A92" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A93" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A94" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS015 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="390">
   <si>
     <t>TC ID</t>
   </si>
@@ -1252,6 +1252,69 @@
   </si>
   <si>
     <t>TC093</t>
+  </si>
+  <si>
+    <t>Verify Timesheets Pending Action page</t>
+  </si>
+  <si>
+    <t>Pending timesheets should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Login as Supervisor/Admin. 
+2. Navigate to Time → Timesheets → Employee Timesheets.</t>
+  </si>
+  <si>
+    <t>Verify viewing submitted timesheet</t>
+  </si>
+  <si>
+    <t>1. Click View on a pending timesheet.</t>
+  </si>
+  <si>
+    <t>Timesheet details should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify timesheet approval functionality</t>
+  </si>
+  <si>
+    <t>Timesheet status should change to Approved.</t>
+  </si>
+  <si>
+    <t>1. Open submitted timesheet. 
+2. Click Approve.</t>
+  </si>
+  <si>
+    <t>Verify timesheet rejection functionality</t>
+  </si>
+  <si>
+    <t>Timesheet status should change to Rejected.</t>
+  </si>
+  <si>
+    <t>1. Open submitted timesheet. 
+2. Click Reject.</t>
+  </si>
+  <si>
+    <t>Verify approved/rejected timesheet status tracking</t>
+  </si>
+  <si>
+    <t>1. Search submitted timesheet after action.</t>
+  </si>
+  <si>
+    <t>Correct status should be displayed.</t>
+  </si>
+  <si>
+    <t>TC094</t>
+  </si>
+  <si>
+    <t>TC095</t>
+  </si>
+  <si>
+    <t>TC096</t>
+  </si>
+  <si>
+    <t>TC097</t>
+  </si>
+  <si>
+    <t>TC098</t>
   </si>
 </sst>
 </file>
@@ -1592,12 +1655,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
@@ -3767,6 +3830,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="95" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A95" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A96" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A97" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G97" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A98" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F98" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G98" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A99" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G99" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS016 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="411">
   <si>
     <t>TC ID</t>
   </si>
@@ -1315,6 +1315,78 @@
   </si>
   <si>
     <t>TC098</t>
+  </si>
+  <si>
+    <t>Recruitment</t>
+  </si>
+  <si>
+    <t>Verify Vacancies page opens successfully</t>
+  </si>
+  <si>
+    <t>Vacancies page should load successfully.</t>
+  </si>
+  <si>
+    <t>1. Login as Admin/HR. 
+2. Navigate to Recruitment → Vacancies.</t>
+  </si>
+  <si>
+    <t>Verify Add Vacancy functionality</t>
+  </si>
+  <si>
+    <t>New vacancy should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add. 
+2. Enter vacancy details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify vacancy search functionality</t>
+  </si>
+  <si>
+    <t>Matching vacancies should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Job Title/Vacancy/Hiring Manager. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Edit Vacancy functionality</t>
+  </si>
+  <si>
+    <t>Vacancy details should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Select a vacancy. 
+2. Click Edit icon. 
+3. Modify details and save.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Delete Vacancy functionality
+</t>
+  </si>
+  <si>
+    <t>Vacancy should be removed from the list.</t>
+  </si>
+  <si>
+    <t>1. Select vacancy. 
+2. Click Delete icon. 
+3. Confirm deletion.</t>
+  </si>
+  <si>
+    <t>TC099</t>
+  </si>
+  <si>
+    <t>TC100</t>
+  </si>
+  <si>
+    <t>TC101</t>
+  </si>
+  <si>
+    <t>TC102</t>
+  </si>
+  <si>
+    <t>TC103</t>
   </si>
 </sst>
 </file>
@@ -1655,11 +1727,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -3945,6 +4017,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="100" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A100" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A101" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="F101" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G101" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G102" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A103" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G103" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A104" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G104" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS017 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="431">
   <si>
     <t>TC ID</t>
   </si>
@@ -1387,6 +1387,71 @@
   </si>
   <si>
     <t>TC103</t>
+  </si>
+  <si>
+    <t>Verify Candidates page opens successfully</t>
+  </si>
+  <si>
+    <t>1. Navigate to Recruitment → Candidates.</t>
+  </si>
+  <si>
+    <t>Candidates page should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify Add Candidate functionality</t>
+  </si>
+  <si>
+    <t>Candidate should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add. 
+2. Enter candidate information. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify candidate search functionality</t>
+  </si>
+  <si>
+    <t>Matching candidate records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Candidate Name/Status/Vacancy. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify candidate profile view functionality</t>
+  </si>
+  <si>
+    <t>1. Click View icon for a candidate.</t>
+  </si>
+  <si>
+    <t>Candidate profile details should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify candidate deletion functionality</t>
+  </si>
+  <si>
+    <t>Candidate record should be deleted successfully.</t>
+  </si>
+  <si>
+    <t>1. Select candidate. 
+2. Click Delete icon. 
+3. Confirm deletion.</t>
+  </si>
+  <si>
+    <t>TC104</t>
+  </si>
+  <si>
+    <t>TC105</t>
+  </si>
+  <si>
+    <t>TC106</t>
+  </si>
+  <si>
+    <t>TC107</t>
+  </si>
+  <si>
+    <t>TC108</t>
   </si>
 </sst>
 </file>
@@ -1727,7 +1792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G109"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -4132,6 +4197,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="105" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A105" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G105" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A106" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A107" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A109" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS018 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="451">
   <si>
     <t>TC ID</t>
   </si>
@@ -1452,6 +1452,71 @@
   </si>
   <si>
     <t>TC108</t>
+  </si>
+  <si>
+    <t>Verify candidate application submission</t>
+  </si>
+  <si>
+    <t>Application should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Create a candidate profile. 
+2. Associate with a vacancy.</t>
+  </si>
+  <si>
+    <t>Verify candidate status progression</t>
+  </si>
+  <si>
+    <t>Status should update correctly (Applied → Shortlisted → Interview, etc.).</t>
+  </si>
+  <si>
+    <t>1. Open candidate profile. 
+2. Move candidate through workflow stages.</t>
+  </si>
+  <si>
+    <t>Verify shortlisted candidate functionality</t>
+  </si>
+  <si>
+    <t>Candidate status should change to Shortlisted.</t>
+  </si>
+  <si>
+    <t>1. Select a candidate. 
+2. Mark as Shortlisted.</t>
+  </si>
+  <si>
+    <t>Verify candidate rejection functionality</t>
+  </si>
+  <si>
+    <t>Candidate status should change to Rejected.</t>
+  </si>
+  <si>
+    <t>1. Open candidate profile. 
+2. Reject application.</t>
+  </si>
+  <si>
+    <t>Verify hired candidate workflow completion</t>
+  </si>
+  <si>
+    <t>Candidate should be moved to Hired status and workflow completed.</t>
+  </si>
+  <si>
+    <t>1. Select eligible candidate. 
+2. Mark candidate as Hired.</t>
+  </si>
+  <si>
+    <t>TC109</t>
+  </si>
+  <si>
+    <t>TC110</t>
+  </si>
+  <si>
+    <t>TC111</t>
+  </si>
+  <si>
+    <t>TC112</t>
+  </si>
+  <si>
+    <t>TC113</t>
   </si>
 </sst>
 </file>
@@ -1792,7 +1857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -4312,6 +4377,121 @@
         <v>36</v>
       </c>
     </row>
+    <row r="110" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A110" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A111" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A112" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A113" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A114" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS019 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="492">
   <si>
     <t>TC ID</t>
   </si>
@@ -1517,6 +1517,140 @@
   </si>
   <si>
     <t>TC113</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Verify User List Display</t>
+  </si>
+  <si>
+    <t>1. Navigate to Admin → User Management.</t>
+  </si>
+  <si>
+    <t>All existing users should be displayed successfully.</t>
+  </si>
+  <si>
+    <t>Verify Add User Functionality</t>
+  </si>
+  <si>
+    <t>New user should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add button. 
+2. Enter valid user details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Edit User Details</t>
+  </si>
+  <si>
+    <t>User information should update successfully.</t>
+  </si>
+  <si>
+    <t>1. Select a user. 
+2. Click Edit icon. 
+3. Modify details. 
+4. Save.</t>
+  </si>
+  <si>
+    <t>Verify Delete User Functionality</t>
+  </si>
+  <si>
+    <t>User should be removed successfully.</t>
+  </si>
+  <si>
+    <t>1. Select a user. 
+2. Click Delete icon. 
+3. Confirm deletion.</t>
+  </si>
+  <si>
+    <t>Verify User Search Functionality</t>
+  </si>
+  <si>
+    <t>Matching user records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter username in search field. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search by User Role</t>
+  </si>
+  <si>
+    <t>1. Select User Role from dropdown. 2. Click Search.</t>
+  </si>
+  <si>
+    <t>Users belonging to selected role should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Search by Employee Name</t>
+  </si>
+  <si>
+    <t>Relevant user record should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter employee name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search by Status</t>
+  </si>
+  <si>
+    <t>1. Select status (Enabled/Disabled). 2. Click Search.</t>
+  </si>
+  <si>
+    <t>Users with selected status should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Reset Search Filters</t>
+  </si>
+  <si>
+    <t>All search filters should be cleared.</t>
+  </si>
+  <si>
+    <t>1. Enter search criteria. 
+2. Click Reset.</t>
+  </si>
+  <si>
+    <t>Verify User Status Update</t>
+  </si>
+  <si>
+    <t>User status should update correctly.</t>
+  </si>
+  <si>
+    <t>1. Edit user status. 
+2. Save changes.</t>
+  </si>
+  <si>
+    <t>TC114</t>
+  </si>
+  <si>
+    <t>TC115</t>
+  </si>
+  <si>
+    <t>TC116</t>
+  </si>
+  <si>
+    <t>TC117</t>
+  </si>
+  <si>
+    <t>TC118</t>
+  </si>
+  <si>
+    <t>TC119</t>
+  </si>
+  <si>
+    <t>TC120</t>
+  </si>
+  <si>
+    <t>TC121</t>
+  </si>
+  <si>
+    <t>TC122</t>
+  </si>
+  <si>
+    <t>TC123</t>
   </si>
 </sst>
 </file>
@@ -1857,7 +1991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -4492,6 +4626,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="115" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A115" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A116" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A117" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G117" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A118" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A119" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G119" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A120" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A121" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G121" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A122" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G122" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A123" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G123" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A124" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G124" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS020 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="532">
   <si>
     <t>TC ID</t>
   </si>
@@ -1651,6 +1651,133 @@
   </si>
   <si>
     <t>TC123</t>
+  </si>
+  <si>
+    <t>Verify Admin Role Access</t>
+  </si>
+  <si>
+    <t>1. Login as Admin user.</t>
+  </si>
+  <si>
+    <t>Admin should access all modules and features.</t>
+  </si>
+  <si>
+    <t>Verify ESS/User Role Access</t>
+  </si>
+  <si>
+    <t>1. Login as ESS/User.</t>
+  </si>
+  <si>
+    <t>User should access only permitted modules.</t>
+  </si>
+  <si>
+    <t>Verify Restricted Page Access</t>
+  </si>
+  <si>
+    <t>Access should be denied.</t>
+  </si>
+  <si>
+    <t>1. Login as non-admin user. 
+2. Open Admin page URL directly.</t>
+  </si>
+  <si>
+    <t>Verify Role Assignment</t>
+  </si>
+  <si>
+    <t>New role should be assigned successfully.</t>
+  </si>
+  <si>
+    <t>1. Edit user. 
+2. Assign new role. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Permission Changes After Role Update</t>
+  </si>
+  <si>
+    <t>Updated permissions should be applied.</t>
+  </si>
+  <si>
+    <t>1. Change user role. 
+2. Login again.</t>
+  </si>
+  <si>
+    <t>Verify Multiple Users with Same Role</t>
+  </si>
+  <si>
+    <t>1. Create multiple users with same role.</t>
+  </si>
+  <si>
+    <t>All users should inherit the assigned permissions.</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized Action Restriction</t>
+  </si>
+  <si>
+    <t>System should block the action.</t>
+  </si>
+  <si>
+    <t>1. Login as restricted user. 
+2. Attempt admin action.</t>
+  </si>
+  <si>
+    <t>Verify Menu Visibility Based on Role</t>
+  </si>
+  <si>
+    <t>1. Login with different roles.</t>
+  </si>
+  <si>
+    <t>Menus should display according to permissions.</t>
+  </si>
+  <si>
+    <t>Verify Session After Role Change</t>
+  </si>
+  <si>
+    <t>Updated permissions should reflect correctly.</t>
+  </si>
+  <si>
+    <t>1. Change logged-in user's role. 
+2. Re-login.</t>
+  </si>
+  <si>
+    <t>Verify Role Persistence</t>
+  </si>
+  <si>
+    <t>Assigned role should remain unchanged.</t>
+  </si>
+  <si>
+    <t>1. Assign role. 
+2. Refresh page/Login again.</t>
+  </si>
+  <si>
+    <t>TC124</t>
+  </si>
+  <si>
+    <t>TC125</t>
+  </si>
+  <si>
+    <t>TC126</t>
+  </si>
+  <si>
+    <t>TC127</t>
+  </si>
+  <si>
+    <t>TC128</t>
+  </si>
+  <si>
+    <t>TC129</t>
+  </si>
+  <si>
+    <t>TC130</t>
+  </si>
+  <si>
+    <t>TC131</t>
+  </si>
+  <si>
+    <t>TC132</t>
+  </si>
+  <si>
+    <t>TC133</t>
   </si>
 </sst>
 </file>
@@ -1991,7 +2118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -4856,6 +4983,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A125" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G125" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G126" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A127" s="1" t="s">
+        <v>524</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G127" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A128" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G128" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A129" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G129" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A130" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G130" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A131" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G131" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A132" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G132" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A133" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G133" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A134" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS021 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="567">
   <si>
     <t>TC ID</t>
   </si>
@@ -1778,6 +1778,117 @@
   </si>
   <si>
     <t>TC133</t>
+  </si>
+  <si>
+    <t>Verify Search by Username</t>
+  </si>
+  <si>
+    <t>Matching user should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter valid username. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Users of selected role should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select role from dropdown. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Relevant user records should be displayed.</t>
+  </si>
+  <si>
+    <t>Users with selected status should appear.</t>
+  </si>
+  <si>
+    <t>1. Select status. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Combined Search Criteria</t>
+  </si>
+  <si>
+    <t>1. Enter username, role, and status. 2. Click Search.</t>
+  </si>
+  <si>
+    <t>Results should match all entered criteria.</t>
+  </si>
+  <si>
+    <t>Verify Search with Invalid Username</t>
+  </si>
+  <si>
+    <t>No records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid username. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Empty Fields</t>
+  </si>
+  <si>
+    <t>All user records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Leave all fields blank. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Partial Username Search</t>
+  </si>
+  <si>
+    <t>Matching usernames should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter partial username. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Reset Button Functionality</t>
+  </si>
+  <si>
+    <t>Filters should clear and default list should display.</t>
+  </si>
+  <si>
+    <t>Verify Search Result Accuracy</t>
+  </si>
+  <si>
+    <t>1. Search existing user.</t>
+  </si>
+  <si>
+    <t>Displayed results should exactly match search criteria.</t>
+  </si>
+  <si>
+    <t>TC134</t>
+  </si>
+  <si>
+    <t>TC135</t>
+  </si>
+  <si>
+    <t>TC136</t>
+  </si>
+  <si>
+    <t>TC137</t>
+  </si>
+  <si>
+    <t>TC138</t>
+  </si>
+  <si>
+    <t>TC139</t>
+  </si>
+  <si>
+    <t>TC140</t>
+  </si>
+  <si>
+    <t>TC141</t>
+  </si>
+  <si>
+    <t>TC142</t>
+  </si>
+  <si>
+    <t>TC143</t>
   </si>
 </sst>
 </file>
@@ -2118,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -5213,6 +5324,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="135" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A135" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G135" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G137" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A138" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G138" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A139" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G139" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A140" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G140" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A141" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G141" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A142" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A143" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G143" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A144" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G144" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS022 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="608">
   <si>
     <t>TC ID</t>
   </si>
@@ -1889,6 +1889,137 @@
   </si>
   <si>
     <t>TC143</t>
+  </si>
+  <si>
+    <t>My Info</t>
+  </si>
+  <si>
+    <t>Verify Personal Details Display</t>
+  </si>
+  <si>
+    <t>1. Navigate to My Info → Personal Details.</t>
+  </si>
+  <si>
+    <t>Employee personal information should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Update Personal Information</t>
+  </si>
+  <si>
+    <t>Updated personal information should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Edit personal details. 
+2. Click Save.</t>
+  </si>
+  <si>
+    <t>Verify Employee Name Update</t>
+  </si>
+  <si>
+    <t>Employee name should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Modify employee name fields. 
+2. Save changes.</t>
+  </si>
+  <si>
+    <t>Verify Nationality Selection</t>
+  </si>
+  <si>
+    <t>Selected nationality should be saved correctly.</t>
+  </si>
+  <si>
+    <t>1. Select a nationality from dropdown. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Marital Status Update</t>
+  </si>
+  <si>
+    <t>Marital status should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Change marital status. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Gender Selection</t>
+  </si>
+  <si>
+    <t>Selected gender should be stored correctly.</t>
+  </si>
+  <si>
+    <t>1. Select gender. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Date of Birth Update</t>
+  </si>
+  <si>
+    <t>Date of Birth should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Select Date of Birth. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Driver's License Details</t>
+  </si>
+  <si>
+    <t>License information should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter Driver's License Number and Expiry Date. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Custom Fields Update</t>
+  </si>
+  <si>
+    <t>Custom field information should be updated successfully.</t>
+  </si>
+  <si>
+    <t>1. Modify custom field values. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Attachment Upload</t>
+  </si>
+  <si>
+    <t>1. Click Add in Attachments section. 2. Upload file.</t>
+  </si>
+  <si>
+    <t>Attachment should be uploaded successfully.</t>
+  </si>
+  <si>
+    <t>TC144</t>
+  </si>
+  <si>
+    <t>TC145</t>
+  </si>
+  <si>
+    <t>TC146</t>
+  </si>
+  <si>
+    <t>TC147</t>
+  </si>
+  <si>
+    <t>TC148</t>
+  </si>
+  <si>
+    <t>TC149</t>
+  </si>
+  <si>
+    <t>TC150</t>
+  </si>
+  <si>
+    <t>TC151</t>
+  </si>
+  <si>
+    <t>TC152</t>
+  </si>
+  <si>
+    <t>TC153</t>
   </si>
 </sst>
 </file>
@@ -2229,7 +2360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G144"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -5554,6 +5685,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="145" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A145" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G145" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A146" s="1" t="s">
+        <v>599</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A147" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G147" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A148" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A149" s="1" t="s">
+        <v>602</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G149" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A150" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G150" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A151" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G151" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A152" s="1" t="s">
+        <v>605</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G152" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A153" s="1" t="s">
+        <v>606</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="F153" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G153" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A154" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G154" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS023 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="648">
   <si>
     <t>TC ID</t>
   </si>
@@ -2020,6 +2020,135 @@
   </si>
   <si>
     <t>TC153</t>
+  </si>
+  <si>
+    <t>Verify Emergency Contacts Page Load</t>
+  </si>
+  <si>
+    <t>1. Navigate to My Info → Emergency Contacts.</t>
+  </si>
+  <si>
+    <t>Emergency Contacts page should load successfully.</t>
+  </si>
+  <si>
+    <t>Verify Add Emergency Contact</t>
+  </si>
+  <si>
+    <t>Emergency contact should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add. 
+2. Enter valid contact details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Mandatory Field Validation</t>
+  </si>
+  <si>
+    <t>Validation messages should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Leave required fields blank. 
+2. Click Save.</t>
+  </si>
+  <si>
+    <t>Verify Edit Emergency Contact</t>
+  </si>
+  <si>
+    <t>Updated contact information should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Select contact. 
+2. Edit details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Delete Emergency Contact</t>
+  </si>
+  <si>
+    <t>Contact should be removed successfully.</t>
+  </si>
+  <si>
+    <t>Verify Relationship Field</t>
+  </si>
+  <si>
+    <t>Relationship should be stored correctly.</t>
+  </si>
+  <si>
+    <t>1. Select contact. 
+2. Delete record.</t>
+  </si>
+  <si>
+    <t>1. Enter relationship information. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Phone Number Validation</t>
+  </si>
+  <si>
+    <t>Validation error should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid phone number. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Multiple Emergency Contacts</t>
+  </si>
+  <si>
+    <t>1. Add multiple contacts.</t>
+  </si>
+  <si>
+    <t>All contacts should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Contact Information Accuracy</t>
+  </si>
+  <si>
+    <t>1. Open saved contact.</t>
+  </si>
+  <si>
+    <t>Stored information should match entered data.</t>
+  </si>
+  <si>
+    <t>Verify Contact Persistence</t>
+  </si>
+  <si>
+    <t>Contact details should remain available.</t>
+  </si>
+  <si>
+    <t>1. Save contact. 
+2. Refresh page.</t>
+  </si>
+  <si>
+    <t>TC154</t>
+  </si>
+  <si>
+    <t>TC155</t>
+  </si>
+  <si>
+    <t>TC156</t>
+  </si>
+  <si>
+    <t>TC157</t>
+  </si>
+  <si>
+    <t>TC158</t>
+  </si>
+  <si>
+    <t>TC159</t>
+  </si>
+  <si>
+    <t>TC160</t>
+  </si>
+  <si>
+    <t>TC161</t>
+  </si>
+  <si>
+    <t>TC162</t>
+  </si>
+  <si>
+    <t>TC163</t>
   </si>
 </sst>
 </file>
@@ -2063,7 +2192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2079,6 +2208,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2360,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -5915,6 +6047,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="155" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G155" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A156" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G156" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G157" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A158" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G158" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A159" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="F159" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G159" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A160" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G160" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A161" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="F161" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G161" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G162" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="E163" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G163" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A164" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G164" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS024 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="686">
   <si>
     <t>TC ID</t>
   </si>
@@ -2149,6 +2149,135 @@
   </si>
   <si>
     <t>TC163</t>
+  </si>
+  <si>
+    <t>Verify Qualifications Page Load</t>
+  </si>
+  <si>
+    <t>1. Navigate to My Info → Qualifications.</t>
+  </si>
+  <si>
+    <t>Qualifications page should load successfully.</t>
+  </si>
+  <si>
+    <t>Verify Add Education Qualification</t>
+  </si>
+  <si>
+    <t>Education qualification should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add Education. 
+2. Enter qualification details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Add Work Experience</t>
+  </si>
+  <si>
+    <t>Work experience record should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add Work Experience. 
+2. Enter details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Add Skill Record</t>
+  </si>
+  <si>
+    <t>Skill record should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add Skill. 
+2. Enter skill details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Add Language Qualification</t>
+  </si>
+  <si>
+    <t>Language qualification should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add Language. 
+2. Enter language details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Add License Record</t>
+  </si>
+  <si>
+    <t>1. Click Add License. 
+2. Enter details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Edit Qualification Record</t>
+  </si>
+  <si>
+    <t>Updated qualification should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Select qualification. 
+2. Edit details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Delete Qualification Record</t>
+  </si>
+  <si>
+    <t>Qualification should be removed successfully.</t>
+  </si>
+  <si>
+    <t>1. Select qualification. 
+2. Delete record.</t>
+  </si>
+  <si>
+    <t>Validation messages should appear.</t>
+  </si>
+  <si>
+    <t>1. Leave required fields blank. 
+2. Save.</t>
+  </si>
+  <si>
+    <t>Verify Qualification Data Persistence</t>
+  </si>
+  <si>
+    <t>Saved qualification details should remain available.</t>
+  </si>
+  <si>
+    <t>1. Save qualification. 
+2. Refresh page.</t>
+  </si>
+  <si>
+    <t>TC164</t>
+  </si>
+  <si>
+    <t>TC165</t>
+  </si>
+  <si>
+    <t>TC166</t>
+  </si>
+  <si>
+    <t>TC167</t>
+  </si>
+  <si>
+    <t>TC168</t>
+  </si>
+  <si>
+    <t>TC169</t>
+  </si>
+  <si>
+    <t>TC170</t>
+  </si>
+  <si>
+    <t>TC171</t>
+  </si>
+  <si>
+    <t>TC172</t>
+  </si>
+  <si>
+    <t>TC173</t>
   </si>
 </sst>
 </file>
@@ -2492,7 +2621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G187"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -6277,6 +6406,340 @@
         <v>36</v>
       </c>
     </row>
+    <row r="165" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A165" s="1" t="s">
+        <v>676</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="F165" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G165" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A166" s="1" t="s">
+        <v>677</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G166" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A167" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G167" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A168" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G168" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G169" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A170" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G170" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
+        <v>682</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="E171" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="F171" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G171" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A172" s="1" t="s">
+        <v>683</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G172" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A173" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="F173" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G173" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A174" s="1" t="s">
+        <v>685</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="F174" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G174" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F175" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G175" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F176" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G176" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="177" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F177" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G177" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="178" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F178" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G178" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="179" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F179" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G179" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="180" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F180" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G180" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="181" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F181" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G181" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="182" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F182" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G182" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="183" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F183" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G183" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="184" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F184" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G184" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="185" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F185" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G185" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="186" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F186" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G186" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="187" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F187" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G187" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS025 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="725">
   <si>
     <t>TC ID</t>
   </si>
@@ -2278,6 +2278,128 @@
   </si>
   <si>
     <t>TC173</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>Verify Search Page Access</t>
+  </si>
+  <si>
+    <t>1. Click Search icon from menu.</t>
+  </si>
+  <si>
+    <t>Search page should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify Search Box Availability</t>
+  </si>
+  <si>
+    <t>1. Open Search page.</t>
+  </si>
+  <si>
+    <t>Search input field should be displayed and accessible.</t>
+  </si>
+  <si>
+    <t>Verify Search with Valid Keyword</t>
+  </si>
+  <si>
+    <t>Relevant search results should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter valid keyword. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Partial Keyword</t>
+  </si>
+  <si>
+    <t>1. Enter partial text. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Exact Match</t>
+  </si>
+  <si>
+    <t>Exact matching result should appear.</t>
+  </si>
+  <si>
+    <t>1. Enter exact employee/module name. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Invalid Keyword</t>
+  </si>
+  <si>
+    <t>No matching records message should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid keyword. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Empty Input</t>
+  </si>
+  <si>
+    <t>Validation message or default behavior should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Leave search field blank. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>1. Search using existing data.</t>
+  </si>
+  <si>
+    <t>Results should match entered search criteria.</t>
+  </si>
+  <si>
+    <t>Verify Case-Insensitive Search</t>
+  </si>
+  <si>
+    <t>1. Search using uppercase and lowercase values.</t>
+  </si>
+  <si>
+    <t>Same results should be returned regardless of case.</t>
+  </si>
+  <si>
+    <t>Verify Search Response Time</t>
+  </si>
+  <si>
+    <t>1. Perform search operation.</t>
+  </si>
+  <si>
+    <t>Results should be displayed within acceptable response time.</t>
+  </si>
+  <si>
+    <t>TC174</t>
+  </si>
+  <si>
+    <t>TC175</t>
+  </si>
+  <si>
+    <t>TC176</t>
+  </si>
+  <si>
+    <t>TC177</t>
+  </si>
+  <si>
+    <t>TC178</t>
+  </si>
+  <si>
+    <t>TC179</t>
+  </si>
+  <si>
+    <t>TC180</t>
+  </si>
+  <si>
+    <t>TC181</t>
+  </si>
+  <si>
+    <t>TC182</t>
+  </si>
+  <si>
+    <t>TC183</t>
   </si>
 </sst>
 </file>
@@ -6637,6 +6759,21 @@
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>689</v>
+      </c>
       <c r="F175" s="3" t="s">
         <v>12</v>
       </c>
@@ -6644,7 +6781,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
+        <v>716</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>692</v>
+      </c>
       <c r="F176" s="3" t="s">
         <v>12</v>
       </c>
@@ -6652,7 +6804,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="177" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C177" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D177" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="E177" s="2" t="s">
+        <v>694</v>
+      </c>
       <c r="F177" s="3" t="s">
         <v>12</v>
       </c>
@@ -6660,7 +6827,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="178" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
+        <v>718</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="E178" s="2" t="s">
+        <v>205</v>
+      </c>
       <c r="F178" s="3" t="s">
         <v>12</v>
       </c>
@@ -6668,7 +6850,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="179" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
+        <v>719</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="D179" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="E179" s="2" t="s">
+        <v>699</v>
+      </c>
       <c r="F179" s="3" t="s">
         <v>12</v>
       </c>
@@ -6676,7 +6873,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="180" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E180" s="2" t="s">
+        <v>702</v>
+      </c>
       <c r="F180" s="3" t="s">
         <v>12</v>
       </c>
@@ -6684,7 +6896,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="181" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A181" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="D181" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="E181" s="2" t="s">
+        <v>705</v>
+      </c>
       <c r="F181" s="3" t="s">
         <v>12</v>
       </c>
@@ -6692,7 +6919,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="182" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="B182" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D182" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="E182" s="2" t="s">
+        <v>708</v>
+      </c>
       <c r="F182" s="3" t="s">
         <v>12</v>
       </c>
@@ -6700,7 +6942,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="183" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A183" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="B183" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="D183" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="E183" s="2" t="s">
+        <v>711</v>
+      </c>
       <c r="F183" s="3" t="s">
         <v>12</v>
       </c>
@@ -6708,7 +6965,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="184" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A184" s="1" t="s">
+        <v>724</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="D184" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="E184" s="2" t="s">
+        <v>714</v>
+      </c>
       <c r="F184" s="3" t="s">
         <v>12</v>
       </c>
@@ -6716,7 +6988,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="185" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F185" s="3" t="s">
         <v>12</v>
       </c>
@@ -6724,7 +6996,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="186" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F186" s="3" t="s">
         <v>12</v>
       </c>
@@ -6732,7 +7004,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F187" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
TS026 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="725">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="753">
   <si>
     <t>TC ID</t>
   </si>
@@ -2400,6 +2400,95 @@
   </si>
   <si>
     <t>TC183</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Verify Employee Review Search Page</t>
+  </si>
+  <si>
+    <t>1. Navigate to Performance → Manage Reviews → Employee Reviews.</t>
+  </si>
+  <si>
+    <t>Employee Reviews page should open successfully.</t>
+  </si>
+  <si>
+    <t>Matching employee review records should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Search by Job Title</t>
+  </si>
+  <si>
+    <t>Reviews matching selected job title should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Search by Review Status</t>
+  </si>
+  <si>
+    <t>Reviews with selected status should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Review Status. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search by Date Range</t>
+  </si>
+  <si>
+    <t>Reviews within selected date range should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select From Date and To Date. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search Using Multiple Filters</t>
+  </si>
+  <si>
+    <t>Filtered review records should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Select Job Title and Review Status.
+3. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Reset Functionality</t>
+  </si>
+  <si>
+    <t>All filter fields should be cleared/reset.</t>
+  </si>
+  <si>
+    <t>Verify Search with No Matching Data</t>
+  </si>
+  <si>
+    <t>1. Enter invalid search criteria. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>TC184</t>
+  </si>
+  <si>
+    <t>TC185</t>
+  </si>
+  <si>
+    <t>TC186</t>
+  </si>
+  <si>
+    <t>TC187</t>
+  </si>
+  <si>
+    <t>TC188</t>
+  </si>
+  <si>
+    <t>TC189</t>
+  </si>
+  <si>
+    <t>TC190</t>
+  </si>
+  <si>
+    <t>TC191</t>
   </si>
 </sst>
 </file>
@@ -2743,7 +2832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:G192"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -6988,7 +7077,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A185" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="D185" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="E185" s="2" t="s">
+        <v>728</v>
+      </c>
       <c r="F185" s="3" t="s">
         <v>12</v>
       </c>
@@ -6996,7 +7100,22 @@
         <v>36</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A186" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D186" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E186" s="2" t="s">
+        <v>729</v>
+      </c>
       <c r="F186" s="3" t="s">
         <v>12</v>
       </c>
@@ -7004,11 +7123,141 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="D187" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E187" s="2" t="s">
+        <v>731</v>
+      </c>
       <c r="F187" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G187" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A188" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C188" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="D188" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="E188" s="2" t="s">
+        <v>733</v>
+      </c>
+      <c r="F188" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G188" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="D189" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="E189" s="2" t="s">
+        <v>736</v>
+      </c>
+      <c r="F189" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G189" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A190" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="D190" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="E190" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="F190" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G190" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A191" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>741</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="F191" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G191" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A192" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="D192" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="E192" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F192" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G192" s="3" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
TS027 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="783">
   <si>
     <t>TC ID</t>
   </si>
@@ -2489,6 +2489,103 @@
   </si>
   <si>
     <t>TC191</t>
+  </si>
+  <si>
+    <t>Verify Filter by Review Status</t>
+  </si>
+  <si>
+    <t>Records should be filtered based on selected status.</t>
+  </si>
+  <si>
+    <t>1. Select Review Status filter. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Reviewer</t>
+  </si>
+  <si>
+    <t>Matching review records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Reviewer name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Employee Name</t>
+  </si>
+  <si>
+    <t>Relevant employee reviews should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Job Title</t>
+  </si>
+  <si>
+    <t>Reviews for selected job title should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Job Title. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Include Option</t>
+  </si>
+  <si>
+    <t>1. Change Include dropdown value. 2. Search.</t>
+  </si>
+  <si>
+    <t>Results should be filtered according to selected option.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Date Range</t>
+  </si>
+  <si>
+    <t>Reviews within selected dates should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select From Date and To Date. 
+2. Search.</t>
+  </si>
+  <si>
+    <t>Verify Combined Filter Criteria</t>
+  </si>
+  <si>
+    <t>Results should satisfy all selected filter criteria.</t>
+  </si>
+  <si>
+    <t>1. Apply multiple filters. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>1. Apply filters. 
+2. Click Reset.</t>
+  </si>
+  <si>
+    <t>TC192</t>
+  </si>
+  <si>
+    <t>TC193</t>
+  </si>
+  <si>
+    <t>TC194</t>
+  </si>
+  <si>
+    <t>TC195</t>
+  </si>
+  <si>
+    <t>TC196</t>
+  </si>
+  <si>
+    <t>TC197</t>
+  </si>
+  <si>
+    <t>TC198</t>
+  </si>
+  <si>
+    <t>TC199</t>
   </si>
 </sst>
 </file>
@@ -2832,7 +2929,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G192"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -7261,6 +7358,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="193" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A193" s="1" t="s">
+        <v>775</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="D193" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="E193" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="F193" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G193" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A194" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="D194" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="E194" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G194" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A195" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>759</v>
+      </c>
+      <c r="D195" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="E195" s="2" t="s">
+        <v>760</v>
+      </c>
+      <c r="F195" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G195" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A196" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="D196" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="E196" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="F196" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G196" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A197" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>765</v>
+      </c>
+      <c r="D197" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="E197" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="F197" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G197" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A198" s="1" t="s">
+        <v>780</v>
+      </c>
+      <c r="B198" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>768</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="E198" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="F198" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G198" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A199" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="D199" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="E199" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="F199" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G199" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A200" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D200" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="E200" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="F200" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G200" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS028 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="783">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="823">
   <si>
     <t>TC ID</t>
   </si>
@@ -2586,6 +2586,131 @@
   </si>
   <si>
     <t>TC199</t>
+  </si>
+  <si>
+    <t>Verify Review Records Display</t>
+  </si>
+  <si>
+    <t>1. Open Manage Reviews page.</t>
+  </si>
+  <si>
+    <t>Existing review records should be displayed in grid.</t>
+  </si>
+  <si>
+    <t>Verify Review Details Display</t>
+  </si>
+  <si>
+    <t>1. Open review record.</t>
+  </si>
+  <si>
+    <t>Review details should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Add Review Functionality</t>
+  </si>
+  <si>
+    <t>New review should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Add button. 
+2. Enter review details. 
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Edit Review Functionality</t>
+  </si>
+  <si>
+    <t>Changes should be saved successfully.</t>
+  </si>
+  <si>
+    <t>1. Select existing review. 
+2. Edit details.
+3. Save.</t>
+  </si>
+  <si>
+    <t>Verify Delete Review Functionality</t>
+  </si>
+  <si>
+    <t>Review should be removed successfully.</t>
+  </si>
+  <si>
+    <t>1. Select review record. 
+2. Delete record.</t>
+  </si>
+  <si>
+    <t>Verify My Reviews Display</t>
+  </si>
+  <si>
+    <t>1. Navigate to My Reviews section.</t>
+  </si>
+  <si>
+    <t>Assigned reviews should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify My Trackers Display</t>
+  </si>
+  <si>
+    <t>1. Open My Trackers tab.</t>
+  </si>
+  <si>
+    <t>User's trackers should be displayed successfully.</t>
+  </si>
+  <si>
+    <t>Verify Employee Trackers Display</t>
+  </si>
+  <si>
+    <t>1. Open Employee Trackers tab.</t>
+  </si>
+  <si>
+    <t>Employee tracker records should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify View Tracker Details</t>
+  </si>
+  <si>
+    <t>1. Click View button for tracker.</t>
+  </si>
+  <si>
+    <t>Tracker information should be displayed successfully.</t>
+  </si>
+  <si>
+    <t>Verify Review Records Sorting</t>
+  </si>
+  <si>
+    <t>1. Click column sort icon.</t>
+  </si>
+  <si>
+    <t>Records should be sorted correctly in ascending/descending order.</t>
+  </si>
+  <si>
+    <t>TC200</t>
+  </si>
+  <si>
+    <t>TC201</t>
+  </si>
+  <si>
+    <t>TC202</t>
+  </si>
+  <si>
+    <t>TC203</t>
+  </si>
+  <si>
+    <t>TC204</t>
+  </si>
+  <si>
+    <t>TC205</t>
+  </si>
+  <si>
+    <t>TC206</t>
+  </si>
+  <si>
+    <t>TC207</t>
+  </si>
+  <si>
+    <t>TC208</t>
+  </si>
+  <si>
+    <t>TC209</t>
   </si>
 </sst>
 </file>
@@ -2929,7 +3054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G210"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -7542,6 +7667,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="201" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A201" s="1" t="s">
+        <v>813</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>783</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="E201" s="2" t="s">
+        <v>785</v>
+      </c>
+      <c r="F201" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G201" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A202" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="B202" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>786</v>
+      </c>
+      <c r="D202" s="2" t="s">
+        <v>787</v>
+      </c>
+      <c r="E202" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="F202" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G202" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A203" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C203" s="2" t="s">
+        <v>789</v>
+      </c>
+      <c r="D203" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="E203" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="F203" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G203" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A204" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="D204" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="E204" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="F204" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G204" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A205" s="1" t="s">
+        <v>817</v>
+      </c>
+      <c r="B205" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="D205" s="2" t="s">
+        <v>797</v>
+      </c>
+      <c r="E205" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="F205" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G205" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A206" s="1" t="s">
+        <v>818</v>
+      </c>
+      <c r="B206" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="D206" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="E206" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="F206" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G206" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A207" s="1" t="s">
+        <v>819</v>
+      </c>
+      <c r="B207" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="D207" s="2" t="s">
+        <v>802</v>
+      </c>
+      <c r="E207" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="F207" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G207" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A208" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="B208" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="D208" s="2" t="s">
+        <v>805</v>
+      </c>
+      <c r="E208" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="F208" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G208" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A209" s="1" t="s">
+        <v>821</v>
+      </c>
+      <c r="B209" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="D209" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="E209" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="F209" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G209" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A210" s="1" t="s">
+        <v>822</v>
+      </c>
+      <c r="B210" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="D210" s="2" t="s">
+        <v>811</v>
+      </c>
+      <c r="E210" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="F210" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G210" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS029 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="823">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="850">
   <si>
     <t>TC ID</t>
   </si>
@@ -2711,6 +2711,91 @@
   </si>
   <si>
     <t>TC209</t>
+  </si>
+  <si>
+    <t>Directory</t>
+  </si>
+  <si>
+    <t>Verify Directory Page Access</t>
+  </si>
+  <si>
+    <t>1. Navigate to Directory module.</t>
+  </si>
+  <si>
+    <t>Directory page should open successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter employee name in Employee Name field. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Partial Employee Name Search</t>
+  </si>
+  <si>
+    <t>Relevant employee records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter partial employee name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search with Full Employee Name</t>
+  </si>
+  <si>
+    <t>1. Enter complete employee name. 2. Click Search.</t>
+  </si>
+  <si>
+    <t>Exact employee profile should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Search with Invalid Employee Name</t>
+  </si>
+  <si>
+    <t>No matching records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid employee name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search Button Functionality</t>
+  </si>
+  <si>
+    <t>Search should execute successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter search criteria. 
+2. Click Search button.</t>
+  </si>
+  <si>
+    <t>Verify Search Results Count</t>
+  </si>
+  <si>
+    <t>1. Perform search.</t>
+  </si>
+  <si>
+    <t>Record count should match displayed employee cards.</t>
+  </si>
+  <si>
+    <t>TC210</t>
+  </si>
+  <si>
+    <t>TC211</t>
+  </si>
+  <si>
+    <t>TC212</t>
+  </si>
+  <si>
+    <t>TC213</t>
+  </si>
+  <si>
+    <t>TC214</t>
+  </si>
+  <si>
+    <t>TC215</t>
+  </si>
+  <si>
+    <t>TC216</t>
   </si>
 </sst>
 </file>
@@ -3054,7 +3139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G210"/>
+  <dimension ref="A1:G217"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -7897,6 +7982,167 @@
         <v>36</v>
       </c>
     </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A211" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="B211" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="D211" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="E211" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="F211" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G211" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A212" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="B212" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D212" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="E212" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G212" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A213" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B213" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="D213" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="E213" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G213" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A214" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="B214" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>831</v>
+      </c>
+      <c r="D214" s="2" t="s">
+        <v>832</v>
+      </c>
+      <c r="E214" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="F214" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G214" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A215" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="B215" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="E215" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="F215" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G215" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A216" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="B216" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>837</v>
+      </c>
+      <c r="D216" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="E216" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="F216" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G216" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A217" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="B217" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C217" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="D217" s="2" t="s">
+        <v>841</v>
+      </c>
+      <c r="E217" s="2" t="s">
+        <v>842</v>
+      </c>
+      <c r="F217" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G217" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS030 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="850">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="874">
   <si>
     <t>TC ID</t>
   </si>
@@ -2796,6 +2796,88 @@
   </si>
   <si>
     <t>TC216</t>
+  </si>
+  <si>
+    <t>Employees matching selected job title should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select a Job Title. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Location</t>
+  </si>
+  <si>
+    <t>Employees from selected location should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Location. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Employee Name and Job Title</t>
+  </si>
+  <si>
+    <t>Filtered employee records should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Select Job Title. 
+3. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter by Employee Name and Location</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Select Location. 
+3. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Filter Using All Fields</t>
+  </si>
+  <si>
+    <t>Results should satisfy all filter conditions.</t>
+  </si>
+  <si>
+    <t>1. Enter Employee Name. 
+2. Select Job Title. 
+3. Select Location.
+ 4. Click Search.</t>
+  </si>
+  <si>
+    <t>All filter values should be cleared.</t>
+  </si>
+  <si>
+    <t>Verify Search After Reset</t>
+  </si>
+  <si>
+    <t>All employee records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Click Reset. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>TC217</t>
+  </si>
+  <si>
+    <t>TC218</t>
+  </si>
+  <si>
+    <t>TC219</t>
+  </si>
+  <si>
+    <t>TC220</t>
+  </si>
+  <si>
+    <t>TC221</t>
+  </si>
+  <si>
+    <t>TC222</t>
+  </si>
+  <si>
+    <t>TC223</t>
   </si>
 </sst>
 </file>
@@ -3139,7 +3221,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G217"/>
+  <dimension ref="A1:G224"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -8143,6 +8225,167 @@
         <v>36</v>
       </c>
     </row>
+    <row r="218" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A218" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="B218" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="F218" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G218" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A219" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="B219" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="D219" s="2" t="s">
+        <v>854</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="F219" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G219" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A220" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>855</v>
+      </c>
+      <c r="D220" s="2" t="s">
+        <v>857</v>
+      </c>
+      <c r="E220" s="2" t="s">
+        <v>856</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G220" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A221" s="1" t="s">
+        <v>870</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>858</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>859</v>
+      </c>
+      <c r="E221" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G221" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A222" s="1" t="s">
+        <v>871</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="D222" s="2" t="s">
+        <v>862</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>861</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G222" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A223" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D223" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="E223" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G223" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A224" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>864</v>
+      </c>
+      <c r="D224" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>865</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G224" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS031 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1624" uniqueCount="903">
   <si>
     <t>TC ID</t>
   </si>
@@ -2878,6 +2878,93 @@
   </si>
   <si>
     <t>TC223</t>
+  </si>
+  <si>
+    <t>Verify Employee Cards Display</t>
+  </si>
+  <si>
+    <t>1. Open Directory page.</t>
+  </si>
+  <si>
+    <t>Employee cards should be displayed properly.</t>
+  </si>
+  <si>
+    <t>Verify Employee Name Display</t>
+  </si>
+  <si>
+    <t>1. View employee card.</t>
+  </si>
+  <si>
+    <t>Employee name should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Employee Profile Image Display</t>
+  </si>
+  <si>
+    <t>Profile image/avatar should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Multiple Employee Records Display</t>
+  </si>
+  <si>
+    <t>Multiple employee records should be visible.</t>
+  </si>
+  <si>
+    <t>Verify Employee Information Consistency</t>
+  </si>
+  <si>
+    <t>1. Compare employee information with employee profile.</t>
+  </si>
+  <si>
+    <t>Information should match system records.</t>
+  </si>
+  <si>
+    <t>Verify Record Count Display</t>
+  </si>
+  <si>
+    <t>Total records count should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Employee Card Layout</t>
+  </si>
+  <si>
+    <t>1. View employee directory cards.</t>
+  </si>
+  <si>
+    <t>Cards should be aligned and displayed properly.</t>
+  </si>
+  <si>
+    <t>Verify Employee Details Accessibility</t>
+  </si>
+  <si>
+    <t>1. Select an employee card (if clickable).</t>
+  </si>
+  <si>
+    <t>Employee details should be accessible successfully.</t>
+  </si>
+  <si>
+    <t>TC224</t>
+  </si>
+  <si>
+    <t>TC225</t>
+  </si>
+  <si>
+    <t>TC226</t>
+  </si>
+  <si>
+    <t>TC227</t>
+  </si>
+  <si>
+    <t>TC228</t>
+  </si>
+  <si>
+    <t>TC229</t>
+  </si>
+  <si>
+    <t>TC230</t>
+  </si>
+  <si>
+    <t>TC231</t>
   </si>
 </sst>
 </file>
@@ -3221,7 +3308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G224"/>
+  <dimension ref="A1:G232"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -8386,6 +8473,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A225" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C225" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="E225" s="2" t="s">
+        <v>876</v>
+      </c>
+      <c r="F225" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G225" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A226" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>877</v>
+      </c>
+      <c r="D226" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="E226" s="2" t="s">
+        <v>879</v>
+      </c>
+      <c r="F226" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G226" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A227" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>880</v>
+      </c>
+      <c r="D227" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="E227" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="F227" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G227" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A228" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="B228" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="D228" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="E228" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="F228" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G228" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A229" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C229" s="2" t="s">
+        <v>884</v>
+      </c>
+      <c r="D229" s="2" t="s">
+        <v>885</v>
+      </c>
+      <c r="E229" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="F229" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G229" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A230" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="D230" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="E230" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="F230" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G230" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A231" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="D231" s="2" t="s">
+        <v>890</v>
+      </c>
+      <c r="E231" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="F231" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G231" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A232" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>892</v>
+      </c>
+      <c r="D232" s="2" t="s">
+        <v>893</v>
+      </c>
+      <c r="E232" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="F232" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G232" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS032 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1624" uniqueCount="903">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1680" uniqueCount="929">
   <si>
     <t>TC ID</t>
   </si>
@@ -2965,6 +2965,88 @@
   </si>
   <si>
     <t>TC231</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Verify Purge Employee Records Page Access</t>
+  </si>
+  <si>
+    <t>1. Navigate to Maintenance → Purge Records.</t>
+  </si>
+  <si>
+    <t>Purge Employee Records page should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify Search Field Availability</t>
+  </si>
+  <si>
+    <t>1. Open Purge Employee Records page.</t>
+  </si>
+  <si>
+    <t>Past Employee search field should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Search Past Employee Record</t>
+  </si>
+  <si>
+    <t>Verify Search with Partial Employee Name</t>
+  </si>
+  <si>
+    <t>No matching record should be found.</t>
+  </si>
+  <si>
+    <t>Verify Mandatory Employee Field Validation</t>
+  </si>
+  <si>
+    <t>1. Leave employee field blank. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Purge Employee Record Process</t>
+  </si>
+  <si>
+    <t>Employee record should be permanently removed.</t>
+  </si>
+  <si>
+    <t>1. Search past employee. 
+2. Select employee. 
+3. Purge record.</t>
+  </si>
+  <si>
+    <t>Verify Purged Employee Record Unavailability</t>
+  </si>
+  <si>
+    <t>Purged employee should not appear in search results.</t>
+  </si>
+  <si>
+    <t>1. Purge employee record. 
+2. Search again.</t>
+  </si>
+  <si>
+    <t>TC232</t>
+  </si>
+  <si>
+    <t>TC233</t>
+  </si>
+  <si>
+    <t>TC234</t>
+  </si>
+  <si>
+    <t>TC235</t>
+  </si>
+  <si>
+    <t>TC236</t>
+  </si>
+  <si>
+    <t>TC237</t>
+  </si>
+  <si>
+    <t>TC238</t>
+  </si>
+  <si>
+    <t>TC239</t>
   </si>
 </sst>
 </file>
@@ -3308,11 +3390,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G232"/>
+  <dimension ref="A1:G240"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -8657,6 +8739,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="233" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A233" s="1" t="s">
+        <v>921</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C233" s="2" t="s">
+        <v>904</v>
+      </c>
+      <c r="D233" s="2" t="s">
+        <v>905</v>
+      </c>
+      <c r="E233" s="2" t="s">
+        <v>906</v>
+      </c>
+      <c r="F233" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G233" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A234" s="1" t="s">
+        <v>922</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>907</v>
+      </c>
+      <c r="D234" s="2" t="s">
+        <v>908</v>
+      </c>
+      <c r="E234" s="2" t="s">
+        <v>909</v>
+      </c>
+      <c r="F234" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G234" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A235" s="1" t="s">
+        <v>923</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C235" s="2" t="s">
+        <v>910</v>
+      </c>
+      <c r="D235" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E235" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="F235" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G235" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A236" s="1" t="s">
+        <v>924</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>911</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="E236" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="F236" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G236" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A237" s="1" t="s">
+        <v>925</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C237" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="D237" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="E237" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="F237" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G237" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A238" s="1" t="s">
+        <v>926</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="D238" s="2" t="s">
+        <v>914</v>
+      </c>
+      <c r="E238" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F238" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G238" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A239" s="1" t="s">
+        <v>927</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C239" s="2" t="s">
+        <v>915</v>
+      </c>
+      <c r="D239" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="E239" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="F239" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G239" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A240" s="1" t="s">
+        <v>928</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C240" s="2" t="s">
+        <v>918</v>
+      </c>
+      <c r="D240" s="2" t="s">
+        <v>920</v>
+      </c>
+      <c r="E240" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="F240" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G240" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS033 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1680" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1736" uniqueCount="955">
   <si>
     <t>TC ID</t>
   </si>
@@ -3047,6 +3047,86 @@
   </si>
   <si>
     <t>TC239</t>
+  </si>
+  <si>
+    <t>Verify Access Records Page Access</t>
+  </si>
+  <si>
+    <t>1. Navigate to Maintenance → Access Records.</t>
+  </si>
+  <si>
+    <t>Access Records page should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify Download Personal Data Page Display</t>
+  </si>
+  <si>
+    <t>1. Open Access Records page.</t>
+  </si>
+  <si>
+    <t>Download Personal Data section should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Employee Search Field Availability</t>
+  </si>
+  <si>
+    <t>1. Open Download Personal Data page.</t>
+  </si>
+  <si>
+    <t>Employee Name search field should be available.</t>
+  </si>
+  <si>
+    <t>Verify Search Employee Personal Data</t>
+  </si>
+  <si>
+    <t>Matching employee information should be retrieved.</t>
+  </si>
+  <si>
+    <t>Verify Search Using Partial Employee Name</t>
+  </si>
+  <si>
+    <t>No matching records should be returned.</t>
+  </si>
+  <si>
+    <t>Verify Mandatory Employee Name Validation</t>
+  </si>
+  <si>
+    <t>1. Leave Employee Name blank. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Personal Data Download Request</t>
+  </si>
+  <si>
+    <t>Personal data request should be processed successfully.</t>
+  </si>
+  <si>
+    <t>1. Search employee. 
+2. Initiate personal data access request.</t>
+  </si>
+  <si>
+    <t>TC240</t>
+  </si>
+  <si>
+    <t>TC241</t>
+  </si>
+  <si>
+    <t>TC242</t>
+  </si>
+  <si>
+    <t>TC243</t>
+  </si>
+  <si>
+    <t>TC244</t>
+  </si>
+  <si>
+    <t>TC245</t>
+  </si>
+  <si>
+    <t>TC246</t>
+  </si>
+  <si>
+    <t>TC247</t>
   </si>
 </sst>
 </file>
@@ -3390,7 +3470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G240"/>
+  <dimension ref="A1:G248"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -8923,6 +9003,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="241" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A241" s="1" t="s">
+        <v>947</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C241" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="D241" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="E241" s="2" t="s">
+        <v>931</v>
+      </c>
+      <c r="F241" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G241" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A242" s="1" t="s">
+        <v>948</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="D242" s="2" t="s">
+        <v>933</v>
+      </c>
+      <c r="E242" s="2" t="s">
+        <v>934</v>
+      </c>
+      <c r="F242" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G242" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A243" s="1" t="s">
+        <v>949</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C243" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="D243" s="2" t="s">
+        <v>936</v>
+      </c>
+      <c r="E243" s="2" t="s">
+        <v>937</v>
+      </c>
+      <c r="F243" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G243" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A244" s="1" t="s">
+        <v>950</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C244" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="D244" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="E244" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="F244" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G244" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A245" s="1" t="s">
+        <v>951</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C245" s="2" t="s">
+        <v>940</v>
+      </c>
+      <c r="D245" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="E245" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="F245" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G245" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A246" s="1" t="s">
+        <v>952</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C246" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="D246" s="2" t="s">
+        <v>836</v>
+      </c>
+      <c r="E246" s="2" t="s">
+        <v>941</v>
+      </c>
+      <c r="F246" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G246" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A247" s="1" t="s">
+        <v>953</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C247" s="2" t="s">
+        <v>942</v>
+      </c>
+      <c r="D247" s="2" t="s">
+        <v>943</v>
+      </c>
+      <c r="E247" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F247" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G247" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A248" s="1" t="s">
+        <v>954</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C248" s="2" t="s">
+        <v>944</v>
+      </c>
+      <c r="D248" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="E248" s="2" t="s">
+        <v>945</v>
+      </c>
+      <c r="F248" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G248" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS034 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1736" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="989">
   <si>
     <t>TC ID</t>
   </si>
@@ -3127,6 +3127,111 @@
   </si>
   <si>
     <t>TC247</t>
+  </si>
+  <si>
+    <t>Verify Administrator Access Prompt</t>
+  </si>
+  <si>
+    <t>1. Navigate to Maintenance module.</t>
+  </si>
+  <si>
+    <t>Administrator Access popup should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Admin Username Display</t>
+  </si>
+  <si>
+    <t>1. Open Administrator Access popup.</t>
+  </si>
+  <si>
+    <t>Logged-in admin username should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Password Field Availability</t>
+  </si>
+  <si>
+    <t>Password field should be available for credential validation.</t>
+  </si>
+  <si>
+    <t>Verify Access with Valid Credentials</t>
+  </si>
+  <si>
+    <t>Access to Maintenance module should be granted.</t>
+  </si>
+  <si>
+    <t>1. Enter valid password. 
+2. Click Confirm.</t>
+  </si>
+  <si>
+    <t>Verify Access with Invalid Credentials</t>
+  </si>
+  <si>
+    <t>Access should be denied and error message displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter incorrect password. 
+2. Click Confirm.</t>
+  </si>
+  <si>
+    <t>Verify Empty Password Validation</t>
+  </si>
+  <si>
+    <t>1. Leave password blank. 
+2. Click Confirm.</t>
+  </si>
+  <si>
+    <t>Verify Cancel Button Functionality</t>
+  </si>
+  <si>
+    <t>1. Click Cancel on Administrator Access popup.</t>
+  </si>
+  <si>
+    <t>Access popup should close and Maintenance page should not open.</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized User Restriction</t>
+  </si>
+  <si>
+    <t>1. Attempt Maintenance access without proper privileges.</t>
+  </si>
+  <si>
+    <t>User should be prevented from accessing Maintenance functions.</t>
+  </si>
+  <si>
+    <t>Verify Session-Based Access Validation</t>
+  </si>
+  <si>
+    <t>1. Access Maintenance module after authentication.</t>
+  </si>
+  <si>
+    <t>Access should remain valid only for authorized session.</t>
+  </si>
+  <si>
+    <t>TC248</t>
+  </si>
+  <si>
+    <t>TC249</t>
+  </si>
+  <si>
+    <t>TC250</t>
+  </si>
+  <si>
+    <t>TC251</t>
+  </si>
+  <si>
+    <t>TC252</t>
+  </si>
+  <si>
+    <t>TC253</t>
+  </si>
+  <si>
+    <t>TC254</t>
+  </si>
+  <si>
+    <t>TC255</t>
+  </si>
+  <si>
+    <t>TC256</t>
   </si>
 </sst>
 </file>
@@ -3470,7 +3575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G248"/>
+  <dimension ref="A1:G257"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -9187,6 +9292,213 @@
         <v>36</v>
       </c>
     </row>
+    <row r="249" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A249" s="1" t="s">
+        <v>980</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C249" s="2" t="s">
+        <v>955</v>
+      </c>
+      <c r="D249" s="2" t="s">
+        <v>956</v>
+      </c>
+      <c r="E249" s="2" t="s">
+        <v>957</v>
+      </c>
+      <c r="F249" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G249" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A250" s="1" t="s">
+        <v>981</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C250" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="D250" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="E250" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="F250" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G250" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A251" s="1" t="s">
+        <v>982</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C251" s="2" t="s">
+        <v>961</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="E251" s="2" t="s">
+        <v>962</v>
+      </c>
+      <c r="F251" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G251" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A252" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C252" s="2" t="s">
+        <v>963</v>
+      </c>
+      <c r="D252" s="2" t="s">
+        <v>965</v>
+      </c>
+      <c r="E252" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="F252" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G252" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A253" s="1" t="s">
+        <v>984</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C253" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="D253" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="E253" s="2" t="s">
+        <v>967</v>
+      </c>
+      <c r="F253" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G253" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A254" s="1" t="s">
+        <v>985</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>969</v>
+      </c>
+      <c r="D254" s="2" t="s">
+        <v>970</v>
+      </c>
+      <c r="E254" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F254" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G254" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A255" s="1" t="s">
+        <v>986</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C255" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="D255" s="2" t="s">
+        <v>972</v>
+      </c>
+      <c r="E255" s="2" t="s">
+        <v>973</v>
+      </c>
+      <c r="F255" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G255" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A256" s="1" t="s">
+        <v>987</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C256" s="2" t="s">
+        <v>974</v>
+      </c>
+      <c r="D256" s="2" t="s">
+        <v>975</v>
+      </c>
+      <c r="E256" s="2" t="s">
+        <v>976</v>
+      </c>
+      <c r="F256" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G256" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A257" s="1" t="s">
+        <v>988</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="C257" s="2" t="s">
+        <v>977</v>
+      </c>
+      <c r="D257" s="2" t="s">
+        <v>978</v>
+      </c>
+      <c r="E257" s="2" t="s">
+        <v>979</v>
+      </c>
+      <c r="F257" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G257" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS035 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="989">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1855" uniqueCount="1020">
   <si>
     <t>TC ID</t>
   </si>
@@ -3232,6 +3232,108 @@
   </si>
   <si>
     <t>TC256</t>
+  </si>
+  <si>
+    <t>Claim</t>
+  </si>
+  <si>
+    <t>Verify Claim Request Creation</t>
+  </si>
+  <si>
+    <t>Claim request should be created successfully.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Claim → Submit Claim. 
+2. Select Event and Currency. 
+3. Enter remarks. 
+4. Click Create.</t>
+  </si>
+  <si>
+    <t>Verify Mandatory Fields Validation</t>
+  </si>
+  <si>
+    <t>1. Leave Event and Currency blank. 2. Click Create.</t>
+  </si>
+  <si>
+    <t>Verify Claim Creation with Valid Data</t>
+  </si>
+  <si>
+    <t>Claim should be submitted successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter all required claim details. 
+2. Click Create.</t>
+  </si>
+  <si>
+    <t>Claim creation should be cancelled and page reset.</t>
+  </si>
+  <si>
+    <t>1. Enter claim details. 
+2. Click Cancel.</t>
+  </si>
+  <si>
+    <t>Verify Employee Claim Assignment</t>
+  </si>
+  <si>
+    <t>Claim should be assigned to selected employee.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Employee Claims. 
+2. Click Assign Claim. 
+3. Select employee and claim details. 
+4. Click Create.</t>
+  </si>
+  <si>
+    <t>Verify Assigned Claim Display</t>
+  </si>
+  <si>
+    <t>Assigned claim should be visible in records list.</t>
+  </si>
+  <si>
+    <t>1. Assign claim to employee. 
+2. Open Employee Claims page.</t>
+  </si>
+  <si>
+    <t>Verify Claim Reference ID Generation</t>
+  </si>
+  <si>
+    <t>1. Create a new claim.</t>
+  </si>
+  <si>
+    <t>Unique claim reference ID should be generated.</t>
+  </si>
+  <si>
+    <t>Verify Assigned Claim Amount Display</t>
+  </si>
+  <si>
+    <t>1. Open Employee Claims page.</t>
+  </si>
+  <si>
+    <t>Correct claim amount should be displayed.</t>
+  </si>
+  <si>
+    <t>TC257</t>
+  </si>
+  <si>
+    <t>TC258</t>
+  </si>
+  <si>
+    <t>TC259</t>
+  </si>
+  <si>
+    <t>TC260</t>
+  </si>
+  <si>
+    <t>TC261</t>
+  </si>
+  <si>
+    <t>TC262</t>
+  </si>
+  <si>
+    <t>TC263</t>
+  </si>
+  <si>
+    <t>TC264</t>
   </si>
 </sst>
 </file>
@@ -3575,7 +3677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G257"/>
+  <dimension ref="A1:G265"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -9499,6 +9601,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="258" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A258" s="1" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C258" s="2" t="s">
+        <v>990</v>
+      </c>
+      <c r="D258" s="2" t="s">
+        <v>992</v>
+      </c>
+      <c r="E258" s="2" t="s">
+        <v>991</v>
+      </c>
+      <c r="F258" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G258" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A259" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C259" s="2" t="s">
+        <v>993</v>
+      </c>
+      <c r="D259" s="2" t="s">
+        <v>994</v>
+      </c>
+      <c r="E259" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F259" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G259" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A260" s="1" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C260" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D260" s="2" t="s">
+        <v>997</v>
+      </c>
+      <c r="E260" s="2" t="s">
+        <v>996</v>
+      </c>
+      <c r="F260" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G260" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A261" s="1" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C261" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="D261" s="2" t="s">
+        <v>999</v>
+      </c>
+      <c r="E261" s="2" t="s">
+        <v>998</v>
+      </c>
+      <c r="F261" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G261" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A262" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C262" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D262" s="2" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E262" s="2" t="s">
+        <v>1001</v>
+      </c>
+      <c r="F262" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G262" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A263" s="1" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C263" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D263" s="2" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E263" s="2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="F263" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G263" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A264" s="1" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C264" s="2" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D264" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E264" s="2" t="s">
+        <v>1008</v>
+      </c>
+      <c r="F264" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G264" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A265" s="1" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C265" s="2" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D265" s="2" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E265" s="2" t="s">
+        <v>1011</v>
+      </c>
+      <c r="F265" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G265" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS036 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1855" uniqueCount="1020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="1055">
   <si>
     <t>TC ID</t>
   </si>
@@ -3334,6 +3334,116 @@
   </si>
   <si>
     <t>TC264</t>
+  </si>
+  <si>
+    <t>Verify My Claims Page Access</t>
+  </si>
+  <si>
+    <t>1. Navigate to Claim → My Claims.</t>
+  </si>
+  <si>
+    <t>My Claims page should open successfully.</t>
+  </si>
+  <si>
+    <t>Verify Search by Reference ID</t>
+  </si>
+  <si>
+    <t>Matching claim record should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter Reference ID. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Search by Event Name</t>
+  </si>
+  <si>
+    <t>Relevant claim records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Event Name. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Claims matching selected status should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Select Status. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Claims within selected date range should be displayed.</t>
+  </si>
+  <si>
+    <t>All search fields should be cleared.</t>
+  </si>
+  <si>
+    <t>Verify View Claim Details</t>
+  </si>
+  <si>
+    <t>1. Click View Details for a claim.</t>
+  </si>
+  <si>
+    <t>Detailed claim information should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Submitted Claims Tracking</t>
+  </si>
+  <si>
+    <t>1. Open My Claims page.</t>
+  </si>
+  <si>
+    <t>Submitted claims and statuses should be visible.</t>
+  </si>
+  <si>
+    <t>Verify Employee Claims Search</t>
+  </si>
+  <si>
+    <t>Matching employee claim records should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Employee Claims. 
+2. Search using employee name or reference ID.</t>
+  </si>
+  <si>
+    <t>Verify Employee Claims Filter by Status</t>
+  </si>
+  <si>
+    <t>Employee claims should be filtered correctly.</t>
+  </si>
+  <si>
+    <t>1. Select Status filter. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>TC265</t>
+  </si>
+  <si>
+    <t>TC266</t>
+  </si>
+  <si>
+    <t>TC267</t>
+  </si>
+  <si>
+    <t>TC268</t>
+  </si>
+  <si>
+    <t>TC269</t>
+  </si>
+  <si>
+    <t>TC270</t>
+  </si>
+  <si>
+    <t>TC271</t>
+  </si>
+  <si>
+    <t>TC272</t>
+  </si>
+  <si>
+    <t>TC273</t>
+  </si>
+  <si>
+    <t>TC274</t>
   </si>
 </sst>
 </file>
@@ -3677,7 +3787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G275"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -9785,6 +9895,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A266" s="1" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C266" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D266" s="2" t="s">
+        <v>1021</v>
+      </c>
+      <c r="E266" s="2" t="s">
+        <v>1022</v>
+      </c>
+      <c r="F266" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G266" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A267" s="1" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C267" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D267" s="2" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E267" s="2" t="s">
+        <v>1024</v>
+      </c>
+      <c r="F267" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G267" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A268" s="1" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C268" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="D268" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="E268" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="F268" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G268" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A269" s="1" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C269" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="D269" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="E269" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="F269" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G269" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A270" s="1" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C270" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="D270" s="2" t="s">
+        <v>737</v>
+      </c>
+      <c r="E270" s="2" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F270" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G270" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A271" s="1" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C271" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="D271" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E271" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="F271" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G271" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A272" s="1" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C272" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D272" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="E272" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="F272" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G272" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A273" s="1" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B273" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C273" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D273" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E273" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="F273" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G273" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A274" s="1" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C274" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D274" s="2" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E274" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="F274" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G274" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A275" s="1" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C275" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D275" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E275" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F275" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G275" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS037 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1925" uniqueCount="1055">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1988" uniqueCount="1089">
   <si>
     <t>TC ID</t>
   </si>
@@ -3444,6 +3444,111 @@
   </si>
   <si>
     <t>TC274</t>
+  </si>
+  <si>
+    <t>Verify Claim Status Display</t>
+  </si>
+  <si>
+    <t>1. Open My Claims or Employee Claims page.</t>
+  </si>
+  <si>
+    <t>Current claim status should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Submitted Status After Claim Creation</t>
+  </si>
+  <si>
+    <t>1. Create and submit claim.</t>
+  </si>
+  <si>
+    <t>Status should be updated to Submitted.</t>
+  </si>
+  <si>
+    <t>Verify Initiated Status Display</t>
+  </si>
+  <si>
+    <t>1. Create draft/initial claim.</t>
+  </si>
+  <si>
+    <t>Status should display as Initiated.</t>
+  </si>
+  <si>
+    <t>Verify Employee Claims Status Tracking</t>
+  </si>
+  <si>
+    <t>Status of each employee claim should be visible.</t>
+  </si>
+  <si>
+    <t>Verify Claim Search Using Status Filter</t>
+  </si>
+  <si>
+    <t>1. Select claim status. 
+2. Click Search.</t>
+  </si>
+  <si>
+    <t>Verify Claim Details Accuracy</t>
+  </si>
+  <si>
+    <t>1. Open claim details page.</t>
+  </si>
+  <si>
+    <t>Claim status, amount, currency, and event should be correct.</t>
+  </si>
+  <si>
+    <t>Verify Assigned Claim Status Update</t>
+  </si>
+  <si>
+    <t>Assigned claim status should update correctly.</t>
+  </si>
+  <si>
+    <t>1. Assign claim to employee. 
+2. Refresh Employee Claims page.</t>
+  </si>
+  <si>
+    <t>Verify Claim Record Consistency</t>
+  </si>
+  <si>
+    <t>1. Compare My Claims and Employee Claims records.</t>
+  </si>
+  <si>
+    <t>Claim information and status should remain consistent across modules.</t>
+  </si>
+  <si>
+    <t>Verify Claim Approval Workflow Visibility</t>
+  </si>
+  <si>
+    <t>Status changes should be reflected accurately throughout workflow.</t>
+  </si>
+  <si>
+    <t>1. Submit claim. 
+2. Track claim through process.</t>
+  </si>
+  <si>
+    <t>TC275</t>
+  </si>
+  <si>
+    <t>TC276</t>
+  </si>
+  <si>
+    <t>TC277</t>
+  </si>
+  <si>
+    <t>TC278</t>
+  </si>
+  <si>
+    <t>TC279</t>
+  </si>
+  <si>
+    <t>TC280</t>
+  </si>
+  <si>
+    <t>TC281</t>
+  </si>
+  <si>
+    <t>TC282</t>
+  </si>
+  <si>
+    <t>TC283</t>
   </si>
 </sst>
 </file>
@@ -3787,7 +3892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G275"/>
+  <dimension ref="A1:G284"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -10125,6 +10230,213 @@
         <v>36</v>
       </c>
     </row>
+    <row r="276" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A276" s="1" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C276" s="2" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D276" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E276" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="F276" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G276" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A277" s="1" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C277" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D277" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="E277" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="F277" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G277" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A278" s="1" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C278" s="2" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D278" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="E278" s="2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="F278" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G278" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A279" s="1" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C279" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D279" s="2" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E279" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="F279" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G279" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A280" s="1" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C280" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D280" s="2" t="s">
+        <v>1067</v>
+      </c>
+      <c r="E280" s="2" t="s">
+        <v>1029</v>
+      </c>
+      <c r="F280" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G280" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A281" s="1" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C281" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D281" s="2" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E281" s="2" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F281" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G281" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A282" s="1" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C282" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D282" s="2" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E282" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F282" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G282" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A283" s="1" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C283" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D283" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E283" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="F283" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G283" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="284" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A284" s="1" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C284" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="D284" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="E284" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F284" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G284" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS038 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1988" uniqueCount="1089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2044" uniqueCount="1121">
   <si>
     <t>TC ID</t>
   </si>
@@ -3549,6 +3549,111 @@
   </si>
   <si>
     <t>TC283</t>
+  </si>
+  <si>
+    <t>Buzz</t>
+  </si>
+  <si>
+    <t>Verify Create Text Post</t>
+  </si>
+  <si>
+    <t>Post should be created successfully and appear in the newsfeed.</t>
+  </si>
+  <si>
+    <t>1. Navigate to Buzz Newsfeed. 
+2. Enter text in "What's on your mind?". 
+3. Click Post.</t>
+  </si>
+  <si>
+    <t>Verify Create Post with Photo</t>
+  </si>
+  <si>
+    <t>Post with image should be published successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Share Photos. 
+2. Upload an image. 
+3. Click Post.</t>
+  </si>
+  <si>
+    <t>Verify Create Post with Video</t>
+  </si>
+  <si>
+    <t>Post with video should be published successfully.</t>
+  </si>
+  <si>
+    <t>1. Click Share Video. 
+2. Upload a video. 
+3. Click Post.</t>
+  </si>
+  <si>
+    <t>Verify Empty Post Validation</t>
+  </si>
+  <si>
+    <t>1. Leave post content empty. 
+2. Click Post.</t>
+  </si>
+  <si>
+    <t>Verify Post Display After Creation</t>
+  </si>
+  <si>
+    <t>1. Create a new post.</t>
+  </si>
+  <si>
+    <t>Newly created post should appear at the top of the newsfeed.</t>
+  </si>
+  <si>
+    <t>Verify Post Timestamp Display</t>
+  </si>
+  <si>
+    <t>1. Create a post.</t>
+  </si>
+  <si>
+    <t>Correct date and time should be displayed with the post.</t>
+  </si>
+  <si>
+    <t>Verify Share Post Functionality</t>
+  </si>
+  <si>
+    <t>Post should be shared successfully.</t>
+  </si>
+  <si>
+    <t>1. Select an existing post. 
+2. Click Share icon.</t>
+  </si>
+  <si>
+    <t>Verify Post Visibility to Users</t>
+  </si>
+  <si>
+    <t>Post should be visible to authorized users.</t>
+  </si>
+  <si>
+    <t>1. Create a post. 
+2. Login as another user.</t>
+  </si>
+  <si>
+    <t>TC284</t>
+  </si>
+  <si>
+    <t>TC285</t>
+  </si>
+  <si>
+    <t>TC286</t>
+  </si>
+  <si>
+    <t>TC287</t>
+  </si>
+  <si>
+    <t>TC288</t>
+  </si>
+  <si>
+    <t>TC289</t>
+  </si>
+  <si>
+    <t>TC290</t>
+  </si>
+  <si>
+    <t>TC291</t>
   </si>
 </sst>
 </file>
@@ -3892,7 +3997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G284"/>
+  <dimension ref="A1:G292"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -10437,6 +10542,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="285" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A285" s="1" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C285" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D285" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E285" s="2" t="s">
+        <v>1091</v>
+      </c>
+      <c r="F285" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G285" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A286" s="1" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C286" s="2" t="s">
+        <v>1093</v>
+      </c>
+      <c r="D286" s="2" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E286" s="2" t="s">
+        <v>1094</v>
+      </c>
+      <c r="F286" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G286" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A287" s="1" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C287" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="D287" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E287" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F287" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G287" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A288" s="1" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C288" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D288" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E288" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F288" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G288" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A289" s="1" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C289" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="D289" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E289" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="F289" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G289" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A290" s="1" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C290" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D290" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F290" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G290" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A291" s="1" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C291" s="2" t="s">
+        <v>1107</v>
+      </c>
+      <c r="D291" s="2" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E291" s="2" t="s">
+        <v>1108</v>
+      </c>
+      <c r="F291" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G291" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A292" s="1" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C292" s="2" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D292" s="2" t="s">
+        <v>1112</v>
+      </c>
+      <c r="E292" s="2" t="s">
+        <v>1111</v>
+      </c>
+      <c r="F292" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G292" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS039 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2044" uniqueCount="1121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="1155">
   <si>
     <t>TC ID</t>
   </si>
@@ -3654,6 +3654,113 @@
   </si>
   <si>
     <t>TC291</t>
+  </si>
+  <si>
+    <t>Verify Like Post Functionality</t>
+  </si>
+  <si>
+    <t>Like count should increase by one.</t>
+  </si>
+  <si>
+    <t>1. Open a post. 
+2. Click Like icon.</t>
+  </si>
+  <si>
+    <t>Verify Unlike Post Functionality</t>
+  </si>
+  <si>
+    <t>Like should be removed and count updated.</t>
+  </si>
+  <si>
+    <t>1. Like a post. 
+2. Click Like icon again.</t>
+  </si>
+  <si>
+    <t>Verify Add Comment Functionality</t>
+  </si>
+  <si>
+    <t>Comment should be added successfully.</t>
+  </si>
+  <si>
+    <t>1. Open a post. 
+2. Add a comment. 
+3. Submit.</t>
+  </si>
+  <si>
+    <t>Verify Comment Count Update</t>
+  </si>
+  <si>
+    <t>1. Add a comment to a post.</t>
+  </si>
+  <si>
+    <t>Comment count should increase accordingly.</t>
+  </si>
+  <si>
+    <t>1. Click Share icon on a post.</t>
+  </si>
+  <si>
+    <t>Verify Share Count Update</t>
+  </si>
+  <si>
+    <t>1. Share a post.</t>
+  </si>
+  <si>
+    <t>Share count should increase correctly.</t>
+  </si>
+  <si>
+    <t>Verify Multiple Likes Handling</t>
+  </si>
+  <si>
+    <t>1. Like a post from different users.</t>
+  </si>
+  <si>
+    <t>Total likes count should update correctly.</t>
+  </si>
+  <si>
+    <t>Verify Interaction Icons Availability</t>
+  </si>
+  <si>
+    <t>1. Open any post.</t>
+  </si>
+  <si>
+    <t>Like, Comment, and Share icons should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Interaction Persistence After Refresh</t>
+  </si>
+  <si>
+    <t>Changes should remain saved and visible.</t>
+  </si>
+  <si>
+    <t>1. Like or comment on a post. 
+2. Refresh page.</t>
+  </si>
+  <si>
+    <t>TC292</t>
+  </si>
+  <si>
+    <t>TC293</t>
+  </si>
+  <si>
+    <t>TC294</t>
+  </si>
+  <si>
+    <t>TC295</t>
+  </si>
+  <si>
+    <t>TC296</t>
+  </si>
+  <si>
+    <t>TC297</t>
+  </si>
+  <si>
+    <t>TC298</t>
+  </si>
+  <si>
+    <t>TC299</t>
+  </si>
+  <si>
+    <t>TC300</t>
   </si>
 </sst>
 </file>
@@ -3997,7 +4104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G292"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -10726,6 +10833,213 @@
         <v>36</v>
       </c>
     </row>
+    <row r="293" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A293" s="1" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C293" s="2" t="s">
+        <v>1121</v>
+      </c>
+      <c r="D293" s="2" t="s">
+        <v>1123</v>
+      </c>
+      <c r="E293" s="2" t="s">
+        <v>1122</v>
+      </c>
+      <c r="F293" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G293" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A294" s="1" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C294" s="2" t="s">
+        <v>1124</v>
+      </c>
+      <c r="D294" s="2" t="s">
+        <v>1126</v>
+      </c>
+      <c r="E294" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="F294" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G294" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A295" s="1" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C295" s="2" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D295" s="2" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E295" s="2" t="s">
+        <v>1128</v>
+      </c>
+      <c r="F295" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G295" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A296" s="1" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C296" s="2" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D296" s="2" t="s">
+        <v>1131</v>
+      </c>
+      <c r="E296" s="2" t="s">
+        <v>1132</v>
+      </c>
+      <c r="F296" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G296" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A297" s="1" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C297" s="2" t="s">
+        <v>1107</v>
+      </c>
+      <c r="D297" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E297" s="2" t="s">
+        <v>1108</v>
+      </c>
+      <c r="F297" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G297" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A298" s="1" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C298" s="2" t="s">
+        <v>1134</v>
+      </c>
+      <c r="D298" s="2" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E298" s="2" t="s">
+        <v>1136</v>
+      </c>
+      <c r="F298" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G298" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A299" s="1" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C299" s="2" t="s">
+        <v>1137</v>
+      </c>
+      <c r="D299" s="2" t="s">
+        <v>1138</v>
+      </c>
+      <c r="E299" s="2" t="s">
+        <v>1139</v>
+      </c>
+      <c r="F299" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G299" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A300" s="1" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C300" s="2" t="s">
+        <v>1140</v>
+      </c>
+      <c r="D300" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E300" s="2" t="s">
+        <v>1142</v>
+      </c>
+      <c r="F300" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G300" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A301" s="1" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C301" s="2" t="s">
+        <v>1143</v>
+      </c>
+      <c r="D301" s="2" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E301" s="2" t="s">
+        <v>1144</v>
+      </c>
+      <c r="F301" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G301" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS040 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="1155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="1193">
   <si>
     <t>TC ID</t>
   </si>
@@ -3761,6 +3761,120 @@
   </si>
   <si>
     <t>TC300</t>
+  </si>
+  <si>
+    <t>Verify Most Recent Posts Display</t>
+  </si>
+  <si>
+    <t>1. Click Most Recent Posts.</t>
+  </si>
+  <si>
+    <t>Latest posts should be displayed in descending order.</t>
+  </si>
+  <si>
+    <t>Verify Most Liked Posts Display</t>
+  </si>
+  <si>
+    <t>1. Click Most Liked Posts.</t>
+  </si>
+  <si>
+    <t>Posts should be sorted by highest likes.</t>
+  </si>
+  <si>
+    <t>Verify Most Commented Posts Display</t>
+  </si>
+  <si>
+    <t>1. Click Most Commented Posts.</t>
+  </si>
+  <si>
+    <t>Posts should be sorted by highest comments.</t>
+  </si>
+  <si>
+    <t>Verify Newsfeed Content Loading</t>
+  </si>
+  <si>
+    <t>1. Open Buzz module.</t>
+  </si>
+  <si>
+    <t>Posts should load successfully in the newsfeed.</t>
+  </si>
+  <si>
+    <t>Verify User Information Display in Posts</t>
+  </si>
+  <si>
+    <t>Username, profile image, and timestamp should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Post Content Display</t>
+  </si>
+  <si>
+    <t>1. Open a post containing text, image, or video.</t>
+  </si>
+  <si>
+    <t>Content should display correctly without formatting issues.</t>
+  </si>
+  <si>
+    <t>Verify Newsfeed Refresh Functionality</t>
+  </si>
+  <si>
+    <t>1. Refresh Buzz page.</t>
+  </si>
+  <si>
+    <t>Latest feed data should load correctly.</t>
+  </si>
+  <si>
+    <t>Verify Post Menu Options</t>
+  </si>
+  <si>
+    <t>1. Click three-dot menu on a post.</t>
+  </si>
+  <si>
+    <t>Available management options should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Upcoming Anniversaries Display</t>
+  </si>
+  <si>
+    <t>Upcoming anniversaries section should display employee details correctly.</t>
+  </si>
+  <si>
+    <t>Verify Feed Consistency Across Filters</t>
+  </si>
+  <si>
+    <t>1. Switch between Recent, Liked, and Commented tabs.</t>
+  </si>
+  <si>
+    <t>Corresponding posts should load correctly without errors.</t>
+  </si>
+  <si>
+    <t>TC301</t>
+  </si>
+  <si>
+    <t>TC302</t>
+  </si>
+  <si>
+    <t>TC303</t>
+  </si>
+  <si>
+    <t>TC304</t>
+  </si>
+  <si>
+    <t>TC305</t>
+  </si>
+  <si>
+    <t>TC306</t>
+  </si>
+  <si>
+    <t>TC307</t>
+  </si>
+  <si>
+    <t>TC308</t>
+  </si>
+  <si>
+    <t>TC309</t>
+  </si>
+  <si>
+    <t>TC310</t>
   </si>
 </sst>
 </file>
@@ -4104,7 +4218,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G301"/>
+  <dimension ref="A1:G311"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -11040,6 +11154,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="302" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A302" s="1" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C302" s="2" t="s">
+        <v>1155</v>
+      </c>
+      <c r="D302" s="2" t="s">
+        <v>1156</v>
+      </c>
+      <c r="E302" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="F302" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G302" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A303" s="1" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C303" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D303" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E303" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="F303" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G303" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A304" s="1" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C304" s="2" t="s">
+        <v>1161</v>
+      </c>
+      <c r="D304" s="2" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E304" s="2" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F304" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G304" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A305" s="1" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C305" s="2" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D305" s="2" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E305" s="2" t="s">
+        <v>1166</v>
+      </c>
+      <c r="F305" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G305" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A306" s="1" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C306" s="2" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D306" s="2" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E306" s="2" t="s">
+        <v>1168</v>
+      </c>
+      <c r="F306" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G306" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A307" s="1" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C307" s="2" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D307" s="2" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E307" s="2" t="s">
+        <v>1171</v>
+      </c>
+      <c r="F307" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G307" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A308" s="1" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C308" s="2" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D308" s="2" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E308" s="2" t="s">
+        <v>1174</v>
+      </c>
+      <c r="F308" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G308" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A309" s="1" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C309" s="2" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D309" s="2" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E309" s="2" t="s">
+        <v>1177</v>
+      </c>
+      <c r="F309" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G309" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A310" s="1" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C310" s="2" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D310" s="2" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E310" s="2" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F310" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G310" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A311" s="1" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C311" s="2" t="s">
+        <v>1180</v>
+      </c>
+      <c r="D311" s="2" t="s">
+        <v>1181</v>
+      </c>
+      <c r="E311" s="2" t="s">
+        <v>1182</v>
+      </c>
+      <c r="F311" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G311" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS041 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2177" uniqueCount="1193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2235" uniqueCount="1225">
   <si>
     <t>TC ID</t>
   </si>
@@ -3875,6 +3875,108 @@
   </si>
   <si>
     <t>TC310</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Verify Login with Valid Credentials</t>
+  </si>
+  <si>
+    <t>User should be authenticated successfully.</t>
+  </si>
+  <si>
+    <t>1. Enter valid username and password. 
+2. Click Login.</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid Password</t>
+  </si>
+  <si>
+    <t>Login should fail with an error message.</t>
+  </si>
+  <si>
+    <t>1. Enter valid username and invalid password. 
+2. Click Login.</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid Username</t>
+  </si>
+  <si>
+    <t>Authentication should be denied.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid username and valid password. 
+2. Click Login.</t>
+  </si>
+  <si>
+    <t>Verify Empty Login Fields Validation</t>
+  </si>
+  <si>
+    <t>1. Leave username and password blank. 
+2. Click Login.</t>
+  </si>
+  <si>
+    <t>Verify Password Masking</t>
+  </si>
+  <si>
+    <t>1. Enter password in login form.</t>
+  </si>
+  <si>
+    <t>Password characters should be masked.</t>
+  </si>
+  <si>
+    <t>Verify Account Lock After Multiple Failed Attempts</t>
+  </si>
+  <si>
+    <t>1. Enter incorrect password multiple times.</t>
+  </si>
+  <si>
+    <t>Account should be temporarily locked or restricted.</t>
+  </si>
+  <si>
+    <t>Verify Logout Functionality</t>
+  </si>
+  <si>
+    <t>User session should end successfully.</t>
+  </si>
+  <si>
+    <t>1. Login successfully. 
+2. Click Logout.</t>
+  </si>
+  <si>
+    <t>Verify Access Restriction After Logout</t>
+  </si>
+  <si>
+    <t>User should be redirected to login page.</t>
+  </si>
+  <si>
+    <t>1. Logout from application. 
+2. Access protected URL directly.</t>
+  </si>
+  <si>
+    <t>TC311</t>
+  </si>
+  <si>
+    <t>TC312</t>
+  </si>
+  <si>
+    <t>TC313</t>
+  </si>
+  <si>
+    <t>TC314</t>
+  </si>
+  <si>
+    <t>TC315</t>
+  </si>
+  <si>
+    <t>TC316</t>
+  </si>
+  <si>
+    <t>TC317</t>
+  </si>
+  <si>
+    <t>TC318</t>
   </si>
 </sst>
 </file>
@@ -4218,7 +4320,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G311"/>
+  <dimension ref="A1:G320"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -11384,6 +11486,198 @@
         <v>36</v>
       </c>
     </row>
+    <row r="312" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A312" s="1" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C312" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D312" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E312" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="F312" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G312" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="313" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A313" s="1" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C313" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D313" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="E313" s="2" t="s">
+        <v>1198</v>
+      </c>
+      <c r="F313" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G313" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A314" s="1" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C314" s="2" t="s">
+        <v>1200</v>
+      </c>
+      <c r="D314" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E314" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="F314" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G314" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="315" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A315" s="1" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C315" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D315" s="2" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E315" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F315" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G315" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A316" s="1" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C316" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D316" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E316" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="F316" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G316" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A317" s="1" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C317" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="D317" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E317" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="F317" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G317" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="318" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A318" s="1" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C318" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="D318" s="2" t="s">
+        <v>1213</v>
+      </c>
+      <c r="E318" s="2" t="s">
+        <v>1212</v>
+      </c>
+      <c r="F318" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G318" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="319" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A319" s="1" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C319" s="2" t="s">
+        <v>1214</v>
+      </c>
+      <c r="D319" s="2" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E319" s="2" t="s">
+        <v>1215</v>
+      </c>
+      <c r="F319" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G319" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F320" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G320" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS042 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2235" uniqueCount="1225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2284" uniqueCount="1251">
   <si>
     <t>TC ID</t>
   </si>
@@ -3977,6 +3977,89 @@
   </si>
   <si>
     <t>TC318</t>
+  </si>
+  <si>
+    <t>Verify Admin Access to Restricted Modules</t>
+  </si>
+  <si>
+    <t>Access should be granted.</t>
+  </si>
+  <si>
+    <t>1. Login as Admin. 
+2. Open Admin module.</t>
+  </si>
+  <si>
+    <t>Verify Employee Restriction from Admin Module</t>
+  </si>
+  <si>
+    <t>1. Login as Employee. 
+2. Attempt to access Admin module.</t>
+  </si>
+  <si>
+    <t>Verify Role-Based Menu Visibility</t>
+  </si>
+  <si>
+    <t>1. Login with different user roles.</t>
+  </si>
+  <si>
+    <t>Only authorized menus should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Unauthorized URL Access Restriction</t>
+  </si>
+  <si>
+    <t>1. Login as Employee. 
+2. Access Admin URL directly.</t>
+  </si>
+  <si>
+    <t>Verify Permission-Based Actions</t>
+  </si>
+  <si>
+    <t>Unauthorized actions should be restricted.</t>
+  </si>
+  <si>
+    <t>1. Open module with limited permissions. 
+2. Attempt Add/Edit/Delete action.</t>
+  </si>
+  <si>
+    <t>Verify Authorized User Actions</t>
+  </si>
+  <si>
+    <t>Action should be completed successfully.</t>
+  </si>
+  <si>
+    <t>1. Login with proper permissions. 
+2. Perform Add/Edit/Delete operation.</t>
+  </si>
+  <si>
+    <t>Verify Access Control Across Modules</t>
+  </si>
+  <si>
+    <t>1. Navigate through various modules.</t>
+  </si>
+  <si>
+    <t>User should only access permitted modules.</t>
+  </si>
+  <si>
+    <t>TC319</t>
+  </si>
+  <si>
+    <t>TC320</t>
+  </si>
+  <si>
+    <t>TC321</t>
+  </si>
+  <si>
+    <t>TC322</t>
+  </si>
+  <si>
+    <t>TC323</t>
+  </si>
+  <si>
+    <t>TC324</t>
+  </si>
+  <si>
+    <t>TC325</t>
   </si>
 </sst>
 </file>
@@ -4320,7 +4403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G320"/>
+  <dimension ref="A1:G327"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -11670,11 +11753,172 @@
         <v>36</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A320" s="1" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C320" s="2" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D320" s="2" t="s">
+        <v>1227</v>
+      </c>
+      <c r="E320" s="2" t="s">
+        <v>1226</v>
+      </c>
       <c r="F320" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G320" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="321" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A321" s="1" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C321" s="2" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D321" s="2" t="s">
+        <v>1229</v>
+      </c>
+      <c r="E321" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="F321" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G321" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="322" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A322" s="1" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C322" s="2" t="s">
+        <v>1230</v>
+      </c>
+      <c r="D322" s="2" t="s">
+        <v>1231</v>
+      </c>
+      <c r="E322" s="2" t="s">
+        <v>1232</v>
+      </c>
+      <c r="F322" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G322" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A323" s="1" t="s">
+        <v>1247</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C323" s="2" t="s">
+        <v>1233</v>
+      </c>
+      <c r="D323" s="2" t="s">
+        <v>1234</v>
+      </c>
+      <c r="E323" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="F323" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G323" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="324" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A324" s="1" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C324" s="2" t="s">
+        <v>1235</v>
+      </c>
+      <c r="D324" s="2" t="s">
+        <v>1237</v>
+      </c>
+      <c r="E324" s="2" t="s">
+        <v>1236</v>
+      </c>
+      <c r="F324" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G324" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A325" s="1" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C325" s="2" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D325" s="2" t="s">
+        <v>1240</v>
+      </c>
+      <c r="E325" s="2" t="s">
+        <v>1239</v>
+      </c>
+      <c r="F325" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G325" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="326" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A326" s="1" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C326" s="2" t="s">
+        <v>1241</v>
+      </c>
+      <c r="D326" s="2" t="s">
+        <v>1242</v>
+      </c>
+      <c r="E326" s="2" t="s">
+        <v>1243</v>
+      </c>
+      <c r="F326" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G326" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="327" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F327" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G327" s="3" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
TS043 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2284" uniqueCount="1251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2331" uniqueCount="1278">
   <si>
     <t>TC ID</t>
   </si>
@@ -4060,6 +4060,90 @@
   </si>
   <si>
     <t>TC325</t>
+  </si>
+  <si>
+    <t>Verify Session Creation After Login</t>
+  </si>
+  <si>
+    <t>1. Login successfully.</t>
+  </si>
+  <si>
+    <t>New user session should be created.</t>
+  </si>
+  <si>
+    <t>Verify Session Expiry After Inactivity</t>
+  </si>
+  <si>
+    <t>Session should expire automatically.</t>
+  </si>
+  <si>
+    <t>1. Login. 
+2. Remain inactive for configured timeout period.</t>
+  </si>
+  <si>
+    <t>Verify Redirect After Session Expiry</t>
+  </si>
+  <si>
+    <t>1. Allow session to expire. 
+2. Perform any action.</t>
+  </si>
+  <si>
+    <t>Verify Browser Back Button After Logout</t>
+  </si>
+  <si>
+    <t>Protected pages should not be accessible.</t>
+  </si>
+  <si>
+    <t>1. Logout. 
+2. Click browser Back button.</t>
+  </si>
+  <si>
+    <t>Verify Multiple Session Handling</t>
+  </si>
+  <si>
+    <t>1. Login from multiple browsers/devices.</t>
+  </si>
+  <si>
+    <t>Session management should work according to system policy.</t>
+  </si>
+  <si>
+    <t>Verify Session Persistence During Activity</t>
+  </si>
+  <si>
+    <t>1. Continuously use application.</t>
+  </si>
+  <si>
+    <t>Session should remain active.</t>
+  </si>
+  <si>
+    <t>Verify Secure Logout Session Cleanup</t>
+  </si>
+  <si>
+    <t>1. Logout from application.</t>
+  </si>
+  <si>
+    <t>Session data should be cleared completely.</t>
+  </si>
+  <si>
+    <t>TC326</t>
+  </si>
+  <si>
+    <t>TC327</t>
+  </si>
+  <si>
+    <t>TC328</t>
+  </si>
+  <si>
+    <t>TC329</t>
+  </si>
+  <si>
+    <t>TC330</t>
+  </si>
+  <si>
+    <t>TC331</t>
+  </si>
+  <si>
+    <t>TC332</t>
   </si>
 </sst>
 </file>
@@ -4403,7 +4487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G327"/>
+  <dimension ref="A1:G335"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -11915,12 +11999,168 @@
       </c>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A327" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C327" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="D327" s="2" t="s">
+        <v>1252</v>
+      </c>
+      <c r="E327" s="2" t="s">
+        <v>1253</v>
+      </c>
       <c r="F327" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G327" s="3" t="s">
         <v>36</v>
       </c>
+    </row>
+    <row r="328" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A328" s="1" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C328" s="2" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D328" s="2" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E328" s="2" t="s">
+        <v>1255</v>
+      </c>
+      <c r="F328" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G328" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="329" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A329" s="1" t="s">
+        <v>1273</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C329" s="2" t="s">
+        <v>1257</v>
+      </c>
+      <c r="D329" s="2" t="s">
+        <v>1258</v>
+      </c>
+      <c r="E329" s="2" t="s">
+        <v>1215</v>
+      </c>
+      <c r="F329" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G329" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="330" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A330" s="1" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C330" s="2" t="s">
+        <v>1259</v>
+      </c>
+      <c r="D330" s="2" t="s">
+        <v>1261</v>
+      </c>
+      <c r="E330" s="2" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F330" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G330" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A331" s="1" t="s">
+        <v>1275</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C331" s="2" t="s">
+        <v>1262</v>
+      </c>
+      <c r="D331" s="2" t="s">
+        <v>1263</v>
+      </c>
+      <c r="E331" s="2" t="s">
+        <v>1264</v>
+      </c>
+      <c r="F331" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G331" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="332" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A332" s="1" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C332" s="2" t="s">
+        <v>1265</v>
+      </c>
+      <c r="D332" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="E332" s="2" t="s">
+        <v>1267</v>
+      </c>
+      <c r="F332" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G332" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="333" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A333" s="1" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C333" s="2" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D333" s="2" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E333" s="2" t="s">
+        <v>1270</v>
+      </c>
+      <c r="F333" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G333" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C335" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
TS044 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2331" uniqueCount="1278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="1312">
   <si>
     <t>TC ID</t>
   </si>
@@ -4144,6 +4144,110 @@
   </si>
   <si>
     <t>TC332</t>
+  </si>
+  <si>
+    <t>Verify SQL Injection Protection</t>
+  </si>
+  <si>
+    <t>Application should reject malicious input safely.</t>
+  </si>
+  <si>
+    <t>1. Enter SQL injection string in input field. 
+2. Submit form.</t>
+  </si>
+  <si>
+    <t>Verify XSS Protection</t>
+  </si>
+  <si>
+    <t>1. Enter JavaScript code in text field. 2. Submit form.</t>
+  </si>
+  <si>
+    <t>Script should not execute.</t>
+  </si>
+  <si>
+    <t>Verify Special Character Validation</t>
+  </si>
+  <si>
+    <t>1. Enter unsupported special characters.</t>
+  </si>
+  <si>
+    <t>Application should handle input securely.</t>
+  </si>
+  <si>
+    <t>Verify Input Length Validation</t>
+  </si>
+  <si>
+    <t>1. Enter data exceeding field limit.</t>
+  </si>
+  <si>
+    <t>Verify Required Field Validation</t>
+  </si>
+  <si>
+    <t>Validation error should appear.</t>
+  </si>
+  <si>
+    <t>1. Leave mandatory fields empty. 
+2. Submit form.</t>
+  </si>
+  <si>
+    <t>Verify Numeric Field Validation</t>
+  </si>
+  <si>
+    <t>1. Enter alphabets in numeric field.</t>
+  </si>
+  <si>
+    <t>System should reject invalid input.</t>
+  </si>
+  <si>
+    <t>Verify Email Format Validation</t>
+  </si>
+  <si>
+    <t>1. Enter invalid email format.</t>
+  </si>
+  <si>
+    <t>Verify File Upload Validation</t>
+  </si>
+  <si>
+    <t>1. Upload unsupported file type.</t>
+  </si>
+  <si>
+    <t>Upload should be rejected.</t>
+  </si>
+  <si>
+    <t>Verify Input Sanitization</t>
+  </si>
+  <si>
+    <t>1. Enter malicious or unexpected input.</t>
+  </si>
+  <si>
+    <t>Input should be sanitized and processed securely.</t>
+  </si>
+  <si>
+    <t>TC333</t>
+  </si>
+  <si>
+    <t>TC334</t>
+  </si>
+  <si>
+    <t>TC335</t>
+  </si>
+  <si>
+    <t>TC336</t>
+  </si>
+  <si>
+    <t>TC337</t>
+  </si>
+  <si>
+    <t>TC338</t>
+  </si>
+  <si>
+    <t>TC339</t>
+  </si>
+  <si>
+    <t>TC340</t>
+  </si>
+  <si>
+    <t>TC341</t>
   </si>
 </sst>
 </file>
@@ -4487,7 +4591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G335"/>
+  <dimension ref="A1:G342"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -12159,8 +12263,212 @@
         <v>36</v>
       </c>
     </row>
-    <row r="335" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C335" s="2"/>
+    <row r="334" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A334" s="1" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C334" s="2" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D334" s="2" t="s">
+        <v>1280</v>
+      </c>
+      <c r="E334" s="2" t="s">
+        <v>1279</v>
+      </c>
+      <c r="F334" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G334" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A335" s="1" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C335" s="2" t="s">
+        <v>1281</v>
+      </c>
+      <c r="D335" s="2" t="s">
+        <v>1282</v>
+      </c>
+      <c r="E335" s="2" t="s">
+        <v>1283</v>
+      </c>
+      <c r="F335" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G335" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="336" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A336" s="1" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C336" s="2" t="s">
+        <v>1284</v>
+      </c>
+      <c r="D336" s="2" t="s">
+        <v>1285</v>
+      </c>
+      <c r="E336" s="2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="F336" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G336" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="337" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A337" s="1" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C337" s="2" t="s">
+        <v>1287</v>
+      </c>
+      <c r="D337" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="E337" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F337" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G337" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="338" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A338" s="1" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C338" s="2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="D338" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="E338" s="2" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F338" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G338" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A339" s="1" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C339" s="2" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D339" s="2" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E339" s="2" t="s">
+        <v>1294</v>
+      </c>
+      <c r="F339" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G339" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="340" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A340" s="1" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C340" s="2" t="s">
+        <v>1295</v>
+      </c>
+      <c r="D340" s="2" t="s">
+        <v>1296</v>
+      </c>
+      <c r="E340" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="F340" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G340" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A341" s="1" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C341" s="2" t="s">
+        <v>1297</v>
+      </c>
+      <c r="D341" s="2" t="s">
+        <v>1298</v>
+      </c>
+      <c r="E341" s="2" t="s">
+        <v>1299</v>
+      </c>
+      <c r="F341" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G341" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="342" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A342" s="1" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C342" s="2" t="s">
+        <v>1300</v>
+      </c>
+      <c r="D342" s="2" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E342" s="2" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F342" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G342" s="3" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
TS045 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="1312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="1345">
   <si>
     <t>TC ID</t>
   </si>
@@ -4248,6 +4248,105 @@
   </si>
   <si>
     <t>TC341</t>
+  </si>
+  <si>
+    <t>UI &amp; Usability</t>
+  </si>
+  <si>
+    <t>Verify Page Layout Consistency</t>
+  </si>
+  <si>
+    <t>1. Navigate across different modules.</t>
+  </si>
+  <si>
+    <t>Layout should remain consistent throughout the application.</t>
+  </si>
+  <si>
+    <t>Verify Menu Visibility</t>
+  </si>
+  <si>
+    <t>1. Login and view navigation menu.</t>
+  </si>
+  <si>
+    <t>All authorized menu items should be displayed correctly.</t>
+  </si>
+  <si>
+    <t>Verify Button Alignment</t>
+  </si>
+  <si>
+    <t>1. Open different forms and pages.</t>
+  </si>
+  <si>
+    <t>Buttons should be properly aligned and visible.</t>
+  </si>
+  <si>
+    <t>Verify Form Field Alignment</t>
+  </si>
+  <si>
+    <t>1. Open data entry forms.</t>
+  </si>
+  <si>
+    <t>Fields and labels should be aligned correctly.</t>
+  </si>
+  <si>
+    <t>Verify Table Display Layout</t>
+  </si>
+  <si>
+    <t>1. Open pages containing data tables.</t>
+  </si>
+  <si>
+    <t>Table headers and data should display properly.</t>
+  </si>
+  <si>
+    <t>Verify Icons Display</t>
+  </si>
+  <si>
+    <t>1. Navigate through modules.</t>
+  </si>
+  <si>
+    <t>Icons should load and display correctly.</t>
+  </si>
+  <si>
+    <t>Verify Font Consistency</t>
+  </si>
+  <si>
+    <t>1. Review multiple pages.</t>
+  </si>
+  <si>
+    <t>Fonts, sizes, and styles should be consistent.</t>
+  </si>
+  <si>
+    <t>Verify Color Theme Consistency</t>
+  </si>
+  <si>
+    <t>1. Navigate through application pages.</t>
+  </si>
+  <si>
+    <t>Theme colors should remain consistent.</t>
+  </si>
+  <si>
+    <t>TC342</t>
+  </si>
+  <si>
+    <t>TC343</t>
+  </si>
+  <si>
+    <t>TC344</t>
+  </si>
+  <si>
+    <t>TC345</t>
+  </si>
+  <si>
+    <t>TC346</t>
+  </si>
+  <si>
+    <t>TC347</t>
+  </si>
+  <si>
+    <t>TC348</t>
+  </si>
+  <si>
+    <t>TC349</t>
   </si>
 </sst>
 </file>
@@ -4591,11 +4690,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G342"/>
+  <dimension ref="A1:G350"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -12470,6 +12569,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="343" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A343" s="1" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C343" s="2" t="s">
+        <v>1313</v>
+      </c>
+      <c r="D343" s="2" t="s">
+        <v>1314</v>
+      </c>
+      <c r="E343" s="2" t="s">
+        <v>1315</v>
+      </c>
+      <c r="F343" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G343" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="344" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A344" s="1" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C344" s="2" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D344" s="2" t="s">
+        <v>1317</v>
+      </c>
+      <c r="E344" s="2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="F344" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G344" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="345" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A345" s="1" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C345" s="2" t="s">
+        <v>1319</v>
+      </c>
+      <c r="D345" s="2" t="s">
+        <v>1320</v>
+      </c>
+      <c r="E345" s="2" t="s">
+        <v>1321</v>
+      </c>
+      <c r="F345" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G345" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A346" s="1" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C346" s="2" t="s">
+        <v>1322</v>
+      </c>
+      <c r="D346" s="2" t="s">
+        <v>1323</v>
+      </c>
+      <c r="E346" s="2" t="s">
+        <v>1324</v>
+      </c>
+      <c r="F346" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G346" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="347" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A347" s="1" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C347" s="2" t="s">
+        <v>1325</v>
+      </c>
+      <c r="D347" s="2" t="s">
+        <v>1326</v>
+      </c>
+      <c r="E347" s="2" t="s">
+        <v>1327</v>
+      </c>
+      <c r="F347" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G347" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="348" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A348" s="1" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C348" s="2" t="s">
+        <v>1328</v>
+      </c>
+      <c r="D348" s="2" t="s">
+        <v>1329</v>
+      </c>
+      <c r="E348" s="2" t="s">
+        <v>1330</v>
+      </c>
+      <c r="F348" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G348" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A349" s="1" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C349" s="2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="D349" s="2" t="s">
+        <v>1332</v>
+      </c>
+      <c r="E349" s="2" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F349" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G349" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="350" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A350" s="1" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B350" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C350" s="2" t="s">
+        <v>1334</v>
+      </c>
+      <c r="D350" s="2" t="s">
+        <v>1335</v>
+      </c>
+      <c r="E350" s="2" t="s">
+        <v>1336</v>
+      </c>
+      <c r="F350" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G350" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS046 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="1345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="1373">
   <si>
     <t>TC ID</t>
   </si>
@@ -4347,6 +4347,90 @@
   </si>
   <si>
     <t>TC349</t>
+  </si>
+  <si>
+    <t>Verify Application on Desktop Resolution</t>
+  </si>
+  <si>
+    <t>1. Open application on desktop browser.</t>
+  </si>
+  <si>
+    <t>UI should display correctly without overlap.</t>
+  </si>
+  <si>
+    <t>Verify Application on Tablet Resolution</t>
+  </si>
+  <si>
+    <t>1. Resize browser to tablet size.</t>
+  </si>
+  <si>
+    <t>Layout should adjust properly.</t>
+  </si>
+  <si>
+    <t>Verify Application on Mobile Resolution</t>
+  </si>
+  <si>
+    <t>1. Open application on mobile device.</t>
+  </si>
+  <si>
+    <t>UI should remain usable and responsive.</t>
+  </si>
+  <si>
+    <t>Verify Responsive Navigation Menu</t>
+  </si>
+  <si>
+    <t>1. Access application on smaller screens.</t>
+  </si>
+  <si>
+    <t>Navigation should adapt correctly.</t>
+  </si>
+  <si>
+    <t>Verify Form Responsiveness</t>
+  </si>
+  <si>
+    <t>1. Open forms on different screen sizes.</t>
+  </si>
+  <si>
+    <t>Fields should resize and remain accessible.</t>
+  </si>
+  <si>
+    <t>Verify Table Responsiveness</t>
+  </si>
+  <si>
+    <t>1. Open data tables on small screens.</t>
+  </si>
+  <si>
+    <t>Tables should remain readable or scroll properly.</t>
+  </si>
+  <si>
+    <t>Verify Button Accessibility on Small Screens</t>
+  </si>
+  <si>
+    <t>1. Access pages using mobile view.</t>
+  </si>
+  <si>
+    <t>Buttons should remain clickable and visible.</t>
+  </si>
+  <si>
+    <t>TC350</t>
+  </si>
+  <si>
+    <t>TC351</t>
+  </si>
+  <si>
+    <t>TC352</t>
+  </si>
+  <si>
+    <t>TC353</t>
+  </si>
+  <si>
+    <t>TC354</t>
+  </si>
+  <si>
+    <t>TC355</t>
+  </si>
+  <si>
+    <t>TC356</t>
   </si>
 </sst>
 </file>
@@ -4690,7 +4774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G350"/>
+  <dimension ref="A1:G357"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -12753,6 +12837,167 @@
         <v>36</v>
       </c>
     </row>
+    <row r="351" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A351" s="1" t="s">
+        <v>1366</v>
+      </c>
+      <c r="B351" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C351" s="2" t="s">
+        <v>1345</v>
+      </c>
+      <c r="D351" s="2" t="s">
+        <v>1346</v>
+      </c>
+      <c r="E351" s="2" t="s">
+        <v>1347</v>
+      </c>
+      <c r="F351" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G351" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="352" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A352" s="1" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C352" s="2" t="s">
+        <v>1348</v>
+      </c>
+      <c r="D352" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="E352" s="2" t="s">
+        <v>1350</v>
+      </c>
+      <c r="F352" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G352" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="353" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A353" s="1" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C353" s="2" t="s">
+        <v>1351</v>
+      </c>
+      <c r="D353" s="2" t="s">
+        <v>1352</v>
+      </c>
+      <c r="E353" s="2" t="s">
+        <v>1353</v>
+      </c>
+      <c r="F353" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G353" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="354" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A354" s="1" t="s">
+        <v>1369</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C354" s="2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="D354" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="E354" s="2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="F354" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G354" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="355" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A355" s="1" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C355" s="2" t="s">
+        <v>1357</v>
+      </c>
+      <c r="D355" s="2" t="s">
+        <v>1358</v>
+      </c>
+      <c r="E355" s="2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="F355" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G355" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="356" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A356" s="1" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C356" s="2" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D356" s="2" t="s">
+        <v>1361</v>
+      </c>
+      <c r="E356" s="2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="F356" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G356" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="357" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A357" s="1" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C357" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="D357" s="2" t="s">
+        <v>1364</v>
+      </c>
+      <c r="E357" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="F357" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G357" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS047 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="1373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="1405">
   <si>
     <t>TC ID</t>
   </si>
@@ -4431,6 +4431,105 @@
   </si>
   <si>
     <t>TC356</t>
+  </si>
+  <si>
+    <t>Verify Module Navigation</t>
+  </si>
+  <si>
+    <t>1. Click different modules from menu.</t>
+  </si>
+  <si>
+    <t>User should navigate successfully to selected module.</t>
+  </si>
+  <si>
+    <t>Verify Submenu Navigation</t>
+  </si>
+  <si>
+    <t>Correct page should open.</t>
+  </si>
+  <si>
+    <t>1. Open module dropdowns. 
+2. Select submenu item.</t>
+  </si>
+  <si>
+    <t>Verify Dashboard Navigation</t>
+  </si>
+  <si>
+    <t>1. Navigate back to dashboard from any module.</t>
+  </si>
+  <si>
+    <t>Dashboard should load successfully.</t>
+  </si>
+  <si>
+    <t>Verify Breadcrumb Navigation</t>
+  </si>
+  <si>
+    <t>1. Open multiple pages.</t>
+  </si>
+  <si>
+    <t>Breadcrumb path should display correctly.</t>
+  </si>
+  <si>
+    <t>Verify Browser Back Button Functionality</t>
+  </si>
+  <si>
+    <t>Previous page should load correctly.</t>
+  </si>
+  <si>
+    <t>1. Navigate between pages. 
+2. Use browser Back button.</t>
+  </si>
+  <si>
+    <t>Verify Browser Forward Button Functionality</t>
+  </si>
+  <si>
+    <t>Next page should open correctly.</t>
+  </si>
+  <si>
+    <t>1. Navigate using Back button. 
+2. Click Forward.</t>
+  </si>
+  <si>
+    <t>Verify User Profile Navigation</t>
+  </si>
+  <si>
+    <t>1. Click user profile menu.</t>
+  </si>
+  <si>
+    <t>Profile-related options should be accessible.</t>
+  </si>
+  <si>
+    <t>Verify Help Icon Navigation</t>
+  </si>
+  <si>
+    <t>1. Click Help icon.</t>
+  </si>
+  <si>
+    <t>Help page or documentation should open.</t>
+  </si>
+  <si>
+    <t>TC357</t>
+  </si>
+  <si>
+    <t>TC358</t>
+  </si>
+  <si>
+    <t>TC359</t>
+  </si>
+  <si>
+    <t>TC360</t>
+  </si>
+  <si>
+    <t>TC361</t>
+  </si>
+  <si>
+    <t>TC362</t>
+  </si>
+  <si>
+    <t>TC363</t>
+  </si>
+  <si>
+    <t>TC364</t>
   </si>
 </sst>
 </file>
@@ -4774,7 +4873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G357"/>
+  <dimension ref="A1:G365"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -12998,6 +13097,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="358" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A358" s="1" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C358" s="2" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D358" s="2" t="s">
+        <v>1374</v>
+      </c>
+      <c r="E358" s="2" t="s">
+        <v>1375</v>
+      </c>
+      <c r="F358" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G358" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="359" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A359" s="1" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B359" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C359" s="2" t="s">
+        <v>1376</v>
+      </c>
+      <c r="D359" s="2" t="s">
+        <v>1378</v>
+      </c>
+      <c r="E359" s="2" t="s">
+        <v>1377</v>
+      </c>
+      <c r="F359" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G359" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="360" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A360" s="1" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C360" s="2" t="s">
+        <v>1379</v>
+      </c>
+      <c r="D360" s="2" t="s">
+        <v>1380</v>
+      </c>
+      <c r="E360" s="2" t="s">
+        <v>1381</v>
+      </c>
+      <c r="F360" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G360" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="361" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A361" s="1" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B361" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C361" s="2" t="s">
+        <v>1382</v>
+      </c>
+      <c r="D361" s="2" t="s">
+        <v>1383</v>
+      </c>
+      <c r="E361" s="2" t="s">
+        <v>1384</v>
+      </c>
+      <c r="F361" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G361" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="362" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A362" s="1" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B362" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>1385</v>
+      </c>
+      <c r="D362" s="2" t="s">
+        <v>1387</v>
+      </c>
+      <c r="E362" s="2" t="s">
+        <v>1386</v>
+      </c>
+      <c r="F362" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G362" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="363" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A363" s="1" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B363" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C363" s="2" t="s">
+        <v>1388</v>
+      </c>
+      <c r="D363" s="2" t="s">
+        <v>1390</v>
+      </c>
+      <c r="E363" s="2" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F363" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G363" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="364" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A364" s="1" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B364" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C364" s="2" t="s">
+        <v>1391</v>
+      </c>
+      <c r="D364" s="2" t="s">
+        <v>1392</v>
+      </c>
+      <c r="E364" s="2" t="s">
+        <v>1393</v>
+      </c>
+      <c r="F364" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G364" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="365" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A365" s="1" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C365" s="2" t="s">
+        <v>1394</v>
+      </c>
+      <c r="D365" s="2" t="s">
+        <v>1395</v>
+      </c>
+      <c r="E365" s="2" t="s">
+        <v>1396</v>
+      </c>
+      <c r="F365" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G365" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS048 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="1405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2611" uniqueCount="1436">
   <si>
     <t>TC ID</t>
   </si>
@@ -4530,6 +4530,100 @@
   </si>
   <si>
     <t>TC364</t>
+  </si>
+  <si>
+    <t>Verify Success Message on Record Creation</t>
+  </si>
+  <si>
+    <t>1. Create a new record.</t>
+  </si>
+  <si>
+    <t>Success message should be displayed.</t>
+  </si>
+  <si>
+    <t>Verify Success Message on Record Update</t>
+  </si>
+  <si>
+    <t>1. Edit and save a record.</t>
+  </si>
+  <si>
+    <t>Update success message should appear.</t>
+  </si>
+  <si>
+    <t>Verify Success Message on Record Deletion</t>
+  </si>
+  <si>
+    <t>1. Delete a record.</t>
+  </si>
+  <si>
+    <t>Deletion success message should appear.</t>
+  </si>
+  <si>
+    <t>Verify Error Message for Invalid Input</t>
+  </si>
+  <si>
+    <t>Appropriate error message should be displayed.</t>
+  </si>
+  <si>
+    <t>1. Enter invalid data. 
+2. Submit form.</t>
+  </si>
+  <si>
+    <t>Verify Required Field Validation Message</t>
+  </si>
+  <si>
+    <t>Validation message should appear.</t>
+  </si>
+  <si>
+    <t>Verify Error Message Clarity</t>
+  </si>
+  <si>
+    <t>1. Trigger an application error.</t>
+  </si>
+  <si>
+    <t>Message should clearly explain the issue.</t>
+  </si>
+  <si>
+    <t>Verify Message Visibility</t>
+  </si>
+  <si>
+    <t>1. Perform successful and failed actions.</t>
+  </si>
+  <si>
+    <t>Messages should be clearly visible to users.</t>
+  </si>
+  <si>
+    <t>Verify Message Auto-Dismiss Behavior</t>
+  </si>
+  <si>
+    <t>1. Trigger a success notification.</t>
+  </si>
+  <si>
+    <t>Message should disappear after configured duration (if applicable).</t>
+  </si>
+  <si>
+    <t>TC365</t>
+  </si>
+  <si>
+    <t>TC366</t>
+  </si>
+  <si>
+    <t>TC367</t>
+  </si>
+  <si>
+    <t>TC368</t>
+  </si>
+  <si>
+    <t>TC369</t>
+  </si>
+  <si>
+    <t>TC370</t>
+  </si>
+  <si>
+    <t>TC371</t>
+  </si>
+  <si>
+    <t>TC372</t>
   </si>
 </sst>
 </file>
@@ -4873,7 +4967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G365"/>
+  <dimension ref="A1:G373"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -13281,6 +13375,190 @@
         <v>36</v>
       </c>
     </row>
+    <row r="366" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A366" s="1" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C366" s="2" t="s">
+        <v>1405</v>
+      </c>
+      <c r="D366" s="2" t="s">
+        <v>1406</v>
+      </c>
+      <c r="E366" s="2" t="s">
+        <v>1407</v>
+      </c>
+      <c r="F366" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G366" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="367" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A367" s="1" t="s">
+        <v>1429</v>
+      </c>
+      <c r="B367" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C367" s="2" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D367" s="2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="E367" s="2" t="s">
+        <v>1410</v>
+      </c>
+      <c r="F367" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G367" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A368" s="1" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C368" s="2" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D368" s="2" t="s">
+        <v>1412</v>
+      </c>
+      <c r="E368" s="2" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F368" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G368" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="369" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A369" s="1" t="s">
+        <v>1431</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C369" s="2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D369" s="2" t="s">
+        <v>1416</v>
+      </c>
+      <c r="E369" s="2" t="s">
+        <v>1415</v>
+      </c>
+      <c r="F369" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G369" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="370" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A370" s="1" t="s">
+        <v>1432</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C370" s="2" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D370" s="2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="E370" s="2" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F370" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G370" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="371" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A371" s="1" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B371" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C371" s="2" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D371" s="2" t="s">
+        <v>1420</v>
+      </c>
+      <c r="E371" s="2" t="s">
+        <v>1421</v>
+      </c>
+      <c r="F371" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G371" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="372" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A372" s="1" t="s">
+        <v>1434</v>
+      </c>
+      <c r="B372" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C372" s="2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D372" s="2" t="s">
+        <v>1423</v>
+      </c>
+      <c r="E372" s="2" t="s">
+        <v>1424</v>
+      </c>
+      <c r="F372" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G372" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="373" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A373" s="1" t="s">
+        <v>1435</v>
+      </c>
+      <c r="B373" s="1" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C373" s="2" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D373" s="2" t="s">
+        <v>1426</v>
+      </c>
+      <c r="E373" s="2" t="s">
+        <v>1427</v>
+      </c>
+      <c r="F373" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G373" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TS049 Test Case Added
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2611" uniqueCount="1436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1474">
   <si>
     <t>TC ID</t>
   </si>
@@ -4624,6 +4624,198 @@
   </si>
   <si>
     <t>TC372</t>
+  </si>
+  <si>
+    <t>End-to-End</t>
+  </si>
+  <si>
+    <t>Verify Leave Request Submission</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leave request should be submitted successfully with status as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pending Approval</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Login as Employee. 
+2. Navigate to Leave Module. 
+3. Apply for leave with valid details. 4. Submit request.</t>
+  </si>
+  <si>
+    <t>Verify Leave Request Appears in Manager Queue</t>
+  </si>
+  <si>
+    <t>Submitted leave request should be visible in approval list.</t>
+  </si>
+  <si>
+    <t>1. Login as Manager. 
+2. Open Leave Approval section.</t>
+  </si>
+  <si>
+    <t>Verify Leave Approval Workflow</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leave status should change to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Approved</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Select pending leave request. 
+2. Click Approve.</t>
+  </si>
+  <si>
+    <t>Verify Leave Rejection Workflow</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leave status should change to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rejected</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Select pending leave request. 
+2. Click Reject.</t>
+  </si>
+  <si>
+    <t>Verify Employee Can View Leave Status</t>
+  </si>
+  <si>
+    <t>1. Login as Employee. 
+2. Open My Leave Requests.</t>
+  </si>
+  <si>
+    <t>Verify Leave Balance Deduction After Approval</t>
+  </si>
+  <si>
+    <t>Leave balance should decrease according to approved leave days.</t>
+  </si>
+  <si>
+    <t>Verify Leave History Record Creation</t>
+  </si>
+  <si>
+    <t>1. Complete leave approval process. 2. Open Leave History.</t>
+  </si>
+  <si>
+    <t>Leave transaction should be recorded in leave history.</t>
+  </si>
+  <si>
+    <t>Verify Leave Cancellation Workflow</t>
+  </si>
+  <si>
+    <t>1. Employee submits leave request. 2. Cancel request before approval.</t>
+  </si>
+  <si>
+    <t>Verify Leave Notification Workflow</t>
+  </si>
+  <si>
+    <t>Appropriate notifications should be sent to employee and manager.</t>
+  </si>
+  <si>
+    <t>1. Submit leave request. 
+2. Approve or reject request.</t>
+  </si>
+  <si>
+    <t>Verify Complete Leave Lifecycle</t>
+  </si>
+  <si>
+    <t>Entire leave workflow should function correctly from submission to completion.</t>
+  </si>
+  <si>
+    <t>1. Submit leave request. 
+2. Manager approves request. 
+3. Employee views approved leave. 4. Check leave balance and history.</t>
+  </si>
+  <si>
+    <t>TC373</t>
+  </si>
+  <si>
+    <t>TC374</t>
+  </si>
+  <si>
+    <t>TC375</t>
+  </si>
+  <si>
+    <t>TC376</t>
+  </si>
+  <si>
+    <t>TC377</t>
+  </si>
+  <si>
+    <t>TC378</t>
+  </si>
+  <si>
+    <t>TC379</t>
+  </si>
+  <si>
+    <t>TC380</t>
+  </si>
+  <si>
+    <t>TC381</t>
+  </si>
+  <si>
+    <t>TC382</t>
   </si>
 </sst>
 </file>
@@ -4967,7 +5159,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G373"/>
+  <dimension ref="A1:G383"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -13559,6 +13751,236 @@
         <v>36</v>
       </c>
     </row>
+    <row r="374" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A374" s="1" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B374" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C374" s="2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="D374" s="2" t="s">
+        <v>1439</v>
+      </c>
+      <c r="E374" s="2" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F374" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G374" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="375" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A375" s="1" t="s">
+        <v>1465</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C375" s="2" t="s">
+        <v>1440</v>
+      </c>
+      <c r="D375" s="2" t="s">
+        <v>1442</v>
+      </c>
+      <c r="E375" s="2" t="s">
+        <v>1441</v>
+      </c>
+      <c r="F375" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G375" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="376" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A376" s="1" t="s">
+        <v>1466</v>
+      </c>
+      <c r="B376" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C376" s="2" t="s">
+        <v>1443</v>
+      </c>
+      <c r="D376" s="2" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E376" s="2" t="s">
+        <v>1444</v>
+      </c>
+      <c r="F376" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G376" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="377" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A377" s="1" t="s">
+        <v>1467</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C377" s="2" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D377" s="2" t="s">
+        <v>1448</v>
+      </c>
+      <c r="E377" s="2" t="s">
+        <v>1447</v>
+      </c>
+      <c r="F377" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G377" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="378" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A378" s="1" t="s">
+        <v>1468</v>
+      </c>
+      <c r="B378" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C378" s="2" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D378" s="2" t="s">
+        <v>1450</v>
+      </c>
+      <c r="E378" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="F378" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G378" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="379" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A379" s="1" t="s">
+        <v>1469</v>
+      </c>
+      <c r="B379" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C379" s="2" t="s">
+        <v>1451</v>
+      </c>
+      <c r="D379" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E379" s="2" t="s">
+        <v>1452</v>
+      </c>
+      <c r="F379" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G379" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A380" s="1" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B380" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C380" s="2" t="s">
+        <v>1453</v>
+      </c>
+      <c r="D380" s="2" t="s">
+        <v>1454</v>
+      </c>
+      <c r="E380" s="2" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F380" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G380" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A381" s="1" t="s">
+        <v>1471</v>
+      </c>
+      <c r="B381" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C381" s="2" t="s">
+        <v>1456</v>
+      </c>
+      <c r="D381" s="2" t="s">
+        <v>1457</v>
+      </c>
+      <c r="E381" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="F381" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G381" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="382" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A382" s="1" t="s">
+        <v>1472</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C382" s="2" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D382" s="2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="E382" s="2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="F382" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G382" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A383" s="1" t="s">
+        <v>1473</v>
+      </c>
+      <c r="B383" s="1" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C383" s="2" t="s">
+        <v>1461</v>
+      </c>
+      <c r="D383" s="2" t="s">
+        <v>1463</v>
+      </c>
+      <c r="E383" s="2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="F383" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G383" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
TC001 to TC017 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1486">
   <si>
     <t>TC ID</t>
   </si>
@@ -4816,6 +4816,43 @@
   </si>
   <si>
     <t>TC382</t>
+  </si>
+  <si>
+    <t>User Redirected to Dashboard Page successfully</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Invalid Credentials Error message displayed successfully</t>
+  </si>
+  <si>
+    <t>Required validation message displayed successfully</t>
+  </si>
+  <si>
+    <t>Password masked successfully</t>
+  </si>
+  <si>
+    <t>Login done successfully</t>
+  </si>
+  <si>
+    <t>Forgot Password page opened successfully</t>
+  </si>
+  <si>
+    <t>Nothing happened only page loads but after some time,
+504 Gateway Time-out , nginx/1.18.0 (ubuntu) Message shows</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Password Reset Message(page) displayed</t>
+  </si>
+  <si>
+    <t>User redireted to login page successfully</t>
+  </si>
+  <si>
+    <t>Access denined successfully but no message displayed</t>
   </si>
 </sst>
 </file>
@@ -5160,19 +5197,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G383"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.7109375" style="1"/>
+    <col min="4" max="4" width="32.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -5195,7 +5232,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -5212,13 +5249,13 @@
         <v>11</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>12</v>
+        <v>1474</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>37</v>
       </c>
@@ -5235,13 +5272,13 @@
         <v>15</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>12</v>
+        <v>1476</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>38</v>
       </c>
@@ -5258,13 +5295,13 @@
         <v>15</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>12</v>
+        <v>1476</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>39</v>
       </c>
@@ -5281,13 +5318,13 @@
         <v>15</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>12</v>
+        <v>1476</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>40</v>
       </c>
@@ -5304,13 +5341,13 @@
         <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>12</v>
+        <v>1477</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
@@ -5327,13 +5364,13 @@
         <v>22</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>12</v>
+        <v>1477</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>42</v>
       </c>
@@ -5350,13 +5387,13 @@
         <v>27</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>12</v>
+        <v>1477</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
@@ -5373,13 +5410,13 @@
         <v>30</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>12</v>
+        <v>1478</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
@@ -5396,13 +5433,13 @@
         <v>33</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>12</v>
+        <v>1479</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>45</v>
       </c>
@@ -5419,13 +5456,13 @@
         <v>33</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>12</v>
+        <v>1479</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -5442,13 +5479,13 @@
         <v>48</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>12</v>
+        <v>1480</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>61</v>
       </c>
@@ -5464,14 +5501,14 @@
       <c r="E13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>12</v>
+      <c r="F13" s="4" t="s">
+        <v>1481</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>62</v>
       </c>
@@ -5488,13 +5525,13 @@
         <v>54</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>12</v>
+        <v>1483</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>63</v>
       </c>
@@ -5511,13 +5548,13 @@
         <v>22</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>12</v>
+        <v>1477</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>64</v>
       </c>
@@ -5534,13 +5571,13 @@
         <v>59</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>12</v>
+        <v>1484</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -5557,13 +5594,13 @@
         <v>59</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>12</v>
+        <v>1484</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
@@ -5580,13 +5617,13 @@
         <v>69</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>12</v>
+        <v>1485</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -5609,7 +5646,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>82</v>
       </c>
@@ -5632,7 +5669,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>83</v>
       </c>
@@ -5655,7 +5692,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>114</v>
       </c>
@@ -5678,7 +5715,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>115</v>
       </c>
@@ -5701,7 +5738,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>116</v>
       </c>
@@ -5724,7 +5761,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>117</v>
       </c>
@@ -5747,7 +5784,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>118</v>
       </c>
@@ -5770,7 +5807,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>119</v>
       </c>
@@ -5793,7 +5830,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>120</v>
       </c>
@@ -5816,7 +5853,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>121</v>
       </c>
@@ -5839,7 +5876,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>122</v>
       </c>
@@ -5862,7 +5899,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>123</v>
       </c>
@@ -5885,7 +5922,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>154</v>
       </c>
@@ -5908,7 +5945,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>155</v>
       </c>
@@ -5931,7 +5968,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>156</v>
       </c>
@@ -5954,7 +5991,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>157</v>
       </c>
@@ -5977,7 +6014,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>158</v>
       </c>
@@ -6000,7 +6037,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>159</v>
       </c>
@@ -6023,7 +6060,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>160</v>
       </c>
@@ -6046,7 +6083,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>161</v>
       </c>
@@ -6069,7 +6106,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>162</v>
       </c>
@@ -6092,7 +6129,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>163</v>
       </c>
@@ -6115,7 +6152,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>188</v>
       </c>
@@ -6138,7 +6175,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>189</v>
       </c>
@@ -6161,7 +6198,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>190</v>
       </c>
@@ -6184,7 +6221,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>191</v>
       </c>
@@ -6207,7 +6244,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>192</v>
       </c>
@@ -6230,7 +6267,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>193</v>
       </c>
@@ -6253,7 +6290,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>194</v>
       </c>
@@ -6276,7 +6313,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>195</v>
       </c>
@@ -6299,7 +6336,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>220</v>
       </c>
@@ -6322,7 +6359,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>221</v>
       </c>
@@ -6345,7 +6382,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>222</v>
       </c>
@@ -6368,7 +6405,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>223</v>
       </c>
@@ -6391,7 +6428,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>224</v>
       </c>
@@ -6414,7 +6451,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>225</v>
       </c>
@@ -6437,7 +6474,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>226</v>
       </c>
@@ -6460,7 +6497,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>227</v>
       </c>
@@ -6483,7 +6520,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>228</v>
       </c>
@@ -6506,7 +6543,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>247</v>
       </c>
@@ -6529,7 +6566,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>248</v>
       </c>
@@ -6552,7 +6589,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>249</v>
       </c>
@@ -6575,7 +6612,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>250</v>
       </c>
@@ -6598,7 +6635,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>251</v>
       </c>
@@ -6621,7 +6658,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>252</v>
       </c>
@@ -6644,7 +6681,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>267</v>
       </c>
@@ -6667,7 +6704,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>268</v>
       </c>
@@ -6690,7 +6727,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>269</v>
       </c>
@@ -6713,7 +6750,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>270</v>
       </c>
@@ -6736,7 +6773,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>271</v>
       </c>
@@ -6759,7 +6796,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>286</v>
       </c>
@@ -6782,7 +6819,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>287</v>
       </c>
@@ -6805,7 +6842,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>288</v>
       </c>
@@ -6828,7 +6865,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>289</v>
       </c>
@@ -6851,7 +6888,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>290</v>
       </c>
@@ -6874,7 +6911,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>306</v>
       </c>
@@ -6897,7 +6934,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>307</v>
       </c>
@@ -6920,7 +6957,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>308</v>
       </c>
@@ -6943,7 +6980,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>309</v>
       </c>
@@ -6966,7 +7003,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>310</v>
       </c>
@@ -6989,7 +7026,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="80" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>324</v>
       </c>
@@ -7012,7 +7049,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>325</v>
       </c>
@@ -7035,7 +7072,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>326</v>
       </c>
@@ -7058,7 +7095,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="83" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>327</v>
       </c>
@@ -7081,7 +7118,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="84" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>328</v>
       </c>
@@ -7104,7 +7141,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>345</v>
       </c>
@@ -7127,7 +7164,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="86" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>346</v>
       </c>
@@ -7150,7 +7187,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>347</v>
       </c>
@@ -7173,7 +7210,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="88" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>348</v>
       </c>
@@ -7196,7 +7233,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="89" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>349</v>
       </c>
@@ -7219,7 +7256,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>365</v>
       </c>
@@ -7242,7 +7279,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="91" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>366</v>
       </c>
@@ -7265,7 +7302,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="92" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>367</v>
       </c>
@@ -7288,7 +7325,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="93" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>368</v>
       </c>
@@ -7311,7 +7348,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="94" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>369</v>
       </c>
@@ -7334,7 +7371,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="95" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>385</v>
       </c>
@@ -7357,7 +7394,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>386</v>
       </c>
@@ -7380,7 +7417,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="97" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>387</v>
       </c>
@@ -7403,7 +7440,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>388</v>
       </c>
@@ -7426,7 +7463,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="99" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>389</v>
       </c>
@@ -7449,7 +7486,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="100" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>406</v>
       </c>
@@ -7472,7 +7509,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>407</v>
       </c>
@@ -7495,7 +7532,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="102" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>408</v>
       </c>
@@ -7518,7 +7555,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="103" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>409</v>
       </c>
@@ -7541,7 +7578,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>410</v>
       </c>
@@ -7564,7 +7601,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>426</v>
       </c>
@@ -7587,7 +7624,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="106" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>427</v>
       </c>
@@ -7610,7 +7647,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="107" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>428</v>
       </c>
@@ -7633,7 +7670,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>429</v>
       </c>
@@ -7656,7 +7693,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="109" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>430</v>
       </c>
@@ -7679,7 +7716,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="110" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>446</v>
       </c>
@@ -7702,7 +7739,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>447</v>
       </c>
@@ -7725,7 +7762,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>448</v>
       </c>
@@ -7748,7 +7785,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>449</v>
       </c>
@@ -7771,7 +7808,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>450</v>
       </c>
@@ -7794,7 +7831,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="115" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>482</v>
       </c>
@@ -7817,7 +7854,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="116" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>483</v>
       </c>
@@ -7840,7 +7877,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="117" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>484</v>
       </c>
@@ -7863,7 +7900,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>485</v>
       </c>
@@ -7886,7 +7923,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="119" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>486</v>
       </c>
@@ -7909,7 +7946,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="120" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>487</v>
       </c>
@@ -7932,7 +7969,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="121" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>488</v>
       </c>
@@ -7955,7 +7992,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="122" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>489</v>
       </c>
@@ -7978,7 +8015,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="123" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>490</v>
       </c>
@@ -8001,7 +8038,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>491</v>
       </c>
@@ -8024,7 +8061,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>522</v>
       </c>
@@ -8047,7 +8084,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>523</v>
       </c>
@@ -8070,7 +8107,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="127" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>524</v>
       </c>
@@ -8093,7 +8130,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>525</v>
       </c>
@@ -8116,7 +8153,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>526</v>
       </c>
@@ -8139,7 +8176,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>527</v>
       </c>
@@ -8162,7 +8199,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>528</v>
       </c>
@@ -8185,7 +8222,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>529</v>
       </c>
@@ -8208,7 +8245,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>530</v>
       </c>
@@ -8231,7 +8268,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>531</v>
       </c>
@@ -8254,7 +8291,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>557</v>
       </c>
@@ -8277,7 +8314,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>558</v>
       </c>
@@ -8300,7 +8337,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>559</v>
       </c>
@@ -8323,7 +8360,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>560</v>
       </c>
@@ -8346,7 +8383,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>561</v>
       </c>
@@ -8369,7 +8406,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>562</v>
       </c>
@@ -8392,7 +8429,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>563</v>
       </c>
@@ -8415,7 +8452,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>564</v>
       </c>
@@ -8438,7 +8475,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="143" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>565</v>
       </c>
@@ -8461,7 +8498,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="144" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>566</v>
       </c>
@@ -8484,7 +8521,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="145" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>598</v>
       </c>
@@ -8507,7 +8544,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="146" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>599</v>
       </c>
@@ -8530,7 +8567,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="147" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>600</v>
       </c>
@@ -8553,7 +8590,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="148" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>601</v>
       </c>
@@ -8576,7 +8613,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>602</v>
       </c>
@@ -8599,7 +8636,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>603</v>
       </c>
@@ -8622,7 +8659,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="151" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>604</v>
       </c>
@@ -8645,7 +8682,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="152" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>605</v>
       </c>
@@ -8668,7 +8705,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>606</v>
       </c>
@@ -8691,7 +8728,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="154" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>607</v>
       </c>
@@ -8714,7 +8751,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="155" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>638</v>
       </c>
@@ -8737,7 +8774,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>639</v>
       </c>
@@ -8760,7 +8797,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="157" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>640</v>
       </c>
@@ -8783,7 +8820,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>641</v>
       </c>
@@ -8806,7 +8843,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="159" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>642</v>
       </c>
@@ -8829,7 +8866,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="160" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>643</v>
       </c>
@@ -8852,7 +8889,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="161" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>644</v>
       </c>
@@ -8875,7 +8912,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>645</v>
       </c>
@@ -8898,7 +8935,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>646</v>
       </c>
@@ -8921,7 +8958,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="164" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>647</v>
       </c>
@@ -8944,7 +8981,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>676</v>
       </c>
@@ -8967,7 +9004,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="166" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>677</v>
       </c>
@@ -8990,7 +9027,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="167" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>678</v>
       </c>
@@ -9013,7 +9050,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="168" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>679</v>
       </c>
@@ -9036,7 +9073,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="169" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>680</v>
       </c>
@@ -9059,7 +9096,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="170" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>681</v>
       </c>
@@ -9082,7 +9119,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="171" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>682</v>
       </c>
@@ -9105,7 +9142,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="172" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>683</v>
       </c>
@@ -9128,7 +9165,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="173" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>684</v>
       </c>
@@ -9151,7 +9188,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="174" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>685</v>
       </c>
@@ -9174,7 +9211,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>715</v>
       </c>
@@ -9197,7 +9234,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>716</v>
       </c>
@@ -9220,7 +9257,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="177" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>717</v>
       </c>
@@ -9243,7 +9280,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="178" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>718</v>
       </c>
@@ -9266,7 +9303,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="179" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>719</v>
       </c>
@@ -9289,7 +9326,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>720</v>
       </c>
@@ -9312,7 +9349,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="181" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>721</v>
       </c>
@@ -9335,7 +9372,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>722</v>
       </c>
@@ -9358,7 +9395,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="183" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>723</v>
       </c>
@@ -9381,7 +9418,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="184" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>724</v>
       </c>
@@ -9404,7 +9441,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="185" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>745</v>
       </c>
@@ -9427,7 +9464,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="186" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>746</v>
       </c>
@@ -9450,7 +9487,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>747</v>
       </c>
@@ -9473,7 +9510,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="188" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>748</v>
       </c>
@@ -9496,7 +9533,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="189" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>749</v>
       </c>
@@ -9519,7 +9556,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="190" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>750</v>
       </c>
@@ -9542,7 +9579,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="191" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>751</v>
       </c>
@@ -9565,7 +9602,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="192" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>752</v>
       </c>
@@ -9588,7 +9625,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="193" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>775</v>
       </c>
@@ -9611,7 +9648,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="194" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>776</v>
       </c>
@@ -9634,7 +9671,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="195" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>777</v>
       </c>
@@ -9657,7 +9694,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="196" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>778</v>
       </c>
@@ -9680,7 +9717,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="197" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>779</v>
       </c>
@@ -9703,7 +9740,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="198" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>780</v>
       </c>
@@ -9726,7 +9763,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="199" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>781</v>
       </c>
@@ -9749,7 +9786,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="200" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>782</v>
       </c>
@@ -9772,7 +9809,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="201" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>813</v>
       </c>
@@ -9795,7 +9832,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>814</v>
       </c>
@@ -9818,7 +9855,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="203" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>815</v>
       </c>
@@ -9841,7 +9878,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="204" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>816</v>
       </c>
@@ -9864,7 +9901,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="205" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>817</v>
       </c>
@@ -9887,7 +9924,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>818</v>
       </c>
@@ -9910,7 +9947,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>819</v>
       </c>
@@ -9933,7 +9970,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="208" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>820</v>
       </c>
@@ -9956,7 +9993,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="209" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>821</v>
       </c>
@@ -9979,7 +10016,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="210" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>822</v>
       </c>
@@ -10002,7 +10039,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>843</v>
       </c>
@@ -10025,7 +10062,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="212" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>844</v>
       </c>
@@ -10048,7 +10085,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="213" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>845</v>
       </c>
@@ -10071,7 +10108,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="214" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>846</v>
       </c>
@@ -10094,7 +10131,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="215" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>847</v>
       </c>
@@ -10117,7 +10154,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="216" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>848</v>
       </c>
@@ -10140,7 +10177,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="217" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>849</v>
       </c>
@@ -10163,7 +10200,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="218" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>867</v>
       </c>
@@ -10186,7 +10223,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="219" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>868</v>
       </c>
@@ -10209,7 +10246,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="220" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>869</v>
       </c>
@@ -10232,7 +10269,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="221" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>870</v>
       </c>
@@ -10255,7 +10292,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="222" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>871</v>
       </c>
@@ -10278,7 +10315,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="223" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>872</v>
       </c>
@@ -10301,7 +10338,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="224" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>873</v>
       </c>
@@ -10324,7 +10361,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>895</v>
       </c>
@@ -10347,7 +10384,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>896</v>
       </c>
@@ -10370,7 +10407,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="227" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>897</v>
       </c>
@@ -10393,7 +10430,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>898</v>
       </c>
@@ -10416,7 +10453,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="229" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>899</v>
       </c>
@@ -10439,7 +10476,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>900</v>
       </c>
@@ -10462,7 +10499,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>901</v>
       </c>
@@ -10485,7 +10522,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="232" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>902</v>
       </c>
@@ -10508,7 +10545,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="233" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>921</v>
       </c>
@@ -10531,7 +10568,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="234" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>922</v>
       </c>
@@ -10554,7 +10591,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="235" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>923</v>
       </c>
@@ -10577,7 +10614,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="236" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>924</v>
       </c>
@@ -10600,7 +10637,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="237" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>925</v>
       </c>
@@ -10623,7 +10660,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="238" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>926</v>
       </c>
@@ -10646,7 +10683,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="239" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>927</v>
       </c>
@@ -10669,7 +10706,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="240" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>928</v>
       </c>
@@ -10692,7 +10729,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="241" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>947</v>
       </c>
@@ -10715,7 +10752,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="242" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>948</v>
       </c>
@@ -10738,7 +10775,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="243" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>949</v>
       </c>
@@ -10761,7 +10798,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="244" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>950</v>
       </c>
@@ -10784,7 +10821,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="245" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>951</v>
       </c>
@@ -10807,7 +10844,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="246" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>952</v>
       </c>
@@ -10830,7 +10867,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="247" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>953</v>
       </c>
@@ -10853,7 +10890,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="248" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>954</v>
       </c>
@@ -10876,7 +10913,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="249" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>980</v>
       </c>
@@ -10899,7 +10936,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="250" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>981</v>
       </c>
@@ -10922,7 +10959,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="251" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>982</v>
       </c>
@@ -10945,7 +10982,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="252" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>983</v>
       </c>
@@ -10968,7 +11005,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="253" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>984</v>
       </c>
@@ -10991,7 +11028,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="254" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>985</v>
       </c>
@@ -11014,7 +11051,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="255" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>986</v>
       </c>
@@ -11037,7 +11074,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="256" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>987</v>
       </c>
@@ -11060,7 +11097,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="257" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>988</v>
       </c>
@@ -11083,7 +11120,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="258" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>1012</v>
       </c>
@@ -11106,7 +11143,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="259" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>1013</v>
       </c>
@@ -11129,7 +11166,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="260" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>1014</v>
       </c>
@@ -11152,7 +11189,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="261" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>1015</v>
       </c>
@@ -11175,7 +11212,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="262" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>1016</v>
       </c>
@@ -11198,7 +11235,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="263" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>1017</v>
       </c>
@@ -11221,7 +11258,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>1018</v>
       </c>
@@ -11244,7 +11281,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>1019</v>
       </c>
@@ -11267,7 +11304,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>1045</v>
       </c>
@@ -11290,7 +11327,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="267" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>1046</v>
       </c>
@@ -11313,7 +11350,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="268" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>1047</v>
       </c>
@@ -11336,7 +11373,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="269" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>1048</v>
       </c>
@@ -11359,7 +11396,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="270" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>1049</v>
       </c>
@@ -11382,7 +11419,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="271" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>1050</v>
       </c>
@@ -11405,7 +11442,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>1051</v>
       </c>
@@ -11428,7 +11465,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>1052</v>
       </c>
@@ -11451,7 +11488,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="274" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>1053</v>
       </c>
@@ -11474,7 +11511,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="275" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>1054</v>
       </c>
@@ -11497,7 +11534,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="276" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>1080</v>
       </c>
@@ -11520,7 +11557,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>1081</v>
       </c>
@@ -11543,7 +11580,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>1082</v>
       </c>
@@ -11566,7 +11603,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>1083</v>
       </c>
@@ -11589,7 +11626,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="280" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>1084</v>
       </c>
@@ -11612,7 +11649,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="281" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>1085</v>
       </c>
@@ -11635,7 +11672,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="282" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>1086</v>
       </c>
@@ -11658,7 +11695,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="283" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>1087</v>
       </c>
@@ -11681,7 +11718,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="284" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>1088</v>
       </c>
@@ -11704,7 +11741,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="285" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>1113</v>
       </c>
@@ -11727,7 +11764,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="286" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>1114</v>
       </c>
@@ -11750,7 +11787,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="287" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>1115</v>
       </c>
@@ -11773,7 +11810,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="288" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>1116</v>
       </c>
@@ -11796,7 +11833,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="289" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>1117</v>
       </c>
@@ -11819,7 +11856,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="290" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>1118</v>
       </c>
@@ -11842,7 +11879,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="291" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>1119</v>
       </c>
@@ -11865,7 +11902,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="292" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>1120</v>
       </c>
@@ -11888,7 +11925,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="293" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>1146</v>
       </c>
@@ -11911,7 +11948,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="294" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>1147</v>
       </c>
@@ -11934,7 +11971,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="295" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>1148</v>
       </c>
@@ -11957,7 +11994,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>1149</v>
       </c>
@@ -11980,7 +12017,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>1150</v>
       </c>
@@ -12003,7 +12040,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>1151</v>
       </c>
@@ -12026,7 +12063,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>1152</v>
       </c>
@@ -12049,7 +12086,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="300" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>1153</v>
       </c>
@@ -12072,7 +12109,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="301" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>1154</v>
       </c>
@@ -12095,7 +12132,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="302" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>1183</v>
       </c>
@@ -12118,7 +12155,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>1184</v>
       </c>
@@ -12141,7 +12178,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>1185</v>
       </c>
@@ -12164,7 +12201,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>1186</v>
       </c>
@@ -12187,7 +12224,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="306" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>1187</v>
       </c>
@@ -12210,7 +12247,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="307" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>1188</v>
       </c>
@@ -12233,7 +12270,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>1189</v>
       </c>
@@ -12256,7 +12293,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="309" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>1190</v>
       </c>
@@ -12279,7 +12316,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="310" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>1191</v>
       </c>
@@ -12302,7 +12339,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="311" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>1192</v>
       </c>
@@ -12325,7 +12362,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="312" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>1217</v>
       </c>
@@ -12348,7 +12385,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="313" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>1218</v>
       </c>
@@ -12371,7 +12408,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="314" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>1219</v>
       </c>
@@ -12394,7 +12431,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="315" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>1220</v>
       </c>
@@ -12417,7 +12454,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>1221</v>
       </c>
@@ -12440,7 +12477,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="317" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>1222</v>
       </c>
@@ -12463,7 +12500,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="318" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>1223</v>
       </c>
@@ -12486,7 +12523,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="319" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>1224</v>
       </c>
@@ -12509,7 +12546,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="320" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>1244</v>
       </c>
@@ -12532,7 +12569,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="321" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>1245</v>
       </c>
@@ -12555,7 +12592,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>1246</v>
       </c>
@@ -12578,7 +12615,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="323" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>1247</v>
       </c>
@@ -12601,7 +12638,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="324" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>1248</v>
       </c>
@@ -12624,7 +12661,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="325" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>1249</v>
       </c>
@@ -12647,7 +12684,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="326" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>1250</v>
       </c>
@@ -12670,7 +12707,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="327" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>1271</v>
       </c>
@@ -12693,7 +12730,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="328" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>1272</v>
       </c>
@@ -12716,7 +12753,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="329" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>1273</v>
       </c>
@@ -12739,7 +12776,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="330" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>1274</v>
       </c>
@@ -12762,7 +12799,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="331" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>1275</v>
       </c>
@@ -12785,7 +12822,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="332" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>1276</v>
       </c>
@@ -12808,7 +12845,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="333" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>1277</v>
       </c>
@@ -12831,7 +12868,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="334" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>1303</v>
       </c>
@@ -12854,7 +12891,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="335" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>1304</v>
       </c>
@@ -12877,7 +12914,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="336" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>1305</v>
       </c>
@@ -12900,7 +12937,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="337" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>1306</v>
       </c>
@@ -12923,7 +12960,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="338" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>1307</v>
       </c>
@@ -12946,7 +12983,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="339" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>1308</v>
       </c>
@@ -12969,7 +13006,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="340" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>1309</v>
       </c>
@@ -12992,7 +13029,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="341" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>1310</v>
       </c>
@@ -13015,7 +13052,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="342" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>1311</v>
       </c>
@@ -13038,7 +13075,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="343" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>1337</v>
       </c>
@@ -13061,7 +13098,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="344" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>1338</v>
       </c>
@@ -13084,7 +13121,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="345" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>1339</v>
       </c>
@@ -13107,7 +13144,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="346" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>1340</v>
       </c>
@@ -13130,7 +13167,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="347" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>1341</v>
       </c>
@@ -13153,7 +13190,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="348" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>1342</v>
       </c>
@@ -13176,7 +13213,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="349" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>1343</v>
       </c>
@@ -13199,7 +13236,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="350" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>1344</v>
       </c>
@@ -13222,7 +13259,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="351" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>1366</v>
       </c>
@@ -13245,7 +13282,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="352" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>1367</v>
       </c>
@@ -13268,7 +13305,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="353" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>1368</v>
       </c>
@@ -13291,7 +13328,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="354" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>1369</v>
       </c>
@@ -13314,7 +13351,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="355" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>1370</v>
       </c>
@@ -13337,7 +13374,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="356" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>1371</v>
       </c>
@@ -13360,7 +13397,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="357" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>1372</v>
       </c>
@@ -13383,7 +13420,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="358" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>1397</v>
       </c>
@@ -13406,7 +13443,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="359" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>1398</v>
       </c>
@@ -13429,7 +13466,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="360" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>1399</v>
       </c>
@@ -13452,7 +13489,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="361" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>1400</v>
       </c>
@@ -13475,7 +13512,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="362" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>1401</v>
       </c>
@@ -13498,7 +13535,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="363" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>1402</v>
       </c>
@@ -13521,7 +13558,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="364" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>1403</v>
       </c>
@@ -13544,7 +13581,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="365" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>1404</v>
       </c>
@@ -13567,7 +13604,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="366" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>1428</v>
       </c>
@@ -13590,7 +13627,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="367" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>1429</v>
       </c>
@@ -13613,7 +13650,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>1430</v>
       </c>
@@ -13636,7 +13673,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="369" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>1431</v>
       </c>
@@ -13659,7 +13696,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="370" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>1432</v>
       </c>
@@ -13682,7 +13719,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="371" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>1433</v>
       </c>
@@ -13705,7 +13742,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="372" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>1434</v>
       </c>
@@ -13728,7 +13765,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="373" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>1435</v>
       </c>
@@ -13751,7 +13788,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="374" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A374" s="1" t="s">
         <v>1464</v>
       </c>
@@ -13774,7 +13811,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="375" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>1465</v>
       </c>
@@ -13797,7 +13834,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="376" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>1466</v>
       </c>
@@ -13820,7 +13857,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="377" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>1467</v>
       </c>
@@ -13843,7 +13880,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="378" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>1468</v>
       </c>
@@ -13866,7 +13903,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="379" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>1469</v>
       </c>
@@ -13889,7 +13926,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="380" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>1470</v>
       </c>
@@ -13912,7 +13949,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="381" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>1471</v>
       </c>
@@ -13935,7 +13972,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="382" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>1472</v>
       </c>
@@ -13958,7 +13995,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="383" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>1473</v>
       </c>

</xml_diff>

<commit_message>
TC018 to TC032 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1500">
   <si>
     <t>TC ID</t>
   </si>
@@ -4853,6 +4853,50 @@
   </si>
   <si>
     <t>Access denined successfully but no message displayed</t>
+  </si>
+  <si>
+    <t>Dashboard accessible after logout</t>
+  </si>
+  <si>
+    <t>Logout option visible successfully</t>
+  </si>
+  <si>
+    <t>Login page displayed successfully</t>
+  </si>
+  <si>
+    <t>Dashboard page load successfully</t>
+  </si>
+  <si>
+    <t>Time at Work widget displayed successfully</t>
+  </si>
+  <si>
+    <t>My Actions widget visible successfully</t>
+  </si>
+  <si>
+    <t>Quick Launch options displayed successfully</t>
+  </si>
+  <si>
+    <t>Buzz Latest Posts section displayed successfully</t>
+  </si>
+  <si>
+    <t>Widget visible with employee leave information 
+successfully</t>
+  </si>
+  <si>
+    <t>Chart displayed properly</t>
+  </si>
+  <si>
+    <t>All widgets displayed valid data without errors</t>
+  </si>
+  <si>
+    <t>Dashboard scroll smoothly and all widgets accessible
+successfully</t>
+  </si>
+  <si>
+    <t>Assign page opened successfully</t>
+  </si>
+  <si>
+    <t>Leave List page opened successfully</t>
   </si>
 </sst>
 </file>
@@ -5640,10 +5684,10 @@
         <v>72</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>12</v>
+        <v>1486</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -5663,10 +5707,10 @@
         <v>75</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>12</v>
+        <v>1487</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -5686,10 +5730,10 @@
         <v>78</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>12</v>
+        <v>1488</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5709,10 +5753,10 @@
         <v>87</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>12</v>
+        <v>1489</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5732,10 +5776,10 @@
         <v>90</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>12</v>
+        <v>1490</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5755,10 +5799,10 @@
         <v>93</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>12</v>
+        <v>1491</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5778,10 +5822,10 @@
         <v>95</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>12</v>
+        <v>1492</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5801,10 +5845,10 @@
         <v>98</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>12</v>
+        <v>1493</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -5823,11 +5867,11 @@
       <c r="E27" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>12</v>
+      <c r="F27" s="4" t="s">
+        <v>1494</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -5847,10 +5891,10 @@
         <v>104</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>12</v>
+        <v>1495</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -5870,10 +5914,10 @@
         <v>104</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>12</v>
+        <v>1495</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5893,10 +5937,10 @@
         <v>109</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>12</v>
+        <v>1496</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5915,11 +5959,11 @@
       <c r="E31" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F31" s="3" t="s">
-        <v>12</v>
+      <c r="F31" s="4" t="s">
+        <v>1497</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -5939,10 +5983,10 @@
         <v>125</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>12</v>
+        <v>1498</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -5962,10 +6006,10 @@
         <v>128</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>12</v>
+        <v>1499</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC033 to TC050 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1518">
   <si>
     <t>TC ID</t>
   </si>
@@ -4897,6 +4897,60 @@
   </si>
   <si>
     <t>Leave List page opened successfully</t>
+  </si>
+  <si>
+    <t>Timesheets page opened successfully</t>
+  </si>
+  <si>
+    <t>Apply Leave page opened successfully</t>
+  </si>
+  <si>
+    <t>My Leave page opened successfully</t>
+  </si>
+  <si>
+    <t>My Timesheet page opened successfully</t>
+  </si>
+  <si>
+    <t>Profile menu options displayed successfully</t>
+  </si>
+  <si>
+    <t>Help page or help information opened successfully</t>
+  </si>
+  <si>
+    <t>Relevent Buzz post detailes displayed successfully</t>
+  </si>
+  <si>
+    <t>Relevent page oped successfully</t>
+  </si>
+  <si>
+    <t>Add Employee page opened successfully</t>
+  </si>
+  <si>
+    <t>Employee created successfully</t>
+  </si>
+  <si>
+    <t>Validation message displayed successfully</t>
+  </si>
+  <si>
+    <t>Image uploaded successfully</t>
+  </si>
+  <si>
+    <t>Employee ID field visible successfully</t>
+  </si>
+  <si>
+    <t>Login credential field displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee details saved successfully</t>
+  </si>
+  <si>
+    <t>User rediredcted without saving data successfully</t>
+  </si>
+  <si>
+    <t>Employee List page displayed successfully</t>
+  </si>
+  <si>
+    <t>Matching employee record displayed successfully</t>
   </si>
 </sst>
 </file>
@@ -6029,10 +6083,10 @@
         <v>131</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>12</v>
+        <v>1500</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6052,10 +6106,10 @@
         <v>134</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>12</v>
+        <v>1501</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6075,10 +6129,10 @@
         <v>137</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>12</v>
+        <v>1502</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6098,10 +6152,10 @@
         <v>140</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>12</v>
+        <v>1503</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6121,10 +6175,10 @@
         <v>143</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>12</v>
+        <v>1504</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6144,10 +6198,10 @@
         <v>146</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>12</v>
+        <v>1505</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6167,10 +6221,10 @@
         <v>149</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>12</v>
+        <v>1506</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -6190,10 +6244,10 @@
         <v>152</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>12</v>
+        <v>1507</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6213,10 +6267,10 @@
         <v>166</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>12</v>
+        <v>1508</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -6236,10 +6290,10 @@
         <v>169</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>12</v>
+        <v>1509</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6259,10 +6313,10 @@
         <v>172</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6282,10 +6336,10 @@
         <v>175</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>12</v>
+        <v>1511</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
@@ -6305,10 +6359,10 @@
         <v>179</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>12</v>
+        <v>1512</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6328,10 +6382,10 @@
         <v>181</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>12</v>
+        <v>1513</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6351,10 +6405,10 @@
         <v>184</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>12</v>
+        <v>1514</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6374,10 +6428,10 @@
         <v>186</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>12</v>
+        <v>1515</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6397,10 +6451,10 @@
         <v>197</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>12</v>
+        <v>1516</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6420,10 +6474,10 @@
         <v>200</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>12</v>
+        <v>1517</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC051 to TC073 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1535">
   <si>
     <t>TC ID</t>
   </si>
@@ -4951,6 +4951,57 @@
   </si>
   <si>
     <t>Matching employee record displayed successfully</t>
+  </si>
+  <si>
+    <t>Matching records displayed successfully</t>
+  </si>
+  <si>
+    <t>All filters cleared successfully</t>
+  </si>
+  <si>
+    <t>Employee records table displayed successfully</t>
+  </si>
+  <si>
+    <t>Edit icon visible for employee records</t>
+  </si>
+  <si>
+    <t>Employee information updated successfully</t>
+  </si>
+  <si>
+    <t>Updated information saved successfully</t>
+  </si>
+  <si>
+    <t>Updated contact information saved successfully</t>
+  </si>
+  <si>
+    <t>Changes stored successfully</t>
+  </si>
+  <si>
+    <t>Changes did't saved</t>
+  </si>
+  <si>
+    <t>Delete icon visible successfully</t>
+  </si>
+  <si>
+    <t>Employee record removed successfully</t>
+  </si>
+  <si>
+    <t>Confirmation popup displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee record did't deleted</t>
+  </si>
+  <si>
+    <t>Employee record did't found</t>
+  </si>
+  <si>
+    <t>Leave request submitted successfully</t>
+  </si>
+  <si>
+    <t>Corresponding leave balance displayed successfully</t>
+  </si>
+  <si>
+    <t>Seleted date displayed correctly</t>
   </si>
 </sst>
 </file>
@@ -6497,10 +6548,10 @@
         <v>200</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>12</v>
+        <v>1517</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6520,10 +6571,10 @@
         <v>205</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>12</v>
+        <v>1518</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6543,10 +6594,10 @@
         <v>205</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>12</v>
+        <v>1518</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6566,10 +6617,10 @@
         <v>210</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>12</v>
+        <v>1517</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6589,10 +6640,10 @@
         <v>205</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>12</v>
+        <v>1518</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6612,10 +6663,10 @@
         <v>215</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>12</v>
+        <v>1519</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -6635,10 +6686,10 @@
         <v>219</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>12</v>
+        <v>1520</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -6658,10 +6709,10 @@
         <v>231</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>12</v>
+        <v>1521</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6681,10 +6732,10 @@
         <v>233</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>12</v>
+        <v>1522</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6704,10 +6755,10 @@
         <v>237</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>12</v>
+        <v>1523</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6727,10 +6778,10 @@
         <v>239</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>12</v>
+        <v>1524</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6750,10 +6801,10 @@
         <v>242</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>12</v>
+        <v>1525</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6773,10 +6824,10 @@
         <v>245</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>12</v>
+        <v>1526</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
@@ -6796,10 +6847,10 @@
         <v>254</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>12</v>
+        <v>1527</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6819,10 +6870,10 @@
         <v>256</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>12</v>
+        <v>1528</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
@@ -6842,10 +6893,10 @@
         <v>260</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>12</v>
+        <v>1529</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6865,10 +6916,10 @@
         <v>262</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>12</v>
+        <v>1530</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6888,10 +6939,10 @@
         <v>265</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>12</v>
+        <v>1531</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -6911,10 +6962,10 @@
         <v>274</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>12</v>
+        <v>1501</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -6934,10 +6985,10 @@
         <v>277</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>12</v>
+        <v>1532</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -6957,10 +7008,10 @@
         <v>172</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
@@ -6980,10 +7031,10 @@
         <v>282</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>12</v>
+        <v>1533</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
@@ -7003,10 +7054,10 @@
         <v>285</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>12</v>
+        <v>1534</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC074 to TC095 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1557">
   <si>
     <t>TC ID</t>
   </si>
@@ -5002,6 +5002,73 @@
   </si>
   <si>
     <t>Seleted date displayed correctly</t>
+  </si>
+  <si>
+    <t>Pending leave requests displayed successfully</t>
+  </si>
+  <si>
+    <t>Leave status changes to Approved successfully</t>
+  </si>
+  <si>
+    <t>Leave status changes to Rejected successfully</t>
+  </si>
+  <si>
+    <t>Leave balance reduced accrodingly</t>
+  </si>
+  <si>
+    <t>Updated leave status displayed correctly</t>
+  </si>
+  <si>
+    <t>Applied leave records displayed successfully</t>
+  </si>
+  <si>
+    <t>Matching leave records displayed successfully</t>
+  </si>
+  <si>
+    <t>Current status displayed successfully</t>
+  </si>
+  <si>
+    <t>Leave request cancelled successfully</t>
+  </si>
+  <si>
+    <t>All selected filter cleared successfully</t>
+  </si>
+  <si>
+    <t>Timesheet page open successfully</t>
+  </si>
+  <si>
+    <t>User able to edit timesheet details successfully</t>
+  </si>
+  <si>
+    <t>New timesheet entry created successfully</t>
+  </si>
+  <si>
+    <t>Timesheet display selected week period successfully</t>
+  </si>
+  <si>
+    <t>"No Records Found" message displayed successfully</t>
+  </si>
+  <si>
+    <t>Submit button enabled successfully</t>
+  </si>
+  <si>
+    <t>Timesheet submitted successfully</t>
+  </si>
+  <si>
+    <t>Status changed from "Not Submitted" to "Submitted" 
+successfully</t>
+  </si>
+  <si>
+    <t>Appropriate validation/error message appear successfully</t>
+  </si>
+  <si>
+    <t>User able to modify submitted timesheet directly</t>
+  </si>
+  <si>
+    <t>Pending timesheets displayed successfully</t>
+  </si>
+  <si>
+    <t>Timesheet details opened successfully</t>
   </si>
 </sst>
 </file>
@@ -7077,10 +7144,10 @@
         <v>292</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>12</v>
+        <v>1535</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7100,10 +7167,10 @@
         <v>295</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>12</v>
+        <v>1536</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7123,10 +7190,10 @@
         <v>298</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>12</v>
+        <v>1537</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7146,10 +7213,10 @@
         <v>301</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>12</v>
+        <v>1538</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7169,10 +7236,10 @@
         <v>305</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>12</v>
+        <v>1539</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7192,10 +7259,10 @@
         <v>312</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>12</v>
+        <v>1540</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7215,10 +7282,10 @@
         <v>315</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>12</v>
+        <v>1541</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7238,10 +7305,10 @@
         <v>318</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>12</v>
+        <v>1542</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7261,10 +7328,10 @@
         <v>321</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>12</v>
+        <v>1543</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7284,10 +7351,10 @@
         <v>323</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>12</v>
+        <v>1544</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7307,10 +7374,10 @@
         <v>331</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>12</v>
+        <v>1545</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7330,10 +7397,10 @@
         <v>334</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>12</v>
+        <v>1546</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7353,10 +7420,10 @@
         <v>337</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>12</v>
+        <v>1547</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
@@ -7376,10 +7443,10 @@
         <v>341</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>12</v>
+        <v>1548</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
@@ -7399,10 +7466,10 @@
         <v>344</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>12</v>
+        <v>1549</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
@@ -7422,10 +7489,10 @@
         <v>352</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>12</v>
+        <v>1550</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7445,10 +7512,10 @@
         <v>354</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>12</v>
+        <v>1551</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7467,11 +7534,11 @@
       <c r="E92" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="F92" s="3" t="s">
-        <v>12</v>
+      <c r="F92" s="4" t="s">
+        <v>1552</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7491,10 +7558,10 @@
         <v>360</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>12</v>
+        <v>1553</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7514,10 +7581,10 @@
         <v>363</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>12</v>
+        <v>1554</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7537,10 +7604,10 @@
         <v>371</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>12</v>
+        <v>1555</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
@@ -7560,10 +7627,10 @@
         <v>375</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>12</v>
+        <v>1556</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC096 to TC114 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1576">
   <si>
     <t>TC ID</t>
   </si>
@@ -5069,6 +5069,63 @@
   </si>
   <si>
     <t>Timesheet details opened successfully</t>
+  </si>
+  <si>
+    <t>Timesheet status chnaged to Approved successfully</t>
+  </si>
+  <si>
+    <t>Timesheet status chnaged to Rejected successfully</t>
+  </si>
+  <si>
+    <t>Correct status displayed successfully</t>
+  </si>
+  <si>
+    <t>Vacancies page load successfully</t>
+  </si>
+  <si>
+    <t>New vacancy created successfully</t>
+  </si>
+  <si>
+    <t>Matching vacancies displayed successfully</t>
+  </si>
+  <si>
+    <t>Vacancy details updated successfully</t>
+  </si>
+  <si>
+    <t>Vacancy removed from the list successfully</t>
+  </si>
+  <si>
+    <t>Candidates page opened successfully</t>
+  </si>
+  <si>
+    <t>Candidate added successfully</t>
+  </si>
+  <si>
+    <t>Matching candidate records displayed successfully</t>
+  </si>
+  <si>
+    <t>Candidate profile details displayed successfully</t>
+  </si>
+  <si>
+    <t>Candidate record deleted successfully</t>
+  </si>
+  <si>
+    <t>Application created successfully</t>
+  </si>
+  <si>
+    <t>Status updated correctly</t>
+  </si>
+  <si>
+    <t>Candidate status chnaged to Shortlisted successfully</t>
+  </si>
+  <si>
+    <t>Candidate status chnaged to Rejected successfully</t>
+  </si>
+  <si>
+    <t>Candidate moved to Hired status and workflow completed</t>
+  </si>
+  <si>
+    <t>All extising users displayed successfully</t>
   </si>
 </sst>
 </file>
@@ -5420,7 +5477,7 @@
     <col min="3" max="3" width="48" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="47.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.7265625" style="1"/>
   </cols>
@@ -7650,10 +7707,10 @@
         <v>377</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>12</v>
+        <v>1557</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7673,10 +7730,10 @@
         <v>380</v>
       </c>
       <c r="F98" s="3" t="s">
-        <v>12</v>
+        <v>1558</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7696,10 +7753,10 @@
         <v>384</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>12</v>
+        <v>1559</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7719,10 +7776,10 @@
         <v>392</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>12</v>
+        <v>1560</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7742,10 +7799,10 @@
         <v>395</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>12</v>
+        <v>1561</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7765,10 +7822,10 @@
         <v>398</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>12</v>
+        <v>1562</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7788,10 +7845,10 @@
         <v>401</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>12</v>
+        <v>1563</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7811,10 +7868,10 @@
         <v>404</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>12</v>
+        <v>1564</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7834,10 +7891,10 @@
         <v>413</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>12</v>
+        <v>1565</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7857,10 +7914,10 @@
         <v>415</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>12</v>
+        <v>1566</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7880,10 +7937,10 @@
         <v>418</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>12</v>
+        <v>1567</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
@@ -7903,10 +7960,10 @@
         <v>422</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>12</v>
+        <v>1568</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7926,10 +7983,10 @@
         <v>424</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>12</v>
+        <v>1569</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7949,10 +8006,10 @@
         <v>432</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>12</v>
+        <v>1570</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -7972,10 +8029,10 @@
         <v>435</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>12</v>
+        <v>1571</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -7995,10 +8052,10 @@
         <v>438</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>12</v>
+        <v>1572</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8018,10 +8075,10 @@
         <v>441</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>12</v>
+        <v>1573</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8041,10 +8098,10 @@
         <v>444</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>12</v>
+        <v>1574</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8064,10 +8121,10 @@
         <v>454</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>12</v>
+        <v>1575</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC115 to TC137 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1599">
   <si>
     <t>TC ID</t>
   </si>
@@ -5126,6 +5126,75 @@
   </si>
   <si>
     <t>All extising users displayed successfully</t>
+  </si>
+  <si>
+    <t>New user created successfully</t>
+  </si>
+  <si>
+    <t>User information updated successfully</t>
+  </si>
+  <si>
+    <t>User removed successfully</t>
+  </si>
+  <si>
+    <t>Matching user records displayed successfully</t>
+  </si>
+  <si>
+    <t>Users belonging to selected role should be displayed</t>
+  </si>
+  <si>
+    <t>Relevent user record displayed successfully</t>
+  </si>
+  <si>
+    <t>Users with selected status displayed successfully</t>
+  </si>
+  <si>
+    <t>All search filters cleared successfully</t>
+  </si>
+  <si>
+    <t>User status updated correctly</t>
+  </si>
+  <si>
+    <t>Admin access all modules and features successfully</t>
+  </si>
+  <si>
+    <t>User access only permitted modules successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access denined successfully </t>
+  </si>
+  <si>
+    <t>New role assigned successfully</t>
+  </si>
+  <si>
+    <t>Updated permissions applied successfully</t>
+  </si>
+  <si>
+    <t>All users inherit the assigned permissions successfully</t>
+  </si>
+  <si>
+    <t>System block the action successfully</t>
+  </si>
+  <si>
+    <t>Menus displayed according to permissions successfully</t>
+  </si>
+  <si>
+    <t>Updated permissions reflect correctly</t>
+  </si>
+  <si>
+    <t>Assigned role remain unchanged</t>
+  </si>
+  <si>
+    <t>Matching user displayed successfully</t>
+  </si>
+  <si>
+    <t>Users of selected role displayed successfully</t>
+  </si>
+  <si>
+    <t>Relevent user records displayed successfully</t>
+  </si>
+  <si>
+    <t>Users with selected status appeared successfully</t>
   </si>
 </sst>
 </file>
@@ -8144,10 +8213,10 @@
         <v>456</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>12</v>
+        <v>1576</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -8167,10 +8236,10 @@
         <v>459</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>12</v>
+        <v>1577</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -8190,10 +8259,10 @@
         <v>462</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>12</v>
+        <v>1578</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8213,10 +8282,10 @@
         <v>465</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>12</v>
+        <v>1579</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8236,10 +8305,10 @@
         <v>469</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>12</v>
+        <v>1580</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8259,10 +8328,10 @@
         <v>471</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>12</v>
+        <v>1581</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8282,10 +8351,10 @@
         <v>475</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>12</v>
+        <v>1582</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8305,10 +8374,10 @@
         <v>477</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>12</v>
+        <v>1583</v>
       </c>
       <c r="G123" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8328,10 +8397,10 @@
         <v>480</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>12</v>
+        <v>1584</v>
       </c>
       <c r="G124" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.35">
@@ -8351,10 +8420,10 @@
         <v>494</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>12</v>
+        <v>1585</v>
       </c>
       <c r="G125" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.35">
@@ -8374,10 +8443,10 @@
         <v>497</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>12</v>
+        <v>1586</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8397,10 +8466,10 @@
         <v>499</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>12</v>
+        <v>1587</v>
       </c>
       <c r="G127" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -8420,10 +8489,10 @@
         <v>502</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>12</v>
+        <v>1588</v>
       </c>
       <c r="G128" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8443,10 +8512,10 @@
         <v>505</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>12</v>
+        <v>1589</v>
       </c>
       <c r="G129" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8466,10 +8535,10 @@
         <v>509</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>12</v>
+        <v>1590</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8489,10 +8558,10 @@
         <v>511</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>12</v>
+        <v>1591</v>
       </c>
       <c r="G131" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.35">
@@ -8512,10 +8581,10 @@
         <v>515</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>12</v>
+        <v>1592</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8535,10 +8604,10 @@
         <v>517</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>12</v>
+        <v>1593</v>
       </c>
       <c r="G133" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8558,10 +8627,10 @@
         <v>520</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>12</v>
+        <v>1594</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8581,10 +8650,10 @@
         <v>533</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>12</v>
+        <v>1595</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8604,10 +8673,10 @@
         <v>535</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>12</v>
+        <v>1596</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8627,10 +8696,10 @@
         <v>537</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>12</v>
+        <v>1597</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8650,10 +8719,10 @@
         <v>538</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>12</v>
+        <v>1598</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC138 to TC159 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1620">
   <si>
     <t>TC ID</t>
   </si>
@@ -5195,6 +5195,69 @@
   </si>
   <si>
     <t>Users with selected status appeared successfully</t>
+  </si>
+  <si>
+    <t>Results match all entered criteria successfully</t>
+  </si>
+  <si>
+    <t>No record displayed</t>
+  </si>
+  <si>
+    <t>All user records displayed successfully</t>
+  </si>
+  <si>
+    <t>Matching usernames did not displayed</t>
+  </si>
+  <si>
+    <t>Filters clear and default list displayed successfully</t>
+  </si>
+  <si>
+    <t>Displayed results exactly matched search criteria successfully</t>
+  </si>
+  <si>
+    <t>Employee personal information displayed correctly</t>
+  </si>
+  <si>
+    <t>Updated personal information saved successfully</t>
+  </si>
+  <si>
+    <t>Employee name updated successfully</t>
+  </si>
+  <si>
+    <t>Selected nationality saved correctly</t>
+  </si>
+  <si>
+    <t>Marital status updated successfully</t>
+  </si>
+  <si>
+    <t>Seleceted gender stored correctly</t>
+  </si>
+  <si>
+    <t>Date of birth updated successfully</t>
+  </si>
+  <si>
+    <t>License infromation saved successfully</t>
+  </si>
+  <si>
+    <t>Custom field infromation updated successfully</t>
+  </si>
+  <si>
+    <t>Attachment uploaded successfully</t>
+  </si>
+  <si>
+    <t>Emergency Contacts page load successfully</t>
+  </si>
+  <si>
+    <t>Emergency contacts added successfully</t>
+  </si>
+  <si>
+    <t>Updated contact infromation saved successfully</t>
+  </si>
+  <si>
+    <t>Contact removed successfully</t>
+  </si>
+  <si>
+    <t>Relationship stored correctly</t>
   </si>
 </sst>
 </file>
@@ -8742,10 +8805,10 @@
         <v>542</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>12</v>
+        <v>1599</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8765,10 +8828,10 @@
         <v>544</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>12</v>
+        <v>1600</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8788,10 +8851,10 @@
         <v>547</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>12</v>
+        <v>1601</v>
       </c>
       <c r="G141" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8811,10 +8874,10 @@
         <v>550</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>12</v>
+        <v>1602</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8834,10 +8897,10 @@
         <v>553</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>12</v>
+        <v>1603</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.35">
@@ -8857,10 +8920,10 @@
         <v>556</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>12</v>
+        <v>1604</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8880,10 +8943,10 @@
         <v>570</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>12</v>
+        <v>1605</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8903,10 +8966,10 @@
         <v>572</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>12</v>
+        <v>1606</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8926,10 +8989,10 @@
         <v>575</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>12</v>
+        <v>1607</v>
       </c>
       <c r="G147" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -8949,10 +9012,10 @@
         <v>578</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>12</v>
+        <v>1608</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8972,10 +9035,10 @@
         <v>581</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>12</v>
+        <v>1609</v>
       </c>
       <c r="G149" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -8995,10 +9058,10 @@
         <v>584</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>12</v>
+        <v>1610</v>
       </c>
       <c r="G150" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9018,10 +9081,10 @@
         <v>587</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>12</v>
+        <v>1611</v>
       </c>
       <c r="G151" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9041,10 +9104,10 @@
         <v>590</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>12</v>
+        <v>1612</v>
       </c>
       <c r="G152" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9064,10 +9127,10 @@
         <v>593</v>
       </c>
       <c r="F153" s="3" t="s">
-        <v>12</v>
+        <v>1613</v>
       </c>
       <c r="G153" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9087,10 +9150,10 @@
         <v>597</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>12</v>
+        <v>1614</v>
       </c>
       <c r="G154" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="155" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9110,10 +9173,10 @@
         <v>610</v>
       </c>
       <c r="F155" s="3" t="s">
-        <v>12</v>
+        <v>1615</v>
       </c>
       <c r="G155" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="156" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9133,10 +9196,10 @@
         <v>612</v>
       </c>
       <c r="F156" s="3" t="s">
-        <v>12</v>
+        <v>1616</v>
       </c>
       <c r="G156" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="157" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9156,10 +9219,10 @@
         <v>615</v>
       </c>
       <c r="F157" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G157" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9179,10 +9242,10 @@
         <v>618</v>
       </c>
       <c r="F158" s="3" t="s">
-        <v>12</v>
+        <v>1617</v>
       </c>
       <c r="G158" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9202,10 +9265,10 @@
         <v>621</v>
       </c>
       <c r="F159" s="3" t="s">
-        <v>12</v>
+        <v>1618</v>
       </c>
       <c r="G159" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9225,10 +9288,10 @@
         <v>623</v>
       </c>
       <c r="F160" s="3" t="s">
-        <v>12</v>
+        <v>1619</v>
       </c>
       <c r="G160" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC160 to TC182 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1641">
   <si>
     <t>TC ID</t>
   </si>
@@ -5258,6 +5258,69 @@
   </si>
   <si>
     <t>Relationship stored correctly</t>
+  </si>
+  <si>
+    <t>Validation error displayed successfully</t>
+  </si>
+  <si>
+    <t>All contect displayed correctly</t>
+  </si>
+  <si>
+    <t>Stored infromation match entered data successfully</t>
+  </si>
+  <si>
+    <t>Contact details remained available successfully</t>
+  </si>
+  <si>
+    <t>Qualifications page laod successfully</t>
+  </si>
+  <si>
+    <t>Education qualification added successfully</t>
+  </si>
+  <si>
+    <t>Work experience record addded successfully</t>
+  </si>
+  <si>
+    <t>Skill record saved successfully</t>
+  </si>
+  <si>
+    <t>Language qualification added successfully</t>
+  </si>
+  <si>
+    <t>Updated qualification saved successfully</t>
+  </si>
+  <si>
+    <t>Qualifications removed successfully</t>
+  </si>
+  <si>
+    <t>Validation messages appeared successfully</t>
+  </si>
+  <si>
+    <t>Saved qualificatiion details remain available successfully</t>
+  </si>
+  <si>
+    <t>Search page opened successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search input field displayed and accessible </t>
+  </si>
+  <si>
+    <t>Relevant search results displayed successfully</t>
+  </si>
+  <si>
+    <t>Exact matching result appeared successfully</t>
+  </si>
+  <si>
+    <t>No message displayed</t>
+  </si>
+  <si>
+    <t>Validation message or default behavior displayed</t>
+  </si>
+  <si>
+    <t>Results match entered search criteria successfully</t>
+  </si>
+  <si>
+    <t>Same results returned regardless of case</t>
   </si>
 </sst>
 </file>
@@ -5318,7 +5381,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9311,10 +9374,10 @@
         <v>627</v>
       </c>
       <c r="F161" s="3" t="s">
-        <v>12</v>
+        <v>1620</v>
       </c>
       <c r="G161" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.35">
@@ -9334,10 +9397,10 @@
         <v>631</v>
       </c>
       <c r="F162" s="3" t="s">
-        <v>12</v>
+        <v>1621</v>
       </c>
       <c r="G162" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.35">
@@ -9357,10 +9420,10 @@
         <v>634</v>
       </c>
       <c r="F163" s="3" t="s">
-        <v>12</v>
+        <v>1622</v>
       </c>
       <c r="G163" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="164" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9380,10 +9443,10 @@
         <v>636</v>
       </c>
       <c r="F164" s="3" t="s">
-        <v>12</v>
+        <v>1623</v>
       </c>
       <c r="G164" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9403,10 +9466,10 @@
         <v>650</v>
       </c>
       <c r="F165" s="3" t="s">
-        <v>12</v>
+        <v>1624</v>
       </c>
       <c r="G165" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="166" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9426,10 +9489,10 @@
         <v>652</v>
       </c>
       <c r="F166" s="3" t="s">
-        <v>12</v>
+        <v>1625</v>
       </c>
       <c r="G166" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="167" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9449,10 +9512,10 @@
         <v>655</v>
       </c>
       <c r="F167" s="3" t="s">
-        <v>12</v>
+        <v>1626</v>
       </c>
       <c r="G167" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="168" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9472,10 +9535,10 @@
         <v>658</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>12</v>
+        <v>1627</v>
       </c>
       <c r="G168" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9495,10 +9558,10 @@
         <v>661</v>
       </c>
       <c r="F169" s="3" t="s">
-        <v>12</v>
+        <v>1628</v>
       </c>
       <c r="G169" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9518,10 +9581,10 @@
         <v>590</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>12</v>
+        <v>1612</v>
       </c>
       <c r="G170" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9541,10 +9604,10 @@
         <v>666</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>12</v>
+        <v>1629</v>
       </c>
       <c r="G171" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="172" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9564,10 +9627,10 @@
         <v>669</v>
       </c>
       <c r="F172" s="3" t="s">
-        <v>12</v>
+        <v>1630</v>
       </c>
       <c r="G172" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="173" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9587,10 +9650,10 @@
         <v>671</v>
       </c>
       <c r="F173" s="3" t="s">
-        <v>12</v>
+        <v>1631</v>
       </c>
       <c r="G173" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9610,10 +9673,10 @@
         <v>674</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>12</v>
+        <v>1632</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.35">
@@ -9633,10 +9696,10 @@
         <v>689</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>12</v>
+        <v>1633</v>
       </c>
       <c r="G175" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.35">
@@ -9656,10 +9719,10 @@
         <v>692</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>12</v>
+        <v>1634</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9679,10 +9742,10 @@
         <v>694</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>12</v>
+        <v>1635</v>
       </c>
       <c r="G177" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9702,10 +9765,10 @@
         <v>205</v>
       </c>
       <c r="F178" s="3" t="s">
-        <v>12</v>
+        <v>1518</v>
       </c>
       <c r="G178" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9725,10 +9788,10 @@
         <v>699</v>
       </c>
       <c r="F179" s="3" t="s">
-        <v>12</v>
+        <v>1636</v>
       </c>
       <c r="G179" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9748,10 +9811,10 @@
         <v>702</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>12</v>
+        <v>1637</v>
       </c>
       <c r="G180" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9771,10 +9834,10 @@
         <v>705</v>
       </c>
       <c r="F181" s="3" t="s">
-        <v>12</v>
+        <v>1638</v>
       </c>
       <c r="G181" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.35">
@@ -9794,10 +9857,10 @@
         <v>708</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>12</v>
+        <v>1639</v>
       </c>
       <c r="G182" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9817,10 +9880,10 @@
         <v>711</v>
       </c>
       <c r="F183" s="3" t="s">
-        <v>12</v>
+        <v>1640</v>
       </c>
       <c r="G183" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC183 to TC206 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1663">
   <si>
     <t>TC ID</t>
   </si>
@@ -5321,6 +5321,72 @@
   </si>
   <si>
     <t>Same results returned regardless of case</t>
+  </si>
+  <si>
+    <t>Results displayed within acceptable response time successfully</t>
+  </si>
+  <si>
+    <t>Employee Reviews page opened successfully</t>
+  </si>
+  <si>
+    <t>Matching employee review records displayed successfully</t>
+  </si>
+  <si>
+    <t>Reviews matching selected job title displayed successfully</t>
+  </si>
+  <si>
+    <t>Reviews with selected status displayed successfully</t>
+  </si>
+  <si>
+    <t>Reviews within selected date range displayed successfully</t>
+  </si>
+  <si>
+    <t>Filtered review records displayed correctly</t>
+  </si>
+  <si>
+    <t>All filter fields cleared/reset successfully</t>
+  </si>
+  <si>
+    <t>Records filtered based on selected status successfully</t>
+  </si>
+  <si>
+    <t>Matching review records displayed successfully</t>
+  </si>
+  <si>
+    <t>Relevant employee reviews displayed successfully</t>
+  </si>
+  <si>
+    <t>Reviews for selected job title displayed successfully</t>
+  </si>
+  <si>
+    <t>Results filtered according to selected option successfully</t>
+  </si>
+  <si>
+    <t>Reviews within selected date displayed successfully</t>
+  </si>
+  <si>
+    <t>Results satisfy all selected filter criteria successfully</t>
+  </si>
+  <si>
+    <t>Existing review records displayed in grid successfully</t>
+  </si>
+  <si>
+    <t>Review details displayed correctly</t>
+  </si>
+  <si>
+    <t>New review created successfully</t>
+  </si>
+  <si>
+    <t>Changes saved successfully</t>
+  </si>
+  <si>
+    <t>Review removed successfully</t>
+  </si>
+  <si>
+    <t>Assigned reviews displayed correctly</t>
+  </si>
+  <si>
+    <t>User's trackers displayed successfully</t>
   </si>
 </sst>
 </file>
@@ -9903,10 +9969,10 @@
         <v>714</v>
       </c>
       <c r="F184" s="3" t="s">
-        <v>12</v>
+        <v>1641</v>
       </c>
       <c r="G184" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -9926,10 +9992,10 @@
         <v>728</v>
       </c>
       <c r="F185" s="3" t="s">
-        <v>12</v>
+        <v>1642</v>
       </c>
       <c r="G185" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9949,10 +10015,10 @@
         <v>729</v>
       </c>
       <c r="F186" s="3" t="s">
-        <v>12</v>
+        <v>1643</v>
       </c>
       <c r="G186" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="187" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9972,10 +10038,10 @@
         <v>731</v>
       </c>
       <c r="F187" s="3" t="s">
-        <v>12</v>
+        <v>1644</v>
       </c>
       <c r="G187" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -9995,10 +10061,10 @@
         <v>733</v>
       </c>
       <c r="F188" s="3" t="s">
-        <v>12</v>
+        <v>1645</v>
       </c>
       <c r="G188" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="189" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10018,10 +10084,10 @@
         <v>736</v>
       </c>
       <c r="F189" s="3" t="s">
-        <v>12</v>
+        <v>1646</v>
       </c>
       <c r="G189" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="190" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10041,10 +10107,10 @@
         <v>739</v>
       </c>
       <c r="F190" s="3" t="s">
-        <v>12</v>
+        <v>1647</v>
       </c>
       <c r="G190" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10064,10 +10130,10 @@
         <v>742</v>
       </c>
       <c r="F191" s="3" t="s">
-        <v>12</v>
+        <v>1648</v>
       </c>
       <c r="G191" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10087,10 +10153,10 @@
         <v>344</v>
       </c>
       <c r="F192" s="3" t="s">
-        <v>12</v>
+        <v>1549</v>
       </c>
       <c r="G192" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10110,10 +10176,10 @@
         <v>754</v>
       </c>
       <c r="F193" s="3" t="s">
-        <v>12</v>
+        <v>1649</v>
       </c>
       <c r="G193" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="194" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10133,10 +10199,10 @@
         <v>757</v>
       </c>
       <c r="F194" s="3" t="s">
-        <v>12</v>
+        <v>1650</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="195" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10156,10 +10222,10 @@
         <v>760</v>
       </c>
       <c r="F195" s="3" t="s">
-        <v>12</v>
+        <v>1651</v>
       </c>
       <c r="G195" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10179,10 +10245,10 @@
         <v>763</v>
       </c>
       <c r="F196" s="3" t="s">
-        <v>12</v>
+        <v>1652</v>
       </c>
       <c r="G196" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="197" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10202,10 +10268,10 @@
         <v>767</v>
       </c>
       <c r="F197" s="3" t="s">
-        <v>12</v>
+        <v>1653</v>
       </c>
       <c r="G197" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="198" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10225,10 +10291,10 @@
         <v>769</v>
       </c>
       <c r="F198" s="3" t="s">
-        <v>12</v>
+        <v>1654</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="199" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10248,10 +10314,10 @@
         <v>772</v>
       </c>
       <c r="F199" s="3" t="s">
-        <v>12</v>
+        <v>1655</v>
       </c>
       <c r="G199" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="200" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10271,10 +10337,10 @@
         <v>323</v>
       </c>
       <c r="F200" s="3" t="s">
-        <v>12</v>
+        <v>1544</v>
       </c>
       <c r="G200" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.35">
@@ -10294,10 +10360,10 @@
         <v>785</v>
       </c>
       <c r="F201" s="3" t="s">
-        <v>12</v>
+        <v>1656</v>
       </c>
       <c r="G201" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.35">
@@ -10317,10 +10383,10 @@
         <v>788</v>
       </c>
       <c r="F202" s="3" t="s">
-        <v>12</v>
+        <v>1657</v>
       </c>
       <c r="G202" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="203" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10340,10 +10406,10 @@
         <v>790</v>
       </c>
       <c r="F203" s="3" t="s">
-        <v>12</v>
+        <v>1658</v>
       </c>
       <c r="G203" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="204" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10363,10 +10429,10 @@
         <v>793</v>
       </c>
       <c r="F204" s="3" t="s">
-        <v>12</v>
+        <v>1659</v>
       </c>
       <c r="G204" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="205" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10386,10 +10452,10 @@
         <v>796</v>
       </c>
       <c r="F205" s="3" t="s">
-        <v>12</v>
+        <v>1660</v>
       </c>
       <c r="G205" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.35">
@@ -10409,10 +10475,10 @@
         <v>800</v>
       </c>
       <c r="F206" s="3" t="s">
-        <v>12</v>
+        <v>1661</v>
       </c>
       <c r="G206" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.35">
@@ -10432,10 +10498,10 @@
         <v>803</v>
       </c>
       <c r="F207" s="3" t="s">
-        <v>12</v>
+        <v>1662</v>
       </c>
       <c r="G207" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="208" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC207 to TC232 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1663">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1688">
   <si>
     <t>TC ID</t>
   </si>
@@ -5387,6 +5387,81 @@
   </si>
   <si>
     <t>User's trackers displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee tracker records displayed correctly</t>
+  </si>
+  <si>
+    <t>Tracker infromation displayed successfully</t>
+  </si>
+  <si>
+    <t>Records sorted correctly in ascending/descending oder</t>
+  </si>
+  <si>
+    <t>Directory page opened successfully</t>
+  </si>
+  <si>
+    <t>No matching records displayed successfully</t>
+  </si>
+  <si>
+    <t>Matching employee records displayed successfully</t>
+  </si>
+  <si>
+    <t>Relevant employee records displayed successfully</t>
+  </si>
+  <si>
+    <t>Exact employee profile displayed successfully</t>
+  </si>
+  <si>
+    <t>Search execute successfully</t>
+  </si>
+  <si>
+    <t>Record count match displayed employee cards successfully</t>
+  </si>
+  <si>
+    <t>Employee matching selected job title displayed successfully</t>
+  </si>
+  <si>
+    <t>Employees from selected location displayed successfully</t>
+  </si>
+  <si>
+    <t>Filtered employee records displayed correctly</t>
+  </si>
+  <si>
+    <t>All filter values cleared successfully</t>
+  </si>
+  <si>
+    <t>Result satisfy all filter conditions successfully</t>
+  </si>
+  <si>
+    <t>All employee records displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee cards displayed properly</t>
+  </si>
+  <si>
+    <t>Employee name displayed correctly</t>
+  </si>
+  <si>
+    <t>Profile image/avatar displayed correctly</t>
+  </si>
+  <si>
+    <t>Multiple employee records visible successfully</t>
+  </si>
+  <si>
+    <t>Information matched system records</t>
+  </si>
+  <si>
+    <t>Total records count displayed correctly</t>
+  </si>
+  <si>
+    <t>Cards aligned and displayed properly</t>
+  </si>
+  <si>
+    <t>Employee details accessible successfully</t>
+  </si>
+  <si>
+    <t>Purge Employee records page opened successfully</t>
   </si>
 </sst>
 </file>
@@ -10521,10 +10596,10 @@
         <v>806</v>
       </c>
       <c r="F208" s="3" t="s">
-        <v>12</v>
+        <v>1663</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.35">
@@ -10544,10 +10619,10 @@
         <v>809</v>
       </c>
       <c r="F209" s="3" t="s">
-        <v>12</v>
+        <v>1664</v>
       </c>
       <c r="G209" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="210" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10567,10 +10642,10 @@
         <v>812</v>
       </c>
       <c r="F210" s="3" t="s">
-        <v>12</v>
+        <v>1665</v>
       </c>
       <c r="G210" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.35">
@@ -10590,10 +10665,10 @@
         <v>826</v>
       </c>
       <c r="F211" s="3" t="s">
-        <v>12</v>
+        <v>1666</v>
       </c>
       <c r="G211" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="212" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10613,10 +10688,10 @@
         <v>210</v>
       </c>
       <c r="F212" s="3" t="s">
-        <v>12</v>
+        <v>1668</v>
       </c>
       <c r="G212" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="213" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10636,10 +10711,10 @@
         <v>829</v>
       </c>
       <c r="F213" s="3" t="s">
-        <v>12</v>
+        <v>1669</v>
       </c>
       <c r="G213" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="214" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10659,10 +10734,10 @@
         <v>833</v>
       </c>
       <c r="F214" s="3" t="s">
-        <v>12</v>
+        <v>1670</v>
       </c>
       <c r="G214" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="215" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10682,10 +10757,10 @@
         <v>835</v>
       </c>
       <c r="F215" s="3" t="s">
-        <v>12</v>
+        <v>1667</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="216" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10705,10 +10780,10 @@
         <v>838</v>
       </c>
       <c r="F216" s="3" t="s">
-        <v>12</v>
+        <v>1671</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.35">
@@ -10728,10 +10803,10 @@
         <v>842</v>
       </c>
       <c r="F217" s="3" t="s">
-        <v>12</v>
+        <v>1672</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="218" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10751,10 +10826,10 @@
         <v>850</v>
       </c>
       <c r="F218" s="3" t="s">
-        <v>12</v>
+        <v>1673</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="219" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10774,10 +10849,10 @@
         <v>853</v>
       </c>
       <c r="F219" s="3" t="s">
-        <v>12</v>
+        <v>1674</v>
       </c>
       <c r="G219" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="220" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10797,10 +10872,10 @@
         <v>856</v>
       </c>
       <c r="F220" s="3" t="s">
-        <v>12</v>
+        <v>1675</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="221" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -10820,10 +10895,10 @@
         <v>210</v>
       </c>
       <c r="F221" s="3" t="s">
-        <v>12</v>
+        <v>1668</v>
       </c>
       <c r="G221" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="222" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -10843,10 +10918,10 @@
         <v>861</v>
       </c>
       <c r="F222" s="3" t="s">
-        <v>12</v>
+        <v>1677</v>
       </c>
       <c r="G222" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="223" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10866,10 +10941,10 @@
         <v>863</v>
       </c>
       <c r="F223" s="3" t="s">
-        <v>12</v>
+        <v>1676</v>
       </c>
       <c r="G223" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="224" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -10889,10 +10964,10 @@
         <v>865</v>
       </c>
       <c r="F224" s="3" t="s">
-        <v>12</v>
+        <v>1678</v>
       </c>
       <c r="G224" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.35">
@@ -10912,10 +10987,10 @@
         <v>876</v>
       </c>
       <c r="F225" s="3" t="s">
-        <v>12</v>
+        <v>1679</v>
       </c>
       <c r="G225" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.35">
@@ -10935,10 +11010,10 @@
         <v>879</v>
       </c>
       <c r="F226" s="3" t="s">
-        <v>12</v>
+        <v>1680</v>
       </c>
       <c r="G226" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.35">
@@ -10958,10 +11033,10 @@
         <v>881</v>
       </c>
       <c r="F227" s="3" t="s">
-        <v>12</v>
+        <v>1681</v>
       </c>
       <c r="G227" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.35">
@@ -10981,10 +11056,10 @@
         <v>883</v>
       </c>
       <c r="F228" s="3" t="s">
-        <v>12</v>
+        <v>1682</v>
       </c>
       <c r="G228" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="229" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11004,10 +11079,10 @@
         <v>886</v>
       </c>
       <c r="F229" s="3" t="s">
-        <v>12</v>
+        <v>1683</v>
       </c>
       <c r="G229" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.35">
@@ -11027,10 +11102,10 @@
         <v>888</v>
       </c>
       <c r="F230" s="3" t="s">
-        <v>12</v>
+        <v>1684</v>
       </c>
       <c r="G230" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.35">
@@ -11050,10 +11125,10 @@
         <v>891</v>
       </c>
       <c r="F231" s="3" t="s">
-        <v>12</v>
+        <v>1685</v>
       </c>
       <c r="G231" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="232" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11073,10 +11148,10 @@
         <v>894</v>
       </c>
       <c r="F232" s="3" t="s">
-        <v>12</v>
+        <v>1686</v>
       </c>
       <c r="G232" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="233" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11096,10 +11171,10 @@
         <v>906</v>
       </c>
       <c r="F233" s="3" t="s">
-        <v>12</v>
+        <v>1687</v>
       </c>
       <c r="G233" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="234" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC233 to TC256 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1706">
   <si>
     <t>TC ID</t>
   </si>
@@ -5462,6 +5462,62 @@
   </si>
   <si>
     <t>Purge Employee records page opened successfully</t>
+  </si>
+  <si>
+    <t>Past Employee search field displayed successfully</t>
+  </si>
+  <si>
+    <t>No matching record found successfully</t>
+  </si>
+  <si>
+    <t>Employee record permanently removed successfully</t>
+  </si>
+  <si>
+    <t>Purged employee not appeared in search results successfully</t>
+  </si>
+  <si>
+    <t>Access Records page opened successfully</t>
+  </si>
+  <si>
+    <t>Dowload Personal Data section displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee Name earch field available successfully</t>
+  </si>
+  <si>
+    <t>Matching employee information retrieved successfully</t>
+  </si>
+  <si>
+    <t>No matching records returned successfully</t>
+  </si>
+  <si>
+    <t>Personal data request processed successfully</t>
+  </si>
+  <si>
+    <t>Administrator Access popup displayed successfully</t>
+  </si>
+  <si>
+    <t>Logged-in admin username displayed successfully</t>
+  </si>
+  <si>
+    <t>Password field available for credential validation successfully</t>
+  </si>
+  <si>
+    <t>Access to Maintenance module granted successfully</t>
+  </si>
+  <si>
+    <t>Access denied and error message displayed successfully</t>
+  </si>
+  <si>
+    <t>Access popup close and Maintenance page not opened 
+successfully</t>
+  </si>
+  <si>
+    <t>User prevented from accessing Maintenance functions 
+successfully</t>
+  </si>
+  <si>
+    <t>Access remian valid only for authorized session successfully</t>
   </si>
 </sst>
 </file>
@@ -11194,10 +11250,10 @@
         <v>909</v>
       </c>
       <c r="F234" s="3" t="s">
-        <v>12</v>
+        <v>1688</v>
       </c>
       <c r="G234" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="235" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11217,10 +11273,10 @@
         <v>200</v>
       </c>
       <c r="F235" s="3" t="s">
-        <v>12</v>
+        <v>1517</v>
       </c>
       <c r="G235" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="236" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11240,10 +11296,10 @@
         <v>829</v>
       </c>
       <c r="F236" s="3" t="s">
-        <v>12</v>
+        <v>1669</v>
       </c>
       <c r="G236" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="237" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11263,10 +11319,10 @@
         <v>912</v>
       </c>
       <c r="F237" s="3" t="s">
-        <v>12</v>
+        <v>1689</v>
       </c>
       <c r="G237" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="238" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11286,10 +11342,10 @@
         <v>172</v>
       </c>
       <c r="F238" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G238" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="239" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -11309,10 +11365,10 @@
         <v>916</v>
       </c>
       <c r="F239" s="3" t="s">
-        <v>12</v>
+        <v>1690</v>
       </c>
       <c r="G239" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="240" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11332,10 +11388,10 @@
         <v>919</v>
       </c>
       <c r="F240" s="3" t="s">
-        <v>12</v>
+        <v>1691</v>
       </c>
       <c r="G240" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="241" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11355,10 +11411,10 @@
         <v>931</v>
       </c>
       <c r="F241" s="3" t="s">
-        <v>12</v>
+        <v>1692</v>
       </c>
       <c r="G241" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.35">
@@ -11378,10 +11434,10 @@
         <v>934</v>
       </c>
       <c r="F242" s="3" t="s">
-        <v>12</v>
+        <v>1693</v>
       </c>
       <c r="G242" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="243" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11401,10 +11457,10 @@
         <v>937</v>
       </c>
       <c r="F243" s="3" t="s">
-        <v>12</v>
+        <v>1694</v>
       </c>
       <c r="G243" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="244" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11424,10 +11480,10 @@
         <v>939</v>
       </c>
       <c r="F244" s="3" t="s">
-        <v>12</v>
+        <v>1695</v>
       </c>
       <c r="G244" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="245" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11447,10 +11503,10 @@
         <v>829</v>
       </c>
       <c r="F245" s="3" t="s">
-        <v>12</v>
+        <v>1669</v>
       </c>
       <c r="G245" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="246" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11470,10 +11526,10 @@
         <v>941</v>
       </c>
       <c r="F246" s="3" t="s">
-        <v>12</v>
+        <v>1696</v>
       </c>
       <c r="G246" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="247" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11493,10 +11549,10 @@
         <v>172</v>
       </c>
       <c r="F247" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G247" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="248" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -11516,10 +11572,10 @@
         <v>945</v>
       </c>
       <c r="F248" s="3" t="s">
-        <v>12</v>
+        <v>1697</v>
       </c>
       <c r="G248" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.35">
@@ -11539,10 +11595,10 @@
         <v>957</v>
       </c>
       <c r="F249" s="3" t="s">
-        <v>12</v>
+        <v>1698</v>
       </c>
       <c r="G249" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.35">
@@ -11562,10 +11618,10 @@
         <v>960</v>
       </c>
       <c r="F250" s="3" t="s">
-        <v>12</v>
+        <v>1699</v>
       </c>
       <c r="G250" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="251" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11585,10 +11641,10 @@
         <v>962</v>
       </c>
       <c r="F251" s="3" t="s">
-        <v>12</v>
+        <v>1700</v>
       </c>
       <c r="G251" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="252" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11608,10 +11664,10 @@
         <v>964</v>
       </c>
       <c r="F252" s="3" t="s">
-        <v>12</v>
+        <v>1701</v>
       </c>
       <c r="G252" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="253" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11631,10 +11687,10 @@
         <v>967</v>
       </c>
       <c r="F253" s="3" t="s">
-        <v>12</v>
+        <v>1702</v>
       </c>
       <c r="G253" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="254" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11654,10 +11710,10 @@
         <v>172</v>
       </c>
       <c r="F254" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G254" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="255" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11676,11 +11732,11 @@
       <c r="E255" s="2" t="s">
         <v>973</v>
       </c>
-      <c r="F255" s="3" t="s">
-        <v>12</v>
+      <c r="F255" s="4" t="s">
+        <v>1703</v>
       </c>
       <c r="G255" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="256" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11699,11 +11755,11 @@
       <c r="E256" s="2" t="s">
         <v>976</v>
       </c>
-      <c r="F256" s="3" t="s">
-        <v>12</v>
+      <c r="F256" s="4" t="s">
+        <v>1704</v>
       </c>
       <c r="G256" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="257" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11723,10 +11779,10 @@
         <v>979</v>
       </c>
       <c r="F257" s="3" t="s">
-        <v>12</v>
+        <v>1705</v>
       </c>
       <c r="G257" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="258" spans="1:7" ht="58" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC257 to TC281 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1730">
   <si>
     <t>TC ID</t>
   </si>
@@ -5467,6 +5467,9 @@
     <t>Past Employee search field displayed successfully</t>
   </si>
   <si>
+    <t>Pas</t>
+  </si>
+  <si>
     <t>No matching record found successfully</t>
   </si>
   <si>
@@ -5518,6 +5521,75 @@
   </si>
   <si>
     <t>Access remian valid only for authorized session successfully</t>
+  </si>
+  <si>
+    <t>Claim request created successfully</t>
+  </si>
+  <si>
+    <t>Claim submitted successfully</t>
+  </si>
+  <si>
+    <t>Claim creation cancelled and page reset successfully</t>
+  </si>
+  <si>
+    <t>Claim assigned to selected employee successfully</t>
+  </si>
+  <si>
+    <t>Assigned claim visible in records list successfully</t>
+  </si>
+  <si>
+    <t>Unique claim reference ID generated successfully</t>
+  </si>
+  <si>
+    <t>Correct claim amount displayed successfully</t>
+  </si>
+  <si>
+    <t>My Claims page opend successfully</t>
+  </si>
+  <si>
+    <t>Matching claim record displayed successfully</t>
+  </si>
+  <si>
+    <t>Relevant claim records displayed successfully</t>
+  </si>
+  <si>
+    <t>Claims matching selected status displayed successfully</t>
+  </si>
+  <si>
+    <t>Claims within selected date range displayed successfully</t>
+  </si>
+  <si>
+    <t>All search fields cleared successfully</t>
+  </si>
+  <si>
+    <t>Detailed claim information displayed successfully</t>
+  </si>
+  <si>
+    <t>Submitted claims and status vissible successfully</t>
+  </si>
+  <si>
+    <t>Macthing employee claim records displayed successfully</t>
+  </si>
+  <si>
+    <t>Employee claims filtered correctly</t>
+  </si>
+  <si>
+    <t>Current claim status displayed correctly</t>
+  </si>
+  <si>
+    <t>Status updated to submitted</t>
+  </si>
+  <si>
+    <t>Status displayed as Initiated successfully</t>
+  </si>
+  <si>
+    <t>Status of each employee claim visible successfully</t>
+  </si>
+  <si>
+    <t>Claim status, amount, currency, and event correct</t>
+  </si>
+  <si>
+    <t>Assigned claim status updated correctly</t>
   </si>
 </sst>
 </file>
@@ -11319,7 +11391,7 @@
         <v>912</v>
       </c>
       <c r="F237" s="3" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
       <c r="G237" s="3" t="s">
         <v>1475</v>
@@ -11365,7 +11437,7 @@
         <v>916</v>
       </c>
       <c r="F239" s="3" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="G239" s="3" t="s">
         <v>1475</v>
@@ -11388,7 +11460,7 @@
         <v>919</v>
       </c>
       <c r="F240" s="3" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
       <c r="G240" s="3" t="s">
         <v>1475</v>
@@ -11411,7 +11483,7 @@
         <v>931</v>
       </c>
       <c r="F241" s="3" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="G241" s="3" t="s">
         <v>1475</v>
@@ -11434,7 +11506,7 @@
         <v>934</v>
       </c>
       <c r="F242" s="3" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
       <c r="G242" s="3" t="s">
         <v>1475</v>
@@ -11457,7 +11529,7 @@
         <v>937</v>
       </c>
       <c r="F243" s="3" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="G243" s="3" t="s">
         <v>1475</v>
@@ -11480,7 +11552,7 @@
         <v>939</v>
       </c>
       <c r="F244" s="3" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
       <c r="G244" s="3" t="s">
         <v>1475</v>
@@ -11526,7 +11598,7 @@
         <v>941</v>
       </c>
       <c r="F246" s="3" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="G246" s="3" t="s">
         <v>1475</v>
@@ -11572,7 +11644,7 @@
         <v>945</v>
       </c>
       <c r="F248" s="3" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="G248" s="3" t="s">
         <v>1475</v>
@@ -11595,7 +11667,7 @@
         <v>957</v>
       </c>
       <c r="F249" s="3" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="G249" s="3" t="s">
         <v>1475</v>
@@ -11618,7 +11690,7 @@
         <v>960</v>
       </c>
       <c r="F250" s="3" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="G250" s="3" t="s">
         <v>1475</v>
@@ -11641,7 +11713,7 @@
         <v>962</v>
       </c>
       <c r="F251" s="3" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="G251" s="3" t="s">
         <v>1475</v>
@@ -11664,7 +11736,7 @@
         <v>964</v>
       </c>
       <c r="F252" s="3" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
       <c r="G252" s="3" t="s">
         <v>1475</v>
@@ -11687,7 +11759,7 @@
         <v>967</v>
       </c>
       <c r="F253" s="3" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="G253" s="3" t="s">
         <v>1475</v>
@@ -11733,7 +11805,7 @@
         <v>973</v>
       </c>
       <c r="F255" s="4" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
       <c r="G255" s="3" t="s">
         <v>1475</v>
@@ -11756,7 +11828,7 @@
         <v>976</v>
       </c>
       <c r="F256" s="4" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="G256" s="3" t="s">
         <v>1475</v>
@@ -11779,7 +11851,7 @@
         <v>979</v>
       </c>
       <c r="F257" s="3" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="G257" s="3" t="s">
         <v>1475</v>
@@ -11802,10 +11874,10 @@
         <v>991</v>
       </c>
       <c r="F258" s="3" t="s">
-        <v>12</v>
+        <v>1707</v>
       </c>
       <c r="G258" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="259" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11825,10 +11897,10 @@
         <v>172</v>
       </c>
       <c r="F259" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G259" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="260" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11848,10 +11920,10 @@
         <v>996</v>
       </c>
       <c r="F260" s="3" t="s">
-        <v>12</v>
+        <v>1708</v>
       </c>
       <c r="G260" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="261" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11871,10 +11943,10 @@
         <v>998</v>
       </c>
       <c r="F261" s="3" t="s">
-        <v>12</v>
+        <v>1709</v>
       </c>
       <c r="G261" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="262" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -11894,10 +11966,10 @@
         <v>1001</v>
       </c>
       <c r="F262" s="3" t="s">
-        <v>12</v>
+        <v>1710</v>
       </c>
       <c r="G262" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="263" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -11917,10 +11989,10 @@
         <v>1004</v>
       </c>
       <c r="F263" s="3" t="s">
-        <v>12</v>
+        <v>1711</v>
       </c>
       <c r="G263" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.35">
@@ -11940,10 +12012,10 @@
         <v>1008</v>
       </c>
       <c r="F264" s="3" t="s">
-        <v>12</v>
+        <v>1712</v>
       </c>
       <c r="G264" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.35">
@@ -11963,10 +12035,10 @@
         <v>1011</v>
       </c>
       <c r="F265" s="3" t="s">
-        <v>12</v>
+        <v>1713</v>
       </c>
       <c r="G265" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.35">
@@ -11986,10 +12058,10 @@
         <v>1022</v>
       </c>
       <c r="F266" s="3" t="s">
-        <v>12</v>
+        <v>1714</v>
       </c>
       <c r="G266" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="267" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12009,10 +12081,10 @@
         <v>1024</v>
       </c>
       <c r="F267" s="3" t="s">
-        <v>12</v>
+        <v>1715</v>
       </c>
       <c r="G267" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="268" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12032,10 +12104,10 @@
         <v>1027</v>
       </c>
       <c r="F268" s="3" t="s">
-        <v>12</v>
+        <v>1716</v>
       </c>
       <c r="G268" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="269" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12055,10 +12127,10 @@
         <v>1029</v>
       </c>
       <c r="F269" s="3" t="s">
-        <v>12</v>
+        <v>1717</v>
       </c>
       <c r="G269" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="270" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12078,10 +12150,10 @@
         <v>1031</v>
       </c>
       <c r="F270" s="3" t="s">
-        <v>12</v>
+        <v>1718</v>
       </c>
       <c r="G270" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="271" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12101,10 +12173,10 @@
         <v>1032</v>
       </c>
       <c r="F271" s="3" t="s">
-        <v>12</v>
+        <v>1719</v>
       </c>
       <c r="G271" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.35">
@@ -12124,10 +12196,10 @@
         <v>1035</v>
       </c>
       <c r="F272" s="3" t="s">
-        <v>12</v>
+        <v>1720</v>
       </c>
       <c r="G272" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.35">
@@ -12147,10 +12219,10 @@
         <v>1038</v>
       </c>
       <c r="F273" s="3" t="s">
-        <v>12</v>
+        <v>1721</v>
       </c>
       <c r="G273" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="274" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -12170,10 +12242,10 @@
         <v>1040</v>
       </c>
       <c r="F274" s="3" t="s">
-        <v>12</v>
+        <v>1722</v>
       </c>
       <c r="G274" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="275" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12193,10 +12265,10 @@
         <v>1043</v>
       </c>
       <c r="F275" s="3" t="s">
-        <v>12</v>
+        <v>1723</v>
       </c>
       <c r="G275" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="276" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12216,10 +12288,10 @@
         <v>1057</v>
       </c>
       <c r="F276" s="3" t="s">
-        <v>12</v>
+        <v>1724</v>
       </c>
       <c r="G276" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.35">
@@ -12239,10 +12311,10 @@
         <v>1060</v>
       </c>
       <c r="F277" s="3" t="s">
-        <v>12</v>
+        <v>1725</v>
       </c>
       <c r="G277" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.35">
@@ -12262,10 +12334,10 @@
         <v>1063</v>
       </c>
       <c r="F278" s="3" t="s">
-        <v>12</v>
+        <v>1726</v>
       </c>
       <c r="G278" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.35">
@@ -12285,10 +12357,10 @@
         <v>1065</v>
       </c>
       <c r="F279" s="3" t="s">
-        <v>12</v>
+        <v>1727</v>
       </c>
       <c r="G279" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="280" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12308,10 +12380,10 @@
         <v>1029</v>
       </c>
       <c r="F280" s="3" t="s">
-        <v>12</v>
+        <v>1717</v>
       </c>
       <c r="G280" s="3" t="s">
-        <v>36</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="281" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12331,10 +12403,10 @@
         <v>1070</v>
       </c>
       <c r="F281" s="3" t="s">
-        <v>12</v>
+        <v>1728</v>
       </c>
       <c r="G281" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="282" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12354,10 +12426,10 @@
         <v>1072</v>
       </c>
       <c r="F282" s="3" t="s">
-        <v>12</v>
+        <v>1729</v>
       </c>
       <c r="G282" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC282 to TC308 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1756">
   <si>
     <t>TC ID</t>
   </si>
@@ -5590,6 +5590,88 @@
   </si>
   <si>
     <t>Assigned claim status updated correctly</t>
+  </si>
+  <si>
+    <t>Claim information and status remain consistent across modules
+successfully</t>
+  </si>
+  <si>
+    <t>Status changes reflected accurately througout workflow
+successfully</t>
+  </si>
+  <si>
+    <t>Post created successfully and appeared in the newsfeed 
+successfully</t>
+  </si>
+  <si>
+    <t>Post with image published successfully</t>
+  </si>
+  <si>
+    <t>Post with video published successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validation message did't displayed </t>
+  </si>
+  <si>
+    <t>Newly created post appeared at the top of the newsfeed
+successfully</t>
+  </si>
+  <si>
+    <t>Correct date and time displayed with the post successfully</t>
+  </si>
+  <si>
+    <t>Post shared successfully</t>
+  </si>
+  <si>
+    <t>Post visible to authorized users successfully</t>
+  </si>
+  <si>
+    <t>Like count increase by one successfully</t>
+  </si>
+  <si>
+    <t>Like removed and count updated successfully</t>
+  </si>
+  <si>
+    <t>Comment added successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment count increase accordingly </t>
+  </si>
+  <si>
+    <t>Share count increase correctly</t>
+  </si>
+  <si>
+    <t>Total likes count upadted correctly</t>
+  </si>
+  <si>
+    <t>Like, Comment, and Share icon displayed successfully</t>
+  </si>
+  <si>
+    <t>Changes remain saved and visible successfully</t>
+  </si>
+  <si>
+    <t>Latest posts displayed in descending successfully</t>
+  </si>
+  <si>
+    <t>Post sorted by highest likes successfully</t>
+  </si>
+  <si>
+    <t>Posts sorted by highest comments successfully</t>
+  </si>
+  <si>
+    <t>Posts load successfully in the newsfeed</t>
+  </si>
+  <si>
+    <t>Username, profile image, and timestamp displayed successfully</t>
+  </si>
+  <si>
+    <t>Content displayed correctly without formatting issues</t>
+  </si>
+  <si>
+    <t>Latest feed data load correctly</t>
+  </si>
+  <si>
+    <t>Available management options displayed successfully</t>
   </si>
 </sst>
 </file>
@@ -12432,7 +12514,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="283" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>1087</v>
       </c>
@@ -12448,11 +12530,11 @@
       <c r="E283" s="2" t="s">
         <v>1076</v>
       </c>
-      <c r="F283" s="3" t="s">
-        <v>12</v>
+      <c r="F283" s="4" t="s">
+        <v>1730</v>
       </c>
       <c r="G283" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="284" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12471,11 +12553,11 @@
       <c r="E284" s="2" t="s">
         <v>1078</v>
       </c>
-      <c r="F284" s="3" t="s">
-        <v>12</v>
+      <c r="F284" s="4" t="s">
+        <v>1731</v>
       </c>
       <c r="G284" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="285" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -12494,11 +12576,11 @@
       <c r="E285" s="2" t="s">
         <v>1091</v>
       </c>
-      <c r="F285" s="3" t="s">
-        <v>12</v>
+      <c r="F285" s="4" t="s">
+        <v>1732</v>
       </c>
       <c r="G285" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="286" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -12518,10 +12600,10 @@
         <v>1094</v>
       </c>
       <c r="F286" s="3" t="s">
-        <v>12</v>
+        <v>1733</v>
       </c>
       <c r="G286" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="287" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -12541,10 +12623,10 @@
         <v>1097</v>
       </c>
       <c r="F287" s="3" t="s">
-        <v>12</v>
+        <v>1734</v>
       </c>
       <c r="G287" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="288" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12564,10 +12646,10 @@
         <v>172</v>
       </c>
       <c r="F288" s="3" t="s">
-        <v>12</v>
+        <v>1735</v>
       </c>
       <c r="G288" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="289" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12586,11 +12668,11 @@
       <c r="E289" s="2" t="s">
         <v>1103</v>
       </c>
-      <c r="F289" s="3" t="s">
-        <v>12</v>
+      <c r="F289" s="4" t="s">
+        <v>1736</v>
       </c>
       <c r="G289" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="290" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12610,10 +12692,10 @@
         <v>1106</v>
       </c>
       <c r="F290" s="3" t="s">
-        <v>12</v>
+        <v>1737</v>
       </c>
       <c r="G290" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="291" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12633,10 +12715,10 @@
         <v>1108</v>
       </c>
       <c r="F291" s="3" t="s">
-        <v>12</v>
+        <v>1738</v>
       </c>
       <c r="G291" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="292" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12656,10 +12738,10 @@
         <v>1111</v>
       </c>
       <c r="F292" s="3" t="s">
-        <v>12</v>
+        <v>1739</v>
       </c>
       <c r="G292" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="293" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12679,10 +12761,10 @@
         <v>1122</v>
       </c>
       <c r="F293" s="3" t="s">
-        <v>12</v>
+        <v>1740</v>
       </c>
       <c r="G293" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="294" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12702,10 +12784,10 @@
         <v>1125</v>
       </c>
       <c r="F294" s="3" t="s">
-        <v>12</v>
+        <v>1741</v>
       </c>
       <c r="G294" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="295" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -12725,10 +12807,10 @@
         <v>1128</v>
       </c>
       <c r="F295" s="3" t="s">
-        <v>12</v>
+        <v>1742</v>
       </c>
       <c r="G295" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.35">
@@ -12748,10 +12830,10 @@
         <v>1132</v>
       </c>
       <c r="F296" s="3" t="s">
-        <v>12</v>
+        <v>1743</v>
       </c>
       <c r="G296" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.35">
@@ -12771,10 +12853,10 @@
         <v>1108</v>
       </c>
       <c r="F297" s="3" t="s">
-        <v>12</v>
+        <v>1738</v>
       </c>
       <c r="G297" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.35">
@@ -12794,10 +12876,10 @@
         <v>1136</v>
       </c>
       <c r="F298" s="3" t="s">
-        <v>12</v>
+        <v>1744</v>
       </c>
       <c r="G298" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.35">
@@ -12817,10 +12899,10 @@
         <v>1139</v>
       </c>
       <c r="F299" s="3" t="s">
-        <v>12</v>
+        <v>1745</v>
       </c>
       <c r="G299" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.35">
@@ -12840,10 +12922,10 @@
         <v>1142</v>
       </c>
       <c r="F300" s="3" t="s">
-        <v>12</v>
+        <v>1746</v>
       </c>
       <c r="G300" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="301" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12863,10 +12945,10 @@
         <v>1144</v>
       </c>
       <c r="F301" s="3" t="s">
-        <v>12</v>
+        <v>1747</v>
       </c>
       <c r="G301" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.35">
@@ -12886,10 +12968,10 @@
         <v>1157</v>
       </c>
       <c r="F302" s="3" t="s">
-        <v>12</v>
+        <v>1748</v>
       </c>
       <c r="G302" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.35">
@@ -12909,10 +12991,10 @@
         <v>1160</v>
       </c>
       <c r="F303" s="3" t="s">
-        <v>12</v>
+        <v>1749</v>
       </c>
       <c r="G303" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.35">
@@ -12932,10 +13014,10 @@
         <v>1163</v>
       </c>
       <c r="F304" s="3" t="s">
-        <v>12</v>
+        <v>1750</v>
       </c>
       <c r="G304" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.35">
@@ -12955,10 +13037,10 @@
         <v>1166</v>
       </c>
       <c r="F305" s="3" t="s">
-        <v>12</v>
+        <v>1751</v>
       </c>
       <c r="G305" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="306" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -12978,10 +13060,10 @@
         <v>1168</v>
       </c>
       <c r="F306" s="3" t="s">
-        <v>12</v>
+        <v>1752</v>
       </c>
       <c r="G306" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="307" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13001,10 +13083,10 @@
         <v>1171</v>
       </c>
       <c r="F307" s="3" t="s">
-        <v>12</v>
+        <v>1753</v>
       </c>
       <c r="G307" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.35">
@@ -13024,10 +13106,10 @@
         <v>1174</v>
       </c>
       <c r="F308" s="3" t="s">
-        <v>12</v>
+        <v>1754</v>
       </c>
       <c r="G308" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.35">
@@ -13047,10 +13129,10 @@
         <v>1177</v>
       </c>
       <c r="F309" s="3" t="s">
-        <v>12</v>
+        <v>1755</v>
       </c>
       <c r="G309" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="310" spans="1:7" ht="29" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
TC309 to TC331 Test Done
</commit_message>
<xml_diff>
--- a/Test Cases/TestCases.xlsx
+++ b/Test Cases/TestCases.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2681" uniqueCount="1777">
   <si>
     <t>TC ID</t>
   </si>
@@ -5672,6 +5672,71 @@
   </si>
   <si>
     <t>Available management options displayed successfully</t>
+  </si>
+  <si>
+    <t>Upcoming anniversaries section displayed employee destails
+correctly</t>
+  </si>
+  <si>
+    <t>Corresponding posts load correctly without errors</t>
+  </si>
+  <si>
+    <t>User authenticated successfully</t>
+  </si>
+  <si>
+    <t>Login fail with an error message successfully</t>
+  </si>
+  <si>
+    <t>Authentication denied successfully</t>
+  </si>
+  <si>
+    <t>Password characters masked successfully</t>
+  </si>
+  <si>
+    <t>Every time "invalid credentials" message shows</t>
+  </si>
+  <si>
+    <t>User session end successfully</t>
+  </si>
+  <si>
+    <t>Retured to dashboard after logout</t>
+  </si>
+  <si>
+    <t>Access granted successfully</t>
+  </si>
+  <si>
+    <t>Access denied successfully</t>
+  </si>
+  <si>
+    <t>Only authorized menus displayed successfully</t>
+  </si>
+  <si>
+    <t>Unauthorized actions restricted successfully</t>
+  </si>
+  <si>
+    <t>Action completed successfully</t>
+  </si>
+  <si>
+    <t>User only access permitted modules successfully</t>
+  </si>
+  <si>
+    <t>New user session created successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session expire automatically </t>
+  </si>
+  <si>
+    <t>User redirected to login page successfully</t>
+  </si>
+  <si>
+    <t>Protected pages accessible After Logout</t>
+  </si>
+  <si>
+    <t>Session management worked accroding to system policy 
+successfully</t>
+  </si>
+  <si>
+    <t>Session remain active successfully</t>
   </si>
 </sst>
 </file>
@@ -13151,11 +13216,11 @@
       <c r="E310" s="2" t="s">
         <v>1179</v>
       </c>
-      <c r="F310" s="3" t="s">
-        <v>12</v>
+      <c r="F310" s="4" t="s">
+        <v>1756</v>
       </c>
       <c r="G310" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="311" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13175,10 +13240,10 @@
         <v>1182</v>
       </c>
       <c r="F311" s="3" t="s">
-        <v>12</v>
+        <v>1757</v>
       </c>
       <c r="G311" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="312" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13198,10 +13263,10 @@
         <v>1195</v>
       </c>
       <c r="F312" s="3" t="s">
-        <v>12</v>
+        <v>1758</v>
       </c>
       <c r="G312" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="313" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13221,10 +13286,10 @@
         <v>1198</v>
       </c>
       <c r="F313" s="3" t="s">
-        <v>12</v>
+        <v>1759</v>
       </c>
       <c r="G313" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="314" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13244,10 +13309,10 @@
         <v>1201</v>
       </c>
       <c r="F314" s="3" t="s">
-        <v>12</v>
+        <v>1760</v>
       </c>
       <c r="G314" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="315" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13267,10 +13332,10 @@
         <v>172</v>
       </c>
       <c r="F315" s="3" t="s">
-        <v>12</v>
+        <v>1510</v>
       </c>
       <c r="G315" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.35">
@@ -13290,10 +13355,10 @@
         <v>1207</v>
       </c>
       <c r="F316" s="3" t="s">
-        <v>12</v>
+        <v>1761</v>
       </c>
       <c r="G316" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="317" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13313,10 +13378,10 @@
         <v>1210</v>
       </c>
       <c r="F317" s="3" t="s">
-        <v>12</v>
+        <v>1762</v>
       </c>
       <c r="G317" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="318" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13336,10 +13401,10 @@
         <v>1212</v>
       </c>
       <c r="F318" s="3" t="s">
-        <v>12</v>
+        <v>1763</v>
       </c>
       <c r="G318" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="319" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13359,10 +13424,10 @@
         <v>1215</v>
       </c>
       <c r="F319" s="3" t="s">
-        <v>12</v>
+        <v>1764</v>
       </c>
       <c r="G319" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="320" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13382,10 +13447,10 @@
         <v>1226</v>
       </c>
       <c r="F320" s="3" t="s">
-        <v>12</v>
+        <v>1765</v>
       </c>
       <c r="G320" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="321" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13405,10 +13470,10 @@
         <v>499</v>
       </c>
       <c r="F321" s="3" t="s">
-        <v>12</v>
+        <v>1766</v>
       </c>
       <c r="G321" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="322" spans="1:7" x14ac:dyDescent="0.35">
@@ -13428,10 +13493,10 @@
         <v>1232</v>
       </c>
       <c r="F322" s="3" t="s">
-        <v>12</v>
+        <v>1767</v>
       </c>
       <c r="G322" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="323" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13451,10 +13516,10 @@
         <v>499</v>
       </c>
       <c r="F323" s="3" t="s">
-        <v>12</v>
+        <v>1766</v>
       </c>
       <c r="G323" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="324" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13474,10 +13539,10 @@
         <v>1236</v>
       </c>
       <c r="F324" s="3" t="s">
-        <v>12</v>
+        <v>1768</v>
       </c>
       <c r="G324" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="325" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13497,10 +13562,10 @@
         <v>1239</v>
       </c>
       <c r="F325" s="3" t="s">
-        <v>12</v>
+        <v>1769</v>
       </c>
       <c r="G325" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.35">
@@ -13520,10 +13585,10 @@
         <v>1243</v>
       </c>
       <c r="F326" s="3" t="s">
-        <v>12</v>
+        <v>1770</v>
       </c>
       <c r="G326" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.35">
@@ -13543,10 +13608,10 @@
         <v>1253</v>
       </c>
       <c r="F327" s="3" t="s">
-        <v>12</v>
+        <v>1771</v>
       </c>
       <c r="G327" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="328" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
@@ -13566,10 +13631,10 @@
         <v>1255</v>
       </c>
       <c r="F328" s="3" t="s">
-        <v>12</v>
+        <v>1772</v>
       </c>
       <c r="G328" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="329" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13589,10 +13654,10 @@
         <v>1215</v>
       </c>
       <c r="F329" s="3" t="s">
-        <v>12</v>
+        <v>1773</v>
       </c>
       <c r="G329" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="330" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13612,10 +13677,10 @@
         <v>1260</v>
       </c>
       <c r="F330" s="3" t="s">
-        <v>12</v>
+        <v>1774</v>
       </c>
       <c r="G330" s="3" t="s">
-        <v>36</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="331" spans="1:7" ht="29" x14ac:dyDescent="0.35">
@@ -13634,11 +13699,11 @@
       <c r="E331" s="2" t="s">
         <v>1264</v>
       </c>
-      <c r="F331" s="3" t="s">
-        <v>12</v>
+      <c r="F331" s="4" t="s">
+        <v>1775</v>
       </c>
       <c r="G331" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="332" spans="1:7" x14ac:dyDescent="0.35">
@@ -13658,10 +13723,10 @@
         <v>1267</v>
       </c>
       <c r="F332" s="3" t="s">
-        <v>12</v>
+        <v>1776</v>
       </c>
       <c r="G332" s="3" t="s">
-        <v>36</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="333" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>